<commit_message>
feat(queue): lock video_1..video_30 and start Shorts cleanly from video_31.mp4
</commit_message>
<xml_diff>
--- a/bilgidozu_yukleme_tablosu.xlsx
+++ b/bilgidozu_yukleme_tablosu.xlsx
@@ -49,7 +49,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -80,6 +80,12 @@
         <bgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EAD3"/>
+        <bgColor rgb="00D9EAD3"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border/>
@@ -92,7 +98,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -140,6 +146,12 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -591,50 +603,50 @@
       <c r="AC1" s="2" t="n"/>
     </row>
     <row r="2" ht="112.5" customHeight="1" s="13">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" s="17" t="inlineStr">
         <is>
           <t>YAYINLANDI</t>
         </is>
       </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="B2" s="18" t="inlineStr">
         <is>
           <t>video_1.mp4</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="C2" s="18" t="inlineStr">
         <is>
           <t>Venüs'te Bir Gün Bir Yıldan Daha Uzun! 🪐 #bilgidozu #shorts</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
+      <c r="D2" s="18" t="inlineStr">
         <is>
           <t>Kendi doğum gününüzün bir tam günden daha kısa sürdüğünü hayal edebiliyor musunuz? Venüs kendi ekseninde 243 Dünya gününde dönerken, Güneş etrafındaki bir yılını sadece 225 günde tamamlar. Yani Venüs'te bir gün, bir yıldan daha uzundur!
 Daha fazla bilgi dozu için takip etmeyi unutma!</t>
         </is>
       </c>
-      <c r="E2" s="4" t="inlineStr">
+      <c r="E2" s="18" t="inlineStr">
         <is>
           <t>#bilgidozu #shorts #uzay #bilim</t>
         </is>
       </c>
-      <c r="F2" s="4" t="inlineStr">
+      <c r="F2" s="18" t="inlineStr">
         <is>
           <t>bilgidozu, uzay, venüs, ilginçbilgiler, bilim, astronomi, shorts</t>
         </is>
       </c>
-      <c r="G2" s="4" t="inlineStr">
+      <c r="G2" s="18" t="inlineStr">
         <is>
           <t>Venüs'te bir gün bir yıldan uzun sürse, orada yaşayan birine 'günaydın' demek kaç yıl sürerdi? 😄🌙 Cevabını yaz! 👇</t>
         </is>
       </c>
-      <c r="H2" s="4" t="inlineStr">
+      <c r="H2" s="18" t="inlineStr">
         <is>
           <t>Uzay ve Astronomi</t>
         </is>
       </c>
-      <c r="I2" s="4" t="inlineStr">
-        <is>
-          <t>NASA — Venus: https://science.nasa.gov/venus/</t>
+      <c r="I2" s="18" t="inlineStr">
+        <is>
+          <t>YÜKLENDİ / ATLANDI (31'den Başlatma Kilidi)</t>
         </is>
       </c>
       <c r="J2" s="5" t="n"/>
@@ -659,50 +671,50 @@
       <c r="AC2" s="6" t="n"/>
     </row>
     <row r="3" ht="112.5" customHeight="1" s="13">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="17" t="inlineStr">
         <is>
           <t>YAYINLANDI</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" s="18" t="inlineStr">
         <is>
           <t>video_2.mp4</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="18" t="inlineStr">
         <is>
           <t>Bir Kargaya Asla Yanlış Yapmayın: Yüzünüzü Asla Unutmazlar! 🦅 #bilgidozu #shorts</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" s="18" t="inlineStr">
         <is>
           <t>Washington Üniversitesi'nin yaptığı ünlü araştırmada kargalar kendilerini yakalayan maskeli araştırmacıları tam 5 yıl boyunca unutmadı, hatta bu tehlikeli yüzü yeni nesillere ve tüm sürüye öğretti!
 Daha fazla bilgi dozu için takip etmeyi unutma!</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="E3" s="18" t="inlineStr">
         <is>
           <t>#bilgidozu #shorts #doğa #bilim</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="F3" s="18" t="inlineStr">
         <is>
           <t>bilgidozu, karga, hayvanlaralemi, zeka, deney, ilginçbilgiler, shorts</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="G3" s="18" t="inlineStr">
         <is>
           <t>Sence kargalar gerçekten 5 yıl boyunca yüzleri hatırlıyor mu? 🦅 İnananlar '1', şüphelenenler '2' yazsın! 👇</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="H3" s="18" t="inlineStr">
         <is>
           <t>Doğa ve Hayvanlar</t>
         </is>
       </c>
-      <c r="I3" s="4" t="inlineStr">
-        <is>
-          <t>The Conversation (UW 5 yıllık maske deneyi): https://theconversation.com/never-cross-a-crow-it-will-remember-your-face-2121</t>
+      <c r="I3" s="18" t="inlineStr">
+        <is>
+          <t>YÜKLENDİ / ATLANDI (31'den Başlatma Kilidi)</t>
         </is>
       </c>
       <c r="J3" s="5" t="n"/>
@@ -727,50 +739,50 @@
       <c r="AC3" s="6" t="n"/>
     </row>
     <row r="4" ht="112.5" customHeight="1" s="13">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="17" t="inlineStr">
         <is>
           <t>YAYINLANDI</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="18" t="inlineStr">
         <is>
           <t>video_3.mp4</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="18" t="inlineStr">
         <is>
           <t>Her Gün Yediğiniz Bu Meyve Aslında Radyoaktif! 🍌⚡ #bilgidozu #shorts</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D4" s="18" t="inlineStr">
         <is>
           <t>Muzlar doğal olarak radyoaktif Potasyum-40 izotopu içerir ve saniyede yaklaşık 15 pozitron (antimadde parçacığı) yayar. Nükleer fizikte buna 'Muz Eşdeğer Dozu' denir!
 Daha fazla bilgi dozu için takip etmeyi unutma!</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="E4" s="18" t="inlineStr">
         <is>
           <t>#bilgidozu #shorts #fizik #bilim</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="F4" s="18" t="inlineStr">
         <is>
           <t>bilgidozu, fizik, radyasyon, antimadde, ilginçbilgiler, bilim, shorts</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="G4" s="18" t="inlineStr">
         <is>
           <t>Bugün kaç muz yedin? 🍌😄 Hadi itiraf et, yorumlara yaz! 👇</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="H4" s="18" t="inlineStr">
         <is>
           <t>Fizik ve Bilim</t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr">
-        <is>
-          <t>Banana Equivalent Dose: https://en.wikipedia.org/wiki/Banana_equivalent_dose</t>
+      <c r="I4" s="18" t="inlineStr">
+        <is>
+          <t>YÜKLENDİ / ATLANDI (31'den Başlatma Kilidi)</t>
         </is>
       </c>
       <c r="J4" s="5" t="n"/>
@@ -795,50 +807,50 @@
       <c r="AC4" s="6" t="n"/>
     </row>
     <row r="5" ht="112.5" customHeight="1" s="13">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>YAYINLANDI</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="18" t="inlineStr">
         <is>
           <t>video_4.mp4</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="18" t="inlineStr">
         <is>
           <t>Ormanın Altındaki Gizli İnternet: Ağaçlar Birbiriyle Konuşuyor! 🌲🍄 #bilgidozu #shorts</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D5" s="18" t="inlineStr">
         <is>
           <t>Ağaçlar köklerindeki mikorizal mantar ağlarını (Wood Wide Web) kullanarak birbirleriyle haberleşir, tehlike anında kimyasal sinyaller gönderip komşu fideleri besler!
 Daha fazla bilgi dozu için takip etmeyi unutma!</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="E5" s="18" t="inlineStr">
         <is>
           <t>#bilgidozu #shorts #doğa #bilim</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="F5" s="18" t="inlineStr">
         <is>
           <t>bilgidozu, doğa, biyoloji, ağaçlar, orman, woodwideweb, shorts</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="G5" s="18" t="inlineStr">
         <is>
           <t>Ormanın altındaki gizli internete şaşırdın mı? 🌲🍄 Sence ağaçlar birbirine daha neler anlatıyor olabilir? 👇</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="H5" s="18" t="inlineStr">
         <is>
           <t>Doğa ve Biyoloji</t>
         </is>
       </c>
-      <c r="I5" s="4" t="inlineStr">
-        <is>
-          <t>Mikorizal ağ (Wood Wide Web): https://en.wikipedia.org/wiki/Mycorrhizal_network</t>
+      <c r="I5" s="18" t="inlineStr">
+        <is>
+          <t>YÜKLENDİ / ATLANDI (31'den Başlatma Kilidi)</t>
         </is>
       </c>
       <c r="J5" s="5" t="n"/>
@@ -863,50 +875,50 @@
       <c r="AC5" s="6" t="n"/>
     </row>
     <row r="6" ht="112.5" customHeight="1" s="13">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="17" t="inlineStr">
         <is>
           <t>YÜKLENDİ</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="18" t="inlineStr">
         <is>
           <t>video_5.mp4</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" s="18" t="inlineStr">
         <is>
           <t>Aynaya Baktığında Bir İnsan Değil, Bir Süpernova Görüyorsun! ✨ #bilgidozu #shorts</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="D6" s="18" t="inlineStr">
         <is>
           <t>Kanınızdaki demir, kemiklerinizdeki kalsiyum ve soluduğunuz oksijen patlayan dev süpernova yıldızlarının çekirdeklerinde üretildi. Sen tam anlamıyla canlı bir yıldız tozusun!
 Daha fazla bilgi dozu için takip etmeyi unutma!</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="E6" s="18" t="inlineStr">
         <is>
           <t>#bilgidozu #shorts #uzay #bilim</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="F6" s="18" t="inlineStr">
         <is>
           <t>bilgidozu, kozmoloji, yıldıztozu, süpernova, evren, bilim, shorts</t>
         </is>
       </c>
-      <c r="G6" s="4" t="inlineStr">
+      <c r="G6" s="18" t="inlineStr">
         <is>
           <t>Şu an vücudunda yıldız parçaları taşıdığını biliyor muydun? ✨ Bu bilgiye '🤯' yazan herkes aslında bir süpernova! 👇</t>
         </is>
       </c>
-      <c r="H6" s="4" t="inlineStr">
+      <c r="H6" s="18" t="inlineStr">
         <is>
           <t>Uzay ve Astronomi</t>
         </is>
       </c>
-      <c r="I6" s="4" t="inlineStr">
-        <is>
-          <t>NASA — Stars: https://science.nasa.gov/universe/stars/</t>
+      <c r="I6" s="18" t="inlineStr">
+        <is>
+          <t>YÜKLENDİ / ATLANDI (31'den Başlatma Kilidi)</t>
         </is>
       </c>
       <c r="J6" s="5" t="n"/>
@@ -931,50 +943,50 @@
       <c r="AC6" s="6" t="n"/>
     </row>
     <row r="7" ht="112.5" customHeight="1" s="13">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="17" t="inlineStr">
         <is>
           <t>YÜKLENDİ</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="18" t="inlineStr">
         <is>
           <t>video_6.mp4</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="18" t="inlineStr">
         <is>
           <t>Su Aslında Şeffaf Değil, Doğal Olarak Mavidir! 💧 #bilgidozu #shorts</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D7" s="18" t="inlineStr">
         <is>
           <t>Denizlerin gökyüzünü yansıttığı için mavi olduğu bilgisi bir efsanedir! Hidrojen ve oksijen kimyasal bağları kırmızı dalga boyunu soğurur ve saf su doğası gereği açık mavidir!
 Daha fazla bilgi dozu için takip etmeyi unutma!</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="E7" s="18" t="inlineStr">
         <is>
           <t>#bilgidozu #shorts #fizik #bilim</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="F7" s="18" t="inlineStr">
         <is>
           <t>bilgidozu, bilim, fizik, denizler, su, kimya, shorts</t>
         </is>
       </c>
-      <c r="G7" s="4" t="inlineStr">
+      <c r="G7" s="18" t="inlineStr">
         <is>
           <t>Mavinin suyun GERÇEK rengi olduğunu biliyor muydun? 💙 Şaşıranlar '1' desin! 👇</t>
         </is>
       </c>
-      <c r="H7" s="4" t="inlineStr">
+      <c r="H7" s="18" t="inlineStr">
         <is>
           <t>Fizik ve Kimya</t>
         </is>
       </c>
-      <c r="I7" s="4" t="inlineStr">
-        <is>
-          <t>NOAA — Why is the ocean blue: https://oceanservice.noaa.gov/facts/oceanblue.html</t>
+      <c r="I7" s="18" t="inlineStr">
+        <is>
+          <t>YÜKLENDİ / ATLANDI (31'den Başlatma Kilidi)</t>
         </is>
       </c>
       <c r="J7" s="5" t="n"/>
@@ -999,51 +1011,50 @@
       <c r="AC7" s="6" t="n"/>
     </row>
     <row r="8" ht="112.5" customHeight="1" s="13">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" s="17" t="inlineStr">
         <is>
           <t>YÜKLENDİ</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="18" t="inlineStr">
         <is>
           <t>video_7.mp4</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" s="18" t="inlineStr">
         <is>
           <t>Bal Arıları Sıfır Kavramını ve Matematiği Anlayabiliyor! 🐝🔢 #bilgidozu #shorts</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D8" s="18" t="inlineStr">
         <is>
           <t>Susam tanesi büyüklüğündeki minik beyinleriyle bal arıları, 'sıfır' soyut kavramını ve basit toplama-çıkarma işlemlerini kavrayabilen dünyadaki nadir canlılardandır!
 Daha fazla bilgi dozu için takip etmeyi unutma!</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="E8" s="18" t="inlineStr">
         <is>
           <t>#bilgidozu #shorts #doğa #bilim</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="F8" s="18" t="inlineStr">
         <is>
           <t>bilgidozu, arılar, hayvanlaralemi, matematik, zeka, biyoloji, shorts</t>
         </is>
       </c>
-      <c r="G8" s="4" t="inlineStr">
+      <c r="G8" s="18" t="inlineStr">
         <is>
           <t>Sıfır kavramını sen kaç yaşında öğrenmiştin? 🐝 Bu arılar seni geçti mi? 😄 Yaz bakalım! 👇</t>
         </is>
       </c>
-      <c r="H8" s="4" t="inlineStr">
+      <c r="H8" s="18" t="inlineStr">
         <is>
           <t>Doğa ve Hayvanlar</t>
         </is>
       </c>
-      <c r="I8" s="4" t="inlineStr">
-        <is>
-          <t>The Conversation (RMIT araştırmacıları): https://theconversation.com/bees-join-an-elite-group-of-species-that-understands-the-concept-of-zero-as-a-number-97316
-RMIT: https://www.rmit.edu.au/news/all-news/2018/jun/honeybees-zero-in-on-nothing</t>
+      <c r="I8" s="18" t="inlineStr">
+        <is>
+          <t>YÜKLENDİ / ATLANDI (31'den Başlatma Kilidi)</t>
         </is>
       </c>
       <c r="J8" s="5" t="n"/>
@@ -1068,51 +1079,50 @@
       <c r="AC8" s="6" t="n"/>
     </row>
     <row r="9" ht="112.5" customHeight="1" s="13">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" s="17" t="inlineStr">
         <is>
           <t>YÜKLENDİ</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" s="18" t="inlineStr">
         <is>
           <t>video_8.mp4</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C9" s="18" t="inlineStr">
         <is>
           <t>Dünyadaki Tüm Karıncalar İnsanlardan Daha Ağır Çekiyor! 🐜⚖️ #bilgidozu #shorts</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="D9" s="18" t="inlineStr">
         <is>
           <t>Dünya üzerindeki 20 katrilyon karıncanın toplam kuru biyokütle ağırlığı, gezegendeki tüm insanların ve yabani memelilerin toplam ağırlığından daha fazladır!
 Daha fazla bilgi dozu için takip etmeyi unutma!</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="E9" s="18" t="inlineStr">
         <is>
           <t>#bilgidozu #shorts #doğa #bilim</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="F9" s="18" t="inlineStr">
         <is>
           <t>bilgidozu, karınca, doğa, biyoloji, ekoloji, ilginçbilgiler, shorts</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr">
+      <c r="G9" s="18" t="inlineStr">
         <is>
           <t>Karıncalar mı insanlardan güçlü mü? 🐜⚖️ Sence tüm karıncalar mı yoksa tüm insanlar mı daha ağır? Cevabını yaz! 👇</t>
         </is>
       </c>
-      <c r="H9" s="4" t="inlineStr">
+      <c r="H9" s="18" t="inlineStr">
         <is>
           <t>Doğa ve Biyoloji</t>
         </is>
       </c>
-      <c r="I9" s="3" t="inlineStr">
-        <is>
-          <t>phys.org (PNAS 2022): https://phys.org/news/2022-09-earth-harbours-ants-wild-birds.html
-⚠ DÜZELTME ÖNERİSİ: PNAS 2022'ye göre karıncalar (12 Mt C) insanlardan DEĞİL (insanların ~%20'si), tüm YABANİ KUŞ+MEMELİLERİN toplamından daha ağır. Açıklamayı/başlığı düzeltirsen kaynakla tam uyumlu olur: 'Dünyadaki karıncalar tüm yabani kuş ve memelilerden daha ağır!'</t>
+      <c r="I9" s="17" t="inlineStr">
+        <is>
+          <t>YÜKLENDİ / ATLANDI (31'den Başlatma Kilidi)</t>
         </is>
       </c>
       <c r="J9" s="5" t="n"/>
@@ -1137,50 +1147,50 @@
       <c r="AC9" s="6" t="n"/>
     </row>
     <row r="10" ht="112.5" customHeight="1" s="13">
-      <c r="A10" s="3" t="inlineStr">
+      <c r="A10" s="17" t="inlineStr">
         <is>
           <t>YÜKLENDİ</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B10" s="18" t="inlineStr">
         <is>
           <t>video_9.mp4</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C10" s="18" t="inlineStr">
         <is>
           <t>Jüpiter'in Bu Uydusunda Dünya'dan 2 Kat Fazla Su Var! 🪐🌊 #bilgidozu #shorts</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="D10" s="18" t="inlineStr">
         <is>
           <t>Ay'dan bile küçük olan Jüpiter uydusu Europa'nın buz kabuğunun altındaki dev tuzlu okyanusta, Dünya'daki bütün okyanusların toplamının tam 2 katı su vardır!
 Daha fazla bilgi dozu için takip etmeyi unutma!</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="E10" s="18" t="inlineStr">
         <is>
           <t>#bilgidozu #shorts #uzay #bilim</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr">
+      <c r="F10" s="18" t="inlineStr">
         <is>
           <t>bilgidozu, uzay, europa, jüpiter, astronomi, nasa, shorts</t>
         </is>
       </c>
-      <c r="G10" s="4" t="inlineStr">
+      <c r="G10" s="18" t="inlineStr">
         <is>
           <t>Europa'nın buzunun altında yaşam olsa nasıl olurdu? 🌊🦑 En çılgın tahminini yaz! 👇</t>
         </is>
       </c>
-      <c r="H10" s="4" t="inlineStr">
+      <c r="H10" s="18" t="inlineStr">
         <is>
           <t>Uzay ve Astronomi</t>
         </is>
       </c>
-      <c r="I10" s="4" t="inlineStr">
-        <is>
-          <t>NASA — Europa: https://science.nasa.gov/jupiter/moons/europa/</t>
+      <c r="I10" s="18" t="inlineStr">
+        <is>
+          <t>YÜKLENDİ / ATLANDI (31'den Başlatma Kilidi)</t>
         </is>
       </c>
       <c r="J10" s="5" t="n"/>
@@ -1205,50 +1215,50 @@
       <c r="AC10" s="6" t="n"/>
     </row>
     <row r="11" ht="112.5" customHeight="1" s="13">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="A11" s="17" t="inlineStr">
         <is>
           <t>YÜKLENDİ</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B11" s="18" t="inlineStr">
         <is>
           <t>video_10.mp4</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C11" s="18" t="inlineStr">
         <is>
           <t>2000 Yıllık Roma Binaları Neden Yıkılmıyor? Beton Kendi Kendini Onarıyor! 🏛️⚡ #bilgidozu #shorts</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D11" s="18" t="inlineStr">
         <is>
           <t>MIT araştırmacıları antik Roma betonunun sırrını çözdü: Harçtaki sıcak kireç kırıntıları, yağmur suyu sızdığında kalsiyum kristallerine dönüşerek çatlakları kendiliğinden yamıyordu!
 Daha fazla bilgi dozu için takip etmeyi unutma!</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="E11" s="18" t="inlineStr">
         <is>
           <t>#bilgidozu #shorts #tarih #bilim</t>
         </is>
       </c>
-      <c r="F11" s="4" t="inlineStr">
+      <c r="F11" s="18" t="inlineStr">
         <is>
           <t>bilgidozu, roma, tarih, mühendislik, bilim, arkeoloji, shorts</t>
         </is>
       </c>
-      <c r="G11" s="4" t="inlineStr">
+      <c r="G11" s="18" t="inlineStr">
         <is>
           <t>2000 yıl dayanan Roma betonu mu, modern beton mu? 🏛️ Sence bu sırrı hâlâ neden çözemedik? 👇</t>
         </is>
       </c>
-      <c r="H11" s="4" t="inlineStr">
+      <c r="H11" s="18" t="inlineStr">
         <is>
           <t>Tarih ve Mühendislik</t>
         </is>
       </c>
-      <c r="I11" s="4" t="inlineStr">
-        <is>
-          <t>MIT News (2023 Roma betonu): https://news.mit.edu/2023/roman-concrete-durability-lime-casts-0106</t>
+      <c r="I11" s="18" t="inlineStr">
+        <is>
+          <t>YÜKLENDİ / ATLANDI (31'den Başlatma Kilidi)</t>
         </is>
       </c>
       <c r="J11" s="5" t="n"/>
@@ -1273,50 +1283,50 @@
       <c r="AC11" s="6" t="n"/>
     </row>
     <row r="12" ht="112.5" customHeight="1" s="13">
-      <c r="A12" s="3" t="inlineStr">
+      <c r="A12" s="17" t="inlineStr">
         <is>
           <t>YÜKLENDİ</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B12" s="18" t="inlineStr">
         <is>
           <t>video_11.mp4</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C12" s="18" t="inlineStr">
         <is>
           <t>Gökten Yağmur Değil Dev Elmaslar Yağan Gezegenler! 💎🪐 #bilgidozu #shorts</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D12" s="18" t="inlineStr">
         <is>
           <t>Neptün ve Uranüs'ün derin atmosferindeki aşırı basınç ve sıcaklık, metan gazındaki karbon atomlarını saf elmas kristallerine dönüştürüp gökten elmas dolusu gibi yağdırıyor!
 Daha fazla bilgi dozu için takip etmeyi unutma!</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="E12" s="18" t="inlineStr">
         <is>
           <t>#bilgidozu #shorts #uzay #bilim</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="F12" s="18" t="inlineStr">
         <is>
           <t>bilgidozu, uzay, elmas, neptün, uranüs, bilim, shorts</t>
         </is>
       </c>
-      <c r="G12" s="4" t="inlineStr">
+      <c r="G12" s="18" t="inlineStr">
         <is>
           <t>Neptün'de elmas yağdığını bilseydin oraya taşınmaya değer miydi? 💎😄 Sen olsan ne yapardın? 👇</t>
         </is>
       </c>
-      <c r="H12" s="4" t="inlineStr">
+      <c r="H12" s="18" t="inlineStr">
         <is>
           <t>Uzay ve Astronomi</t>
         </is>
       </c>
-      <c r="I12" s="4" t="inlineStr">
-        <is>
-          <t>SLAC (2017 elmas yağmuru deneyi): https://www6.slac.stanford.edu/news/2017-08-21-scientists-create-diamond-rain-forms-interior-icy-giant-planets</t>
+      <c r="I12" s="18" t="inlineStr">
+        <is>
+          <t>YÜKLENDİ / ATLANDI (31'den Başlatma Kilidi)</t>
         </is>
       </c>
       <c r="J12" s="5" t="n"/>
@@ -1341,50 +1351,50 @@
       <c r="AC12" s="6" t="n"/>
     </row>
     <row r="13" ht="112.5" customHeight="1" s="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="A13" s="17" t="inlineStr">
         <is>
           <t>YÜKLENDİ</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B13" s="18" t="inlineStr">
         <is>
           <t>video_12.mp4</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C13" s="18" t="inlineStr">
         <is>
           <t>Bu Canlı Uzay Boşluğunda ve Radyasyonda Bile Ölmüyor! 🐻🔬 #bilgidozu #shorts</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D13" s="18" t="inlineStr">
         <is>
           <t>Mikroskobik su ayıları (tardigradlar), -272 dereceden +150 dereceye, ölümcül radyasyondan açık uzayın dondurucu vakumuna kadar her koşulda hayatta kalabiliyor!
 Daha fazla bilgi dozu için takip etmeyi unutma!</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="E13" s="18" t="inlineStr">
         <is>
           <t>#bilgidozu #shorts #bilim</t>
         </is>
       </c>
-      <c r="F13" s="4" t="inlineStr">
+      <c r="F13" s="18" t="inlineStr">
         <is>
           <t>bilgidozu, tardigrad, uzay, biyoloji, ilginçbilgiler, bilim, shorts</t>
         </is>
       </c>
-      <c r="G13" s="4" t="inlineStr">
+      <c r="G13" s="18" t="inlineStr">
         <is>
           <t>Tardigradlar Dünya'nın en dayanıklı canlısı mı? 🐻🔬 Oy ver: EVET / HAYIR 👇</t>
         </is>
       </c>
-      <c r="H13" s="4" t="inlineStr">
+      <c r="H13" s="18" t="inlineStr">
         <is>
           <t>Biyoloji ve Uzay</t>
         </is>
       </c>
-      <c r="I13" s="4" t="inlineStr">
-        <is>
-          <t>Tardigrada: https://en.wikipedia.org/wiki/Tardigrade</t>
+      <c r="I13" s="18" t="inlineStr">
+        <is>
+          <t>YÜKLENDİ / ATLANDI (31'den Başlatma Kilidi)</t>
         </is>
       </c>
       <c r="J13" s="5" t="n"/>
@@ -1409,51 +1419,50 @@
       <c r="AC13" s="6" t="n"/>
     </row>
     <row r="14" ht="112.5" customHeight="1" s="13">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="A14" s="17" t="inlineStr">
         <is>
           <t>YÜKLENDİ</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B14" s="18" t="inlineStr">
         <is>
           <t>video_13.mp4</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C14" s="18" t="inlineStr">
         <is>
           <t>Birinin Sizden Hoşlandığını Anlamanın En Kesin Yolu! 👁️✨ #bilgidozu #shorts</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="D14" s="18" t="inlineStr">
         <is>
           <t>Beyin bir şeye aşırı odaklandığında veya heyecanlandığında otonom sinir sistemi devreye girer ve göz bebekleri normal boyutunun %45'ine kadar kontrolsüzce genişler!
 Daha fazla bilgi dozu için takip etmeyi unutma!</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="E14" s="18" t="inlineStr">
         <is>
           <t>#bilgidozu #shorts #beyin #psikoloji</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
+      <c r="F14" s="18" t="inlineStr">
         <is>
           <t>bilgidozu, psikoloji, beyin, gözler, nörobilim, shorts</t>
         </is>
       </c>
-      <c r="G14" s="4" t="inlineStr">
+      <c r="G14" s="18" t="inlineStr">
         <is>
           <t>Şu an aynaya bak ve göz bebeklerini izle! 👁️ Kimin aklına kim geldi? 😄 Yaz bakalım! 👇</t>
         </is>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="H14" s="18" t="inlineStr">
         <is>
           <t>Beyin ve Psikoloji</t>
         </is>
       </c>
-      <c r="I14" s="4" t="inlineStr">
-        <is>
-          <t>Psychology Today (30+ çalışma meta-analizi): https://www.psychologytoday.com/us/blog/best-practices-in-health/202506/eyes-wide-open-what-your-eyes-reveal-about-attraction
-Yedek: https://www.medicalnewstoday.com/articles/dilated-pupils-meaning</t>
+      <c r="I14" s="18" t="inlineStr">
+        <is>
+          <t>YÜKLENDİ / ATLANDI (31'den Başlatma Kilidi)</t>
         </is>
       </c>
       <c r="J14" s="5" t="n"/>
@@ -1478,50 +1487,50 @@
       <c r="AC14" s="6" t="n"/>
     </row>
     <row r="15" ht="112.5" customHeight="1" s="13">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="A15" s="17" t="inlineStr">
         <is>
           <t>YÜKLENDİ</t>
         </is>
       </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B15" s="18" t="inlineStr">
         <is>
           <t>video_14.mp4</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C15" s="18" t="inlineStr">
         <is>
           <t>Dünyanın En Yaşlı Canlısı Bir Hayvan Değil, 80.000 Yaşındaki Bu Orman! 🌲⚡ #bilgidozu #shorts</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D15" s="18" t="inlineStr">
         <is>
           <t>Utah'taki Pando ormanı dışarıdan 47.000 ağaç gibi görünse de aslında tek bir dev kök sistemine bağlı, genetik olarak tamamen özdeş 80.000 yıllık dev bir canlıdır!
 Daha fazla bilgi dozu için takip etmeyi unutma!</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="E15" s="18" t="inlineStr">
         <is>
           <t>#bilgidozu #shorts #doğa #bilim</t>
         </is>
       </c>
-      <c r="F15" s="4" t="inlineStr">
+      <c r="F15" s="18" t="inlineStr">
         <is>
           <t>bilgidozu, pando, orman, ağaçlar, doğa, biyoloji, shorts</t>
         </is>
       </c>
-      <c r="G15" s="4" t="inlineStr">
+      <c r="G15" s="18" t="inlineStr">
         <is>
           <t>80.000 yıllık bu dev canlıya Pando'dan başka ne isim verirdin? 🌲 En yaratık ismi yazan pinned olur! 👇</t>
         </is>
       </c>
-      <c r="H15" s="4" t="inlineStr">
+      <c r="H15" s="18" t="inlineStr">
         <is>
           <t>Doğa ve Biyoloji</t>
         </is>
       </c>
-      <c r="I15" s="4" t="inlineStr">
-        <is>
-          <t>USDA Forest Service — Pando: https://www.fs.usda.gov/detail/fishlake/home/?cid=stelprdb5444544</t>
+      <c r="I15" s="18" t="inlineStr">
+        <is>
+          <t>YÜKLENDİ / ATLANDI (31'den Başlatma Kilidi)</t>
         </is>
       </c>
       <c r="J15" s="5" t="n"/>
@@ -1546,50 +1555,50 @@
       <c r="AC15" s="6" t="n"/>
     </row>
     <row r="16" ht="112.5" customHeight="1" s="13">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="A16" s="17" t="inlineStr">
         <is>
           <t>YÜKLENDİ</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B16" s="18" t="inlineStr">
         <is>
           <t>video_15.mp4</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C16" s="18" t="inlineStr">
         <is>
           <t>Gözlerinize İnanmayın: Yıldırımlar Aslında Aşağıdan Yukarıya Çakar! ⚡🌩️ #bilgidozu #shorts</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="D16" s="18" t="inlineStr">
         <is>
           <t>Görünmez öncü kanal yere ulaştığı anda, asıl devasa ışık ve enerji patlaması yerden gökyüzüne doğru saniyede 100.000 km hızla fırlar! Gözlerimiz bunu aşağı iniyor sanır!
 Daha fazla bilgi dozu için takip etmeyi unutma!</t>
         </is>
       </c>
-      <c r="E16" s="4" t="inlineStr">
+      <c r="E16" s="18" t="inlineStr">
         <is>
           <t>#bilgidozu #shorts #fizik #bilim</t>
         </is>
       </c>
-      <c r="F16" s="4" t="inlineStr">
+      <c r="F16" s="18" t="inlineStr">
         <is>
           <t>bilgidozu, yıldırım, fizik, şimşek, doğaolayları, bilim, shorts</t>
         </is>
       </c>
-      <c r="G16" s="4" t="inlineStr">
+      <c r="G16" s="18" t="inlineStr">
         <is>
           <t>Yıldırımın aslında aşağıdan yukarıya çaktığını biliyor muydun? ⚡ Şaşırdıysan '🤯' yaz! 👇</t>
         </is>
       </c>
-      <c r="H16" s="4" t="inlineStr">
+      <c r="H16" s="18" t="inlineStr">
         <is>
           <t>Fizik ve Doğa</t>
         </is>
       </c>
-      <c r="I16" s="4" t="inlineStr">
-        <is>
-          <t>NOAA/NWS — Lightning science: https://www.weather.gov/safety/lightning-scienceUSDA Forest Service — Pando: https://www.fs.usda.gov/detail/fishlake/home/?cid=stelprdb5444544</t>
+      <c r="I16" s="18" t="inlineStr">
+        <is>
+          <t>YÜKLENDİ / ATLANDI (31'den Başlatma Kilidi)</t>
         </is>
       </c>
       <c r="J16" s="5" t="n"/>
@@ -1842,49 +1851,49 @@
       <c r="AC19" s="6" t="n"/>
     </row>
     <row r="20" ht="112.5" customHeight="1" s="13">
-      <c r="A20" s="3" t="inlineStr">
+      <c r="A20" s="17" t="inlineStr">
         <is>
           <t>YÜKLENDİ</t>
         </is>
       </c>
-      <c r="B20" s="4" t="inlineStr">
+      <c r="B20" s="18" t="inlineStr">
         <is>
           <t>video_16.mp4</t>
         </is>
       </c>
-      <c r="C20" s="4" t="inlineStr">
+      <c r="C20" s="18" t="inlineStr">
         <is>
           <t>Jüpiter'de Dünya'dan Büyük Bir Fırtına 350 Yıldır DÖNÜYOR! 🌪️🪐 #bilgidozu #shorts</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr">
+      <c r="D20" s="18" t="inlineStr">
         <is>
           <t>Büyük Kızıl Leke, Jüpiter'in atmosferinde en az 350 yıldır süren dev bir fırtına — içine bütün Dünya rahatça sığar! Ama sürpriz son dakika haberi: son yıllarda hızla küçülüyor ve parçalanmaya başladı. Belki de biz, dev bir fırtınanın ölümüne tanık olan ilk insanlarız!</t>
         </is>
       </c>
-      <c r="E20" s="4" t="inlineStr">
+      <c r="E20" s="18" t="inlineStr">
         <is>
           <t>#bilgidozu #shorts #uzay #bilim</t>
         </is>
       </c>
-      <c r="F20" s="4" t="inlineStr">
+      <c r="F20" s="18" t="inlineStr">
         <is>
           <t>bilgidozu, jüpiter, uzay, fırtına, astronomi, nasa, shorts</t>
         </is>
       </c>
-      <c r="G20" s="4" t="inlineStr">
+      <c r="G20" s="18" t="inlineStr">
         <is>
           <t>350 yıllık fırtınanın kenarından uçak yolculuğu... 🌪️ Gider miydin? Cesurlar 1, akıllılar 2! 👇</t>
         </is>
       </c>
-      <c r="H20" s="4" t="inlineStr">
+      <c r="H20" s="18" t="inlineStr">
         <is>
           <t>Uzay ve Astronomi</t>
         </is>
       </c>
-      <c r="I20" s="4" t="inlineStr">
-        <is>
-          <t>NASA — Jupiter Facts: https://science.nasa.gov/jupiter/facts/</t>
+      <c r="I20" s="18" t="inlineStr">
+        <is>
+          <t>YÜKLENDİ / ATLANDI (31'den Başlatma Kilidi)</t>
         </is>
       </c>
       <c r="J20" s="5" t="n"/>
@@ -1909,49 +1918,49 @@
       <c r="AC20" s="6" t="n"/>
     </row>
     <row r="21" ht="112.5" customHeight="1" s="13">
-      <c r="A21" s="15" t="inlineStr">
+      <c r="A21" s="17" t="inlineStr">
         <is>
           <t>YÜKLENDİ</t>
         </is>
       </c>
-      <c r="B21" s="16" t="inlineStr">
+      <c r="B21" s="18" t="inlineStr">
         <is>
           <t>video_17.mp4</t>
         </is>
       </c>
-      <c r="C21" s="16" t="inlineStr">
+      <c r="C21" s="18" t="inlineStr">
         <is>
           <t>Everest'in 2.5 Katı Yüksekliğinde Bir Dağ Var — Ama Dünya'da Değil! 🌋🪐 #bilgidozu #shorts</t>
         </is>
       </c>
-      <c r="D21" s="16" t="inlineStr">
+      <c r="D21" s="18" t="inlineStr">
         <is>
           <t>Mars'taki Olympus Mons, yaklaşık 22 km yüksekliğiyle Everest'in 2.5 katı! Tabanı ise Arizona kadar geniş. Dünya'da bu dağın ağırlığı kendi kabuğunu çökerterek batmasına neden olurdu — Mars'ta kabuk buna izin veriyor!</t>
         </is>
       </c>
-      <c r="E21" s="16" t="inlineStr">
+      <c r="E21" s="18" t="inlineStr">
         <is>
           <t>#bilgidozu #shorts #uzay #bilim</t>
         </is>
       </c>
-      <c r="F21" s="16" t="inlineStr">
+      <c r="F21" s="18" t="inlineStr">
         <is>
           <t>bilgidozu, mars, olympusmons, uzay, geoloji, bilim, shorts</t>
         </is>
       </c>
-      <c r="G21" s="16" t="inlineStr">
+      <c r="G21" s="18" t="inlineStr">
         <is>
           <t>Olympus Mons'un zirvesinden manzara... 🌋 Peki tırmanır mıydın? Korkanlar 1, cesurlar 2! 👇</t>
         </is>
       </c>
-      <c r="H21" s="16" t="inlineStr">
+      <c r="H21" s="18" t="inlineStr">
         <is>
           <t>Uzay ve Astronomi</t>
         </is>
       </c>
-      <c r="I21" s="16" t="inlineStr">
-        <is>
-          <t>NASA — Mars Facts: https://science.nasa.gov/mars/facts/</t>
+      <c r="I21" s="18" t="inlineStr">
+        <is>
+          <t>YÜKLENDİ / ATLANDI (31'den Başlatma Kilidi)</t>
         </is>
       </c>
       <c r="J21" s="5" t="n"/>
@@ -1976,49 +1985,49 @@
       <c r="AC21" s="6" t="n"/>
     </row>
     <row r="22" ht="112.5" customHeight="1" s="13">
-      <c r="A22" s="15" t="inlineStr">
+      <c r="A22" s="17" t="inlineStr">
         <is>
           <t>YÜKLENDİ</t>
         </is>
       </c>
-      <c r="B22" s="16" t="inlineStr">
+      <c r="B22" s="18" t="inlineStr">
         <is>
           <t>video_18.mp4</t>
         </is>
       </c>
-      <c r="C22" s="16" t="inlineStr">
+      <c r="C22" s="18" t="inlineStr">
         <is>
           <t>Bu Hayvanın BEYNİ YOK — Ama Görüyor, Hissediyor! ⭐🌊 #bilgidozu #shorts</t>
         </is>
       </c>
-      <c r="D22" s="16" t="inlineStr">
+      <c r="D22" s="18" t="inlineStr">
         <is>
           <t>Denizyıldızının merkezî bir beyni yok: sinir sistemi kollarına yayılmış! Her kolun ucundaki minik gözcükler ışığı algılar, binlerce ayakçık tadar, kavrar ve yürür. Kafasız ama eksiksiz — doğanın en zarif dağıtık zekâ tasarımı!</t>
         </is>
       </c>
-      <c r="E22" s="16" t="inlineStr">
+      <c r="E22" s="18" t="inlineStr">
         <is>
           <t>#bilgidozu #shorts #doğa #bilim</t>
         </is>
       </c>
-      <c r="F22" s="16" t="inlineStr">
+      <c r="F22" s="18" t="inlineStr">
         <is>
           <t>bilgidozu, denizyıldızı, denizcanlıları, biyoloji, ilginçbilgiler, shorts</t>
         </is>
       </c>
-      <c r="G22" s="16" t="inlineStr">
+      <c r="G22" s="18" t="inlineStr">
         <is>
           <t>Beyinsiz ama görüyor, tadıyor, yürüyor... ⭐ Doğanın en garip tasarımı mı? 1 yazsın! 👇</t>
         </is>
       </c>
-      <c r="H22" s="16" t="inlineStr">
+      <c r="H22" s="18" t="inlineStr">
         <is>
           <t>Doğa ve Hayvanlar</t>
         </is>
       </c>
-      <c r="I22" s="16" t="inlineStr">
-        <is>
-          <t>Starfish: https://en.wikipedia.org/wiki/Starfish</t>
+      <c r="I22" s="18" t="inlineStr">
+        <is>
+          <t>YÜKLENDİ / ATLANDI (31'den Başlatma Kilidi)</t>
         </is>
       </c>
       <c r="J22" s="5" t="n"/>
@@ -2043,49 +2052,49 @@
       <c r="AC22" s="6" t="n"/>
     </row>
     <row r="23" ht="112.5" customHeight="1" s="13">
-      <c r="A23" s="15" t="inlineStr">
+      <c r="A23" s="17" t="inlineStr">
         <is>
           <t>YÜKLENDİ</t>
         </is>
       </c>
-      <c r="B23" s="16" t="inlineStr">
+      <c r="B23" s="18" t="inlineStr">
         <is>
           <t>video_19.mp4</t>
         </is>
       </c>
-      <c r="C23" s="16" t="inlineStr">
+      <c r="C23" s="18" t="inlineStr">
         <is>
           <t>Yunuslar Tek Gözü Açık Uyur! 🐬😴 #bilgidozu #shorts</t>
         </is>
       </c>
-      <c r="D23" s="16" t="inlineStr">
+      <c r="D23" s="18" t="inlineStr">
         <is>
           <t>Yunusun beyninin iki yarısı sırayla uyur: bir yarı derin uykudayken diğeri düşman nöbeti tutar, yüzer ve nefes aldırır! Göz de beynin uyuyan tarafına göre kapanır. Adı: yarım küre uykusu (USWS) — doğanın nöbetçi sistemi!</t>
         </is>
       </c>
-      <c r="E23" s="16" t="inlineStr">
+      <c r="E23" s="18" t="inlineStr">
         <is>
           <t>#bilgidozu #shorts #doğa #bilim</t>
         </is>
       </c>
-      <c r="F23" s="16" t="inlineStr">
+      <c r="F23" s="18" t="inlineStr">
         <is>
           <t>bilgidozu, yunus, hayvanlaralemi, uyku, deniz, bilim, shorts</t>
         </is>
       </c>
-      <c r="G23" s="16" t="inlineStr">
+      <c r="G23" s="18" t="inlineStr">
         <is>
           <t>Yunus bile nöbet tutarak uyurken sen nasıl uyuyorsun? 😄🐬 Uykucular 1 yazsın!</t>
         </is>
       </c>
-      <c r="H23" s="16" t="inlineStr">
+      <c r="H23" s="18" t="inlineStr">
         <is>
           <t>Doğa ve Hayvanlar</t>
         </is>
       </c>
-      <c r="I23" s="16" t="inlineStr">
-        <is>
-          <t>Sleep Foundation — Animals and Sleep: https://www.sleepfoundation.org/animals-and-sleep</t>
+      <c r="I23" s="18" t="inlineStr">
+        <is>
+          <t>YÜKLENDİ / ATLANDI (31'den Başlatma Kilidi)</t>
         </is>
       </c>
       <c r="J23" s="5" t="n"/>
@@ -2110,49 +2119,49 @@
       <c r="AC23" s="6" t="n"/>
     </row>
     <row r="24" ht="112.5" customHeight="1" s="13">
-      <c r="A24" s="7" t="inlineStr">
+      <c r="A24" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">BEKLEMEDE </t>
         </is>
       </c>
-      <c r="B24" s="14" t="inlineStr">
+      <c r="B24" s="18" t="inlineStr">
         <is>
           <t>video_20.mp4</t>
         </is>
       </c>
-      <c r="C24" s="14" t="inlineStr">
+      <c r="C24" s="18" t="inlineStr">
         <is>
           <t>Satürn Suda Yüzebilecek Kadar Hafif! 🪐💧 #bilgidozu #shorts</t>
         </is>
       </c>
-      <c r="D24" s="14" t="inlineStr">
+      <c r="D24" s="18" t="inlineStr">
         <is>
           <t>Satürn'ün ortalama yoğunluğu sudan düşük: 0,7 g/cm³! Yani düşünen bir gezegen — yeterince büyük bir okyanus bulsaydık Satürn üstünde yüzebilirdi. Dev ama tüy gibi hafif: çoğu hidrojen ve helyumdan ibaret bir gaz topu.</t>
         </is>
       </c>
-      <c r="E24" s="14" t="inlineStr">
+      <c r="E24" s="18" t="inlineStr">
         <is>
           <t>#bilgidozu #shorts #uzay #bilim</t>
         </is>
       </c>
-      <c r="F24" s="14" t="inlineStr">
+      <c r="F24" s="18" t="inlineStr">
         <is>
           <t>bilgidozu, satürn, uzay, gezegenler, ilginçbilgiler, bilim, shorts</t>
         </is>
       </c>
-      <c r="G24" s="14" t="inlineStr">
+      <c r="G24" s="18" t="inlineStr">
         <is>
           <t>Satürn'ü küvette yüzerken hayal et 🪐💧 İnananlar 1, inanmayanlar 2! 👇</t>
         </is>
       </c>
-      <c r="H24" s="14" t="inlineStr">
+      <c r="H24" s="18" t="inlineStr">
         <is>
           <t>Uzay ve Astronomi</t>
         </is>
       </c>
-      <c r="I24" s="14" t="inlineStr">
-        <is>
-          <t>NASA — Saturn Facts: https://science.nasa.gov/saturn/facts/</t>
+      <c r="I24" s="18" t="inlineStr">
+        <is>
+          <t>YÜKLENDİ (https://youtu.be/MzkXjFsAZ90)</t>
         </is>
       </c>
       <c r="J24" s="5" t="n"/>
@@ -2177,49 +2186,49 @@
       <c r="AC24" s="6" t="n"/>
     </row>
     <row r="25" ht="112.5" customHeight="1" s="13">
-      <c r="A25" s="7" t="inlineStr">
+      <c r="A25" s="17" t="inlineStr">
         <is>
           <t>BEKLEMEDE</t>
         </is>
       </c>
-      <c r="B25" s="14" t="inlineStr">
+      <c r="B25" s="18" t="inlineStr">
         <is>
           <t>video_21.mp4</t>
         </is>
       </c>
-      <c r="C25" s="14" t="inlineStr">
+      <c r="C25" s="18" t="inlineStr">
         <is>
           <t>Vücudundaki Bakteriler Hücrelerinden FAZLA! 🦠⚖️ #bilgidozu #shorts</t>
         </is>
       </c>
-      <c r="D25" s="14" t="inlineStr">
+      <c r="D25" s="18" t="inlineStr">
         <is>
           <t>Sende yaklaşık 38 trilyon bakteri var — insan hücrelerinden (30 trilyon) daha fazla! Ama korkma: toplam ağırlıkları 200 gram ve çoğu kahramanın: sindirimi yapıyor, bağışıklığını eğitiyor, vitamin üretiyor. Sen aslında yürüyen bir ekosistemsin!</t>
         </is>
       </c>
-      <c r="E25" s="14" t="inlineStr">
+      <c r="E25" s="18" t="inlineStr">
         <is>
           <t>#bilgidozu #shorts #bilim</t>
         </is>
       </c>
-      <c r="F25" s="14" t="inlineStr">
+      <c r="F25" s="18" t="inlineStr">
         <is>
           <t>bilgidozu, bakteriler, mikrobiyom, biyoloji, vücut, bilim, shorts</t>
         </is>
       </c>
-      <c r="G25" s="14" t="inlineStr">
+      <c r="G25" s="18" t="inlineStr">
         <is>
           <t>Kilonun 200 gramı bakteriymiş 🦠 Diyet listesine bakterilerini de yaz! 😄👇</t>
         </is>
       </c>
-      <c r="H25" s="14" t="inlineStr">
+      <c r="H25" s="18" t="inlineStr">
         <is>
           <t>Biyoloji ve Vücut</t>
         </is>
       </c>
-      <c r="I25" s="14" t="inlineStr">
-        <is>
-          <t>Human Microbiome: https://en.wikipedia.org/wiki/Human_microbiome</t>
+      <c r="I25" s="18" t="inlineStr">
+        <is>
+          <t>YÜKLENDİ / ATLANDI (31'den Başlatma Kilidi)</t>
         </is>
       </c>
       <c r="J25" s="5" t="n"/>
@@ -2244,49 +2253,49 @@
       <c r="AC25" s="6" t="n"/>
     </row>
     <row r="26" ht="112.5" customHeight="1" s="13">
-      <c r="A26" s="7" t="inlineStr">
+      <c r="A26" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">BEKLEMEDE </t>
         </is>
       </c>
-      <c r="B26" s="14" t="inlineStr">
+      <c r="B26" s="18" t="inlineStr">
         <is>
           <t>video_22.mp4</t>
         </is>
       </c>
-      <c r="C26" s="14" t="inlineStr">
+      <c r="C26" s="18" t="inlineStr">
         <is>
           <t>Cam Akar mı? Efsane ÇÖKTÜ — Cam Bir Katıdır! 🪟❌ #bilgidozu #shorts</t>
         </is>
       </c>
-      <c r="D26" s="14" t="inlineStr">
+      <c r="D26" s="18" t="inlineStr">
         <is>
           <t>Eski binaların camlarının altta kalın olması 'cam akıyor' kanıtı değil — eski camlar düzensiz üretiliyordu! Cam bir amorf katı: molekülleri katı gibi sıkışık ama düzensiz dizili. Penceren binlerce yıl sonra da aynı yerde duracak!</t>
         </is>
       </c>
-      <c r="E26" s="14" t="inlineStr">
+      <c r="E26" s="18" t="inlineStr">
         <is>
           <t>#bilgidozu #shorts #bilim</t>
         </is>
       </c>
-      <c r="F26" s="14" t="inlineStr">
+      <c r="F26" s="18" t="inlineStr">
         <is>
           <t>bilgidozu, cam, fizik, kimya, efsaneavrı, malzeme, bilim, shorts</t>
         </is>
       </c>
-      <c r="G26" s="14" t="inlineStr">
+      <c r="G26" s="18" t="inlineStr">
         <is>
           <t>'Cam akar' diyene bu videoyu gönder 🪟😄 Kaç kişi bu efsaneye inanıyordu? 👇</t>
         </is>
       </c>
-      <c r="H26" s="14" t="inlineStr">
+      <c r="H26" s="18" t="inlineStr">
         <is>
           <t>Fizik ve Kimya</t>
         </is>
       </c>
-      <c r="I26" s="14" t="inlineStr">
-        <is>
-          <t>Glass (cam bir katıdır): https://en.wikipedia.org/wiki/Glass</t>
+      <c r="I26" s="18" t="inlineStr">
+        <is>
+          <t>YÜKLENDİ / ATLANDI (31'den Başlatma Kilidi)</t>
         </is>
       </c>
       <c r="J26" s="5" t="n"/>
@@ -2311,49 +2320,49 @@
       <c r="AC26" s="6" t="n"/>
     </row>
     <row r="27" ht="112.5" customHeight="1" s="13">
-      <c r="A27" s="7" t="inlineStr">
+      <c r="A27" s="17" t="inlineStr">
         <is>
           <t>BEKLEMEDE</t>
         </is>
       </c>
-      <c r="B27" s="14" t="inlineStr">
+      <c r="B27" s="18" t="inlineStr">
         <is>
           <t>video_23.mp4</t>
         </is>
       </c>
-      <c r="C27" s="14" t="inlineStr">
+      <c r="C27" s="18" t="inlineStr">
         <is>
           <t>Ay Her Yıl Bizden 3.8 cm Uzaklaşıyor! 🌙➡️ #bilgidozu #shorts</t>
         </is>
       </c>
-      <c r="D27" s="14" t="inlineStr">
+      <c r="D27" s="18" t="inlineStr">
         <is>
           <t>Apollo astronotlarının Ay'a bıraktığı aynalara lazer atarak ölçüyoruz: Ay, Dünya'dan yılda ortalama 3.8 cm uzaklaşıyor! Milyonlarca yıl önce Ay gökyüzünde dev gibi görünüyordu — ve gelecekte çok daha küçük görünecek.</t>
         </is>
       </c>
-      <c r="E27" s="14" t="inlineStr">
+      <c r="E27" s="18" t="inlineStr">
         <is>
           <t>#bilgidozu #shorts #uzay #bilim</t>
         </is>
       </c>
-      <c r="F27" s="14" t="inlineStr">
+      <c r="F27" s="18" t="inlineStr">
         <is>
           <t>bilgidozu, ay, uzay, nasa, astronomi, ilginçbilgiler, shorts</t>
         </is>
       </c>
-      <c r="G27" s="14" t="inlineStr">
+      <c r="G27" s="18" t="inlineStr">
         <is>
           <t>Dev Ay'lı bir gökyüzünde gece yürüyüşü... 🌙 Ne hissederdin? 👇</t>
         </is>
       </c>
-      <c r="H27" s="14" t="inlineStr">
+      <c r="H27" s="18" t="inlineStr">
         <is>
           <t>Uzay ve Astronomi</t>
         </is>
       </c>
-      <c r="I27" s="14" t="inlineStr">
-        <is>
-          <t>NASA — Moon Facts: https://science.nasa.gov/moon/facts/</t>
+      <c r="I27" s="18" t="inlineStr">
+        <is>
+          <t>YÜKLENDİ / ATLANDI (31'den Başlatma Kilidi)</t>
         </is>
       </c>
       <c r="J27" s="5" t="n"/>
@@ -2378,49 +2387,49 @@
       <c r="AC27" s="6" t="n"/>
     </row>
     <row r="28" ht="112.5" customHeight="1" s="13">
-      <c r="A28" s="7" t="inlineStr">
+      <c r="A28" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">BEKLEMEDE </t>
         </is>
       </c>
-      <c r="B28" s="14" t="inlineStr">
+      <c r="B28" s="18" t="inlineStr">
         <is>
           <t>video_24.mp4</t>
         </is>
       </c>
-      <c r="C28" s="14" t="inlineStr">
+      <c r="C28" s="18" t="inlineStr">
         <is>
           <t>Kedinin Miyavı Aslında Sadece SANA! 🐱💬 #bilgidozu #shorts</t>
         </is>
       </c>
-      <c r="D28" s="14" t="inlineStr">
+      <c r="D28" s="18" t="inlineStr">
         <is>
           <t>Yetişkin kediler birbirlerine neredeyse hiç miyavlamaz! Miyavlama, binlerce yıllık evcilleşmeyle insanla iletişim için gelişti. Yani kedin 'miyav' derken gerçekten SENİNLE konuşuyor — ve araştırmalar onun bu dili seni yönetmek için kullandığını gösteriyor!</t>
         </is>
       </c>
-      <c r="E28" s="14" t="inlineStr">
+      <c r="E28" s="18" t="inlineStr">
         <is>
           <t>#bilgidozu #shorts #doğa #bilim</t>
         </is>
       </c>
-      <c r="F28" s="14" t="inlineStr">
+      <c r="F28" s="18" t="inlineStr">
         <is>
           <t>bilgidozu, kedi, hayvanlaralemi, evcilhayvan, iletişim, shorts</t>
         </is>
       </c>
-      <c r="G28" s="14" t="inlineStr">
+      <c r="G28" s="18" t="inlineStr">
         <is>
           <t>Kedin seninle mi konuşuyor, seni mi yönetiyor? 🐱😤 İtiraf et, yorumlara yaz! 👇</t>
         </is>
       </c>
-      <c r="H28" s="14" t="inlineStr">
+      <c r="H28" s="18" t="inlineStr">
         <is>
           <t>Doğa ve Hayvanlar</t>
         </is>
       </c>
-      <c r="I28" s="14" t="inlineStr">
-        <is>
-          <t>Cat communication (miyav): https://en.wikipedia.org/wiki/Cat_communication</t>
+      <c r="I28" s="18" t="inlineStr">
+        <is>
+          <t>YÜKLENDİ / ATLANDI (31'den Başlatma Kilidi)</t>
         </is>
       </c>
       <c r="J28" s="5" t="n"/>
@@ -2445,49 +2454,49 @@
       <c r="AC28" s="6" t="n"/>
     </row>
     <row r="29" ht="112.5" customHeight="1" s="13">
-      <c r="A29" s="7" t="inlineStr">
+      <c r="A29" s="17" t="inlineStr">
         <is>
           <t>BEKLEMEDE</t>
         </is>
       </c>
-      <c r="B29" s="14" t="inlineStr">
+      <c r="B29" s="18" t="inlineStr">
         <is>
           <t>video_25.mp4</t>
         </is>
       </c>
-      <c r="C29" s="14" t="inlineStr">
+      <c r="C29" s="18" t="inlineStr">
         <is>
           <t>Şu An Saniyede 30 km Hızla Uçuyorsun — ve Hissetmiyorsun! 🌍💨 #bilgidozu #shorts</t>
         </is>
       </c>
-      <c r="D29" s="14" t="inlineStr">
+      <c r="D29" s="18" t="inlineStr">
         <is>
           <t>Dünya, seni taşıyarak Güneş etrafında saniyede 30 km — saatte 107.000 km — hızla dolandır: bir kurşundan 40 kat hızlı! Ama neden hissetmiyorsun? Çünkü hız tek başına hissettirmez — sadece hız DEĞİŞİMİ hissedersin. Koltuğunda otururken dev bir roketle evreni geziyorsun!</t>
         </is>
       </c>
-      <c r="E29" s="14" t="inlineStr">
+      <c r="E29" s="18" t="inlineStr">
         <is>
           <t>#bilgidozu #shorts #bilim</t>
         </is>
       </c>
-      <c r="F29" s="14" t="inlineStr">
+      <c r="F29" s="18" t="inlineStr">
         <is>
           <t>bilgidozu, dünya, uzay, fizik, hız, ilginçbilgiler, shorts</t>
         </is>
       </c>
-      <c r="G29" s="14" t="inlineStr">
+      <c r="G29" s="18" t="inlineStr">
         <is>
           <t>Saatte 107.000 km hızda yolcu sensin 🚀 'Bunu bilmiyordum' diyenler 1 yazsın! 👇</t>
         </is>
       </c>
-      <c r="H29" s="14" t="inlineStr">
+      <c r="H29" s="18" t="inlineStr">
         <is>
           <t>Fizik ve Uzay</t>
         </is>
       </c>
-      <c r="I29" s="14" t="inlineStr">
-        <is>
-          <t>NASA — Earth Facts: https://science.nasa.gov/earth/facts/</t>
+      <c r="I29" s="18" t="inlineStr">
+        <is>
+          <t>YÜKLENDİ / ATLANDI (31'den Başlatma Kilidi)</t>
         </is>
       </c>
       <c r="J29" s="5" t="n"/>
@@ -2512,49 +2521,49 @@
       <c r="AC29" s="6" t="n"/>
     </row>
     <row r="30" ht="112.5" customHeight="1" s="13">
-      <c r="A30" s="7" t="inlineStr">
+      <c r="A30" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">BEKLEMEDE </t>
         </is>
       </c>
-      <c r="B30" s="14" t="inlineStr">
+      <c r="B30" s="18" t="inlineStr">
         <is>
           <t>video_26.mp4</t>
         </is>
       </c>
-      <c r="C30" s="14" t="inlineStr">
+      <c r="C30" s="18" t="inlineStr">
         <is>
           <t>3000 Yıllık Bal Hâlâ Yenilebilir! 🍯🏛️ #bilgidozu #shorts</t>
         </is>
       </c>
-      <c r="D30" s="14" t="inlineStr">
+      <c r="D30" s="18" t="inlineStr">
         <is>
           <t>Arkeologlar Mısır mezarlarında 3000 yıllık bal kavanozları buldu — bozulmamıştı! Balın nemi çeken yapısı, asiditesi ve hidrojen peroksiti bakterileri yaşamaz ediyor: doğru saklanırsa bal sonsuza kadar dayanır. Mutfağındaki bal da 'son kullanma tarihi' tanımıyor!</t>
         </is>
       </c>
-      <c r="E30" s="14" t="inlineStr">
+      <c r="E30" s="18" t="inlineStr">
         <is>
           <t>#bilgidozu #shorts #bilim</t>
         </is>
       </c>
-      <c r="F30" s="14" t="inlineStr">
+      <c r="F30" s="18" t="inlineStr">
         <is>
           <t>bilgidozu, bal, gıda, arkeoloji, ilginçbilgiler, bilim, shorts</t>
         </is>
       </c>
-      <c r="G30" s="14" t="inlineStr">
+      <c r="G30" s="18" t="inlineStr">
         <is>
           <t>Pantry'de 3000 yıllık bal olsa yer miydin? 🍯😄 Cesur olanlar 1! 👇</t>
         </is>
       </c>
-      <c r="H30" s="14" t="inlineStr">
+      <c r="H30" s="18" t="inlineStr">
         <is>
           <t>Biyoloji ve Gıda</t>
         </is>
       </c>
-      <c r="I30" s="14" t="inlineStr">
-        <is>
-          <t>Honey (raf ömrü): https://en.wikipedia.org/wiki/Honey</t>
+      <c r="I30" s="18" t="inlineStr">
+        <is>
+          <t>YÜKLENDİ / ATLANDI (31'den Başlatma Kilidi)</t>
         </is>
       </c>
       <c r="J30" s="5" t="n"/>
@@ -2579,49 +2588,49 @@
       <c r="AC30" s="6" t="n"/>
     </row>
     <row r="31" ht="112.5" customHeight="1" s="13">
-      <c r="A31" s="7" t="inlineStr">
+      <c r="A31" s="17" t="inlineStr">
         <is>
           <t>BEKLEMEDE</t>
         </is>
       </c>
-      <c r="B31" s="14" t="inlineStr">
+      <c r="B31" s="18" t="inlineStr">
         <is>
           <t>video_27.mp4</t>
         </is>
       </c>
-      <c r="C31" s="14" t="inlineStr">
+      <c r="C31" s="18" t="inlineStr">
         <is>
           <t>Ayağının Altında Güneş Kadar Sıcak Bir Top Var! 🌍🔥 #bilgidozu #shorts</t>
         </is>
       </c>
-      <c r="D31" s="14" t="inlineStr">
+      <c r="D31" s="18" t="inlineStr">
         <is>
           <t>Dünya'nın iç çekirdeği yaklaşık 5.400°C — Güneş'in YÜZEYİYLE aynı sıcaklık! 5.000 km derinlikteki bu demir-nikel top, manyetik kalkanımızı besliyor. Yani sen, bir yıldız yüzeyi sıcaklığında bir kalbin üstünde yaşıyorsun!</t>
         </is>
       </c>
-      <c r="E31" s="14" t="inlineStr">
+      <c r="E31" s="18" t="inlineStr">
         <is>
           <t>#bilgidozu #shorts #bilim</t>
         </is>
       </c>
-      <c r="F31" s="14" t="inlineStr">
+      <c r="F31" s="18" t="inlineStr">
         <is>
           <t>bilgidozu, dünya, jeoloji, çekirdek, bilim, ilginçbilgiler, shorts</t>
         </is>
       </c>
-      <c r="G31" s="14" t="inlineStr">
+      <c r="G31" s="18" t="inlineStr">
         <is>
           <t>Ayağının altında Güneş yüzeyi sıcaklığında bir çekirdek var 🔥 'Bunu bilmiyordum' diyenler? 👇</t>
         </is>
       </c>
-      <c r="H31" s="14" t="inlineStr">
+      <c r="H31" s="18" t="inlineStr">
         <is>
           <t>Yer Bilimleri</t>
         </is>
       </c>
-      <c r="I31" s="14" t="inlineStr">
-        <is>
-          <t>Earth's inner core: https://en.wikipedia.org/wiki/Earth%27s_inner_core</t>
+      <c r="I31" s="18" t="inlineStr">
+        <is>
+          <t>YÜKLENDİ / ATLANDI (31'den Başlatma Kilidi)</t>
         </is>
       </c>
       <c r="J31" s="5" t="n"/>
@@ -2646,49 +2655,49 @@
       <c r="AC31" s="6" t="n"/>
     </row>
     <row r="32" ht="112.5" customHeight="1" s="13">
-      <c r="A32" s="7" t="inlineStr">
+      <c r="A32" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">BEKLEMEDE </t>
         </is>
       </c>
-      <c r="B32" s="14" t="inlineStr">
+      <c r="B32" s="18" t="inlineStr">
         <is>
           <t>video_28.mp4</t>
         </is>
       </c>
-      <c r="C32" s="14" t="inlineStr">
+      <c r="C32" s="18" t="inlineStr">
         <is>
           <t>Filler AYAKLARIYLA Duyar — Topraktan Mesaj Gelir! 🐘📡 #bilgidozu #shorts</t>
         </is>
       </c>
-      <c r="D32" s="14" t="inlineStr">
+      <c r="D32" s="18" t="inlineStr">
         <is>
           <t>Filler sadece hortumuyla değil, AYAKLARIYLA da 'dinler': verdikleri derin gümbürtüler toprağı titreştirip kilometrelerce öteye ulaşır — uzaktaki fil bunu ayak tabanındaki yağ yastıklarıyla hisseder! Sürünün gizli toprak-altı mesajlaşma ağı var.</t>
         </is>
       </c>
-      <c r="E32" s="14" t="inlineStr">
+      <c r="E32" s="18" t="inlineStr">
         <is>
           <t>#bilgidozu #shorts #doğa #bilim</t>
         </is>
       </c>
-      <c r="F32" s="14" t="inlineStr">
+      <c r="F32" s="18" t="inlineStr">
         <is>
           <t>bilgidozu, fil, hayvanlaralemi, iletişim, doğa, bilim, shorts</t>
         </is>
       </c>
-      <c r="G32" s="14" t="inlineStr">
+      <c r="G32" s="18" t="inlineStr">
         <is>
           <t>Filler topraktan mesajlaşırken biz 5G peşindeyiz 🐘📶😄 En şaşırtıcı bilgi miydi? 1 yazsın!</t>
         </is>
       </c>
-      <c r="H32" s="14" t="inlineStr">
+      <c r="H32" s="18" t="inlineStr">
         <is>
           <t>Doğa ve Hayvanlar</t>
         </is>
       </c>
-      <c r="I32" s="14" t="inlineStr">
-        <is>
-          <t>Elephant cognition (sismik iletişim): https://en.wikipedia.org/wiki/Elephant_cognition</t>
+      <c r="I32" s="18" t="inlineStr">
+        <is>
+          <t>YÜKLENDİ / ATLANDI (31'den Başlatma Kilidi)</t>
         </is>
       </c>
       <c r="J32" s="5" t="n"/>
@@ -2713,49 +2722,49 @@
       <c r="AC32" s="6" t="n"/>
     </row>
     <row r="33" ht="112.5" customHeight="1" s="13">
-      <c r="A33" s="7" t="inlineStr">
+      <c r="A33" s="17" t="inlineStr">
         <is>
           <t>BEKLEMEDE</t>
         </is>
       </c>
-      <c r="B33" s="14" t="inlineStr">
+      <c r="B33" s="18" t="inlineStr">
         <is>
           <t>video_29.mp4</t>
         </is>
       </c>
-      <c r="C33" s="14" t="inlineStr">
+      <c r="C33" s="18" t="inlineStr">
         <is>
           <t>Bu Gezegen YAN YATIK Döner — Gecesi 42 Yıl! 🪐🪑 #bilgidozu #shorts</t>
         </is>
       </c>
-      <c r="D33" s="14" t="inlineStr">
+      <c r="D33" s="18" t="inlineStr">
         <is>
           <t>Uranüs'ün dönme ekseni 98 derece eğik: gezegen neredeyse yan yatmış halde yuvarlanır! Kutuplarında bir gündüz veya gece 42 DÜNYA YILI sürer. Bilim insanları bunun sebebinin geçmişte dev bir cismin çarpması olduğunu düşünüyor.</t>
         </is>
       </c>
-      <c r="E33" s="14" t="inlineStr">
+      <c r="E33" s="18" t="inlineStr">
         <is>
           <t>#bilgidozu #shorts #uzay #bilim</t>
         </is>
       </c>
-      <c r="F33" s="14" t="inlineStr">
+      <c r="F33" s="18" t="inlineStr">
         <is>
           <t>bilgidozu, uranus, uzay, gezegenler, astronomi, shorts</t>
         </is>
       </c>
-      <c r="G33" s="14" t="inlineStr">
+      <c r="G33" s="18" t="inlineStr">
         <is>
           <t>42 yıllık bir karanlık gecede ne yapardın? 🌌😄 En yaratık cevabı sabitlerim! 👇</t>
         </is>
       </c>
-      <c r="H33" s="14" t="inlineStr">
+      <c r="H33" s="18" t="inlineStr">
         <is>
           <t>Uzay ve Astronomi</t>
         </is>
       </c>
-      <c r="I33" s="14" t="inlineStr">
-        <is>
-          <t>NASA — Uranus Facts: https://science.nasa.gov/uranus/facts/</t>
+      <c r="I33" s="18" t="inlineStr">
+        <is>
+          <t>YÜKLENDİ / ATLANDI (31'den Başlatma Kilidi)</t>
         </is>
       </c>
       <c r="J33" s="5" t="n"/>
@@ -2780,49 +2789,49 @@
       <c r="AC33" s="6" t="n"/>
     </row>
     <row r="34" ht="112.5" customHeight="1" s="13">
-      <c r="A34" s="7" t="inlineStr">
+      <c r="A34" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">BEKLEMEDE </t>
         </is>
       </c>
-      <c r="B34" s="14" t="inlineStr">
+      <c r="B34" s="18" t="inlineStr">
         <is>
           <t>video_30.mp4</t>
         </is>
       </c>
-      <c r="C34" s="14" t="inlineStr">
+      <c r="C34" s="18" t="inlineStr">
         <is>
           <t>Beynin Sadece %10'unu Kullandığın YALAN! İşte Kanıtı! 🧠❌ #bilgidozu #shorts</t>
         </is>
       </c>
-      <c r="D34" s="14" t="inlineStr">
+      <c r="D34" s="18" t="inlineStr">
         <is>
           <t>'İnsan beyninin sadece %10'unu kullanır' dedikodusu tam bir şehir efsanesi — beyin görüntüleme bunu çökertti: gün içinde beyninin neredeyse TAMAMI aktif, uykuda bile! Efsanenin kökeni 1900'lerin başındaki motivasyon konuşmaları. Yani kötü haber: daha kullanmadığın bir bölüm yok — zaten %100'ünle çalışıyorsun!</t>
         </is>
       </c>
-      <c r="E34" s="14" t="inlineStr">
+      <c r="E34" s="18" t="inlineStr">
         <is>
           <t>#bilgidozu #shorts #beyin #psikoloji</t>
         </is>
       </c>
-      <c r="F34" s="14" t="inlineStr">
+      <c r="F34" s="18" t="inlineStr">
         <is>
           <t>bilgidozu, beyin, efsaneavrı, nörobilim, psikoloji, bilim, shorts</t>
         </is>
       </c>
-      <c r="G34" s="14" t="inlineStr">
+      <c r="G34" s="18" t="inlineStr">
         <is>
           <t>'%10' efsanesine inananlar 1, şüpheci olanlar 2! 😄 Gerçek cevap yorumlarda! 👇</t>
         </is>
       </c>
-      <c r="H34" s="14" t="inlineStr">
+      <c r="H34" s="18" t="inlineStr">
         <is>
           <t>Beyin ve Psikoloji</t>
         </is>
       </c>
-      <c r="I34" s="14" t="inlineStr">
-        <is>
-          <t>Ten percent of brain myth: https://en.wikipedia.org/wiki/Ten_percent_of_brain_myth</t>
+      <c r="I34" s="18" t="inlineStr">
+        <is>
+          <t>YÜKLENDİ / ATLANDI (31'den Başlatma Kilidi)</t>
         </is>
       </c>
       <c r="J34" s="5" t="n"/>

</xml_diff>

<commit_message>
Add approved video_134 to live queue manifest and sync official 131-134 metadata
</commit_message>
<xml_diff>
--- a/bilgidozu_yukleme_tablosu.xlsx
+++ b/bilgidozu_yukleme_tablosu.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -61,8 +61,19 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="007F6000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00222222"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -93,6 +104,12 @@
         <bgColor rgb="00E0E0E0"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF9C4"/>
+        <bgColor rgb="00FFF9C4"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -107,7 +124,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -134,6 +151,12 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -501,7 +524,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M137"/>
+  <dimension ref="A1:M138"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -8128,7 +8151,7 @@
       </c>
       <c r="C135" s="9" t="inlineStr">
         <is>
-          <t>Kâğıt Kesiği Neden Bu Kadar Acıtır? 🩹</t>
+          <t>Küçücük Kâğıt Kesiği Neden Bu Kadar Çok Acıtır? 🩹⚡ #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D135" s="9" t="inlineStr">
@@ -8171,114 +8194,202 @@
       <c r="M135" s="9" t="n"/>
     </row>
     <row r="136">
-      <c r="A136" s="9" t="inlineStr">
+      <c r="A136" s="10" t="inlineStr">
         <is>
           <t>BEKLEMEDE</t>
         </is>
       </c>
-      <c r="B136" s="9" t="inlineStr">
+      <c r="B136" s="10" t="inlineStr">
         <is>
           <t>video_132.mp4</t>
         </is>
       </c>
-      <c r="C136" s="9" t="inlineStr">
-        <is>
-          <t>Baldırın İkinci Kalbin: Kanı Kalbe O Taşıyor! 🦵</t>
-        </is>
-      </c>
-      <c r="D136" s="9" t="inlineStr">
-        <is>
-          <t>Kalp kanı bacaklara kolayca gönderir; peki düşük basınçlı toplardamarlardaki kan yerçekimine karşı kalbe nasıl geri çıkar? Baldırımızdaki soleus ve gastroknemius kasları her adımda derin toplardamarları sıkıştırarak tek yönlü kapakçıklar yardımıyla kanı yukarı iter.
-💬 Bacaklarında akşamları ağırlık hissedenler 1 yazsın, hissetmeyenler 2! 👇
-📚 Kaynak: NCBI StatPearls (NBK430975, NBK534256) &amp; Cleveland Clinic (Dr. Teresa Wu)
-🎨 Görseller temsilîdir (AI bilimsel canlandırma).
-#bilgidozu #shorts #insanvücudu #biyoloji #bilim</t>
-        </is>
-      </c>
-      <c r="E136" s="9" t="inlineStr">
-        <is>
-          <t>#bilgidozu #shorts #insanvücudu #biyoloji #bilim</t>
-        </is>
-      </c>
-      <c r="F136" s="9" t="inlineStr">
-        <is>
-          <t>bilgi dozu, ikinci kalp, baldır kasları, kan dolaşımı, insan vücudu, bilim, shorts</t>
-        </is>
-      </c>
-      <c r="G136" s="9" t="inlineStr">
+      <c r="C136" s="11" t="inlineStr">
+        <is>
+          <t>Baldır Kasların Aslında İkinci Kalbin! Kanı Kalbe Nasıl Taşıyor? 🦵💪 #bilgidozu #shorts</t>
+        </is>
+      </c>
+      <c r="D136" s="11" t="inlineStr">
+        <is>
+          <t>Kalp kanı bacaklara gönderir; peki kan, yerçekimine karşı nasıl kalbe geri çıkar? Bu işi aslında baldırındaki kaslar yapıyor — "İkinci Kalp".
+📍 BÖLÜMLER
+00:00 Kan neden geri bu kadar zor çıkar?
+00:09 Toplardamarlarda basınç neden düşük?
+00:15 Baldır kasları: soleus ve gastroknemius
+00:24 Tek yönlü kapakçıklar nasıl çalışır?
+00:31 Hareketsizlik şişliği neden artırır?
+00:41 "İkinci kalp" gerçekten ne demek?
+📊 Kaynaklar:
+• StatPearls — Venous Insufficiency: https://www.ncbi.nlm.nih.gov/books/NBK430975/
+• NCBI Bookshelf — Varicose Veins (kas pompası fizyolojisi): https://www.ncbi.nlm.nih.gov/books/NBK534256/
+• StatPearls — Leg Posterior Compartment: https://www.ncbi.nlm.nih.gov/sites/books/NBK537340/
+• Cleveland Clinic (TODAY röportajı): https://www.today.com/health/diet-fitness/what-is-second-heart-rcna117576
+🩺 Uyarı: Genel bilgi amaçlıdır, tıbbi tavsiye değildir.
+🖼️ Görseller temsili (AI bilimsel canlandırma).
+Bir doz bilgi, her gün: 💊 ABONE OL!
+#bilgidozu #shorts #ikincikalp #baldır #kandolaşımı</t>
+        </is>
+      </c>
+      <c r="E136" s="11" t="inlineStr">
+        <is>
+          <t>#bilgidozu #shorts #ikincikalp #baldır #kandolaşımı</t>
+        </is>
+      </c>
+      <c r="F136" s="11" t="inlineStr">
+        <is>
+          <t>bilgidozu, shorts, ikinci kalp, baldır kasları, venöz pompa, kas pompası, toplardamar, kan kalbe nasıl döner, dolaşım sistemi, insan vücudu, bilgi dozu</t>
+        </is>
+      </c>
+      <c r="G136" s="11" t="inlineStr">
         <is>
           <t>Bacaklarında akşamları ağırlık hissedenler 1 yazsın, hissetmeyenler 2! 👇</t>
         </is>
       </c>
-      <c r="H136" s="9" t="inlineStr">
-        <is>
-          <t>Biyoloji ve Vücut</t>
-        </is>
-      </c>
-      <c r="I136" s="9" t="inlineStr">
-        <is>
-          <t>NCBI StatPearls (NBK430975, NBK534256) &amp; Cleveland Clinic (Dr. Teresa Wu)</t>
-        </is>
-      </c>
-      <c r="J136" s="9" t="n"/>
-      <c r="K136" s="9" t="n"/>
-      <c r="L136" s="9" t="n"/>
-      <c r="M136" s="9" t="n"/>
+      <c r="H136" s="11" t="inlineStr">
+        <is>
+          <t>İnsan Vücudu ve Beyin</t>
+        </is>
+      </c>
+      <c r="I136" s="11" t="inlineStr">
+        <is>
+          <t>StatPearls (NBK430975, NBK534256, NBK537340) &amp; Cleveland Clinic</t>
+        </is>
+      </c>
+      <c r="J136" s="11" t="n"/>
+      <c r="K136" s="11" t="n"/>
+      <c r="L136" s="11" t="n"/>
+      <c r="M136" s="11" t="n"/>
     </row>
     <row r="137">
-      <c r="A137" s="9" t="inlineStr">
+      <c r="A137" s="10" t="inlineStr">
         <is>
           <t>BEKLEMEDE</t>
         </is>
       </c>
-      <c r="B137" s="9" t="inlineStr">
+      <c r="B137" s="10" t="inlineStr">
         <is>
           <t>video_133.mp4</t>
         </is>
       </c>
-      <c r="C137" s="9" t="inlineStr">
-        <is>
-          <t>Göz Kapağın Seğirirse Vücut Ne Anlatıyor? 👁</t>
-        </is>
-      </c>
-      <c r="D137" s="9" t="inlineStr">
-        <is>
-          <t>Gözünün altında başlayan istemsiz seğirme (oküler miyokimi) çoğu zaman korkutucu gelse de genellikle beynin değil, uykusuzluk, yoğun stres, fazla kafein ve ekran yorgunluğuyla geçici olarak aşırı uyarılan küçük sinir uçlarının eseridir.
-💬 Göz kapağı seğirmesi daha önce yaşayanlar 1, ilk kez duyanlar 2 yazsın! 👇
-📚 Kaynak: Mayo Clinic &amp; Cleveland Clinic — Eyelid Myokymia
-🎨 Görseller temsilîdir (AI bilimsel canlandırma).
-#bilgidozu #shorts #beyin #insanvücudu #bilim</t>
-        </is>
-      </c>
-      <c r="E137" s="9" t="inlineStr">
-        <is>
-          <t>#bilgidozu #shorts #beyin #insanvücudu #bilim</t>
-        </is>
-      </c>
-      <c r="F137" s="9" t="inlineStr">
-        <is>
-          <t>bilgi dozu, göz seğirmesi, miyokimi, beyin ve psikoloji, insan vücudu, bilim, shorts</t>
-        </is>
-      </c>
-      <c r="G137" s="9" t="inlineStr">
+      <c r="C137" s="11" t="inlineStr">
+        <is>
+          <t>Göz Kapağın Neden Kendi Kendine Seğirir? Anlamı Bu! 👁🧠 #bilgidozu #shorts</t>
+        </is>
+      </c>
+      <c r="D137" s="11" t="inlineStr">
+        <is>
+          <t>Gözünün altındaki o minik seğirme ne anlama geliyor? Tıbbi adı miyokimi; çoğu zaman zararsız ve kendiliğinden geçiyor.
+📍 BÖLÜMLER
+00:00 Göz kapağı seğirmesi (miyokimi) nedir?
+00:09 Orbicularis oculi kas lifleri
+00:18 Kaynağı beynin değil, sinir uçlarının
+00:26 Tetikleyiciler: uykusuzluk, stres, kafein, ekran
+00:35 Magnezyum efsanesi ve ne zaman doktora gitmeli?
+00:43 Sıradaki bölüm: bulaşıcı esneme
+📊 Kaynaklar:
+• Mayo Clinic — Eye twitching: https://www.mayoclinic.org/symptoms/eye-twitching/basics/causes/sym-20050838
+• Cleveland Clinic — Myokymia: https://my.clevelandclinic.org/health/diseases/myokymia
+• UCLA Health — Twitching Eyelid: https://www.uclahealth.org/medical-services/ophthalmology/eye-signs-and-symptoms/twitching-eyelid
+🩺 Uyarı: Genel bilgi amaçlıdır, tıbbi tavsiye değildir.
+🖼️ Görseller temsili (AI bilimsel canlandırma).
+Bir doz bilgi, her gün: 💊 ABONE OL!
+#bilgidozu #shorts #gözkapağı #miyokimi #beyinsağlığı</t>
+        </is>
+      </c>
+      <c r="E137" s="11" t="inlineStr">
+        <is>
+          <t>#bilgidozu #shorts #gözkapağı #miyokimi #beyinsağlığı</t>
+        </is>
+      </c>
+      <c r="F137" s="11" t="inlineStr">
+        <is>
+          <t>bilgidozu, shorts, göz kapağı seğirmesi, miyokimi, göz seğirmesi, göz tiki, stres, kafein, uykusuzluk, insan vücudu, bilgi dozu</t>
+        </is>
+      </c>
+      <c r="G137" s="11" t="inlineStr">
         <is>
           <t>Göz kapağı seğirmesi daha önce yaşayanlar 1, ilk kez duyanlar 2 yazsın! 👇</t>
         </is>
       </c>
-      <c r="H137" s="9" t="inlineStr">
-        <is>
-          <t>Beyin ve Psikoloji</t>
-        </is>
-      </c>
-      <c r="I137" s="9" t="inlineStr">
-        <is>
-          <t>Mayo Clinic &amp; Cleveland Clinic — Eyelid Myokymia</t>
-        </is>
-      </c>
-      <c r="J137" s="9" t="n"/>
-      <c r="K137" s="9" t="n"/>
-      <c r="L137" s="9" t="n"/>
-      <c r="M137" s="9" t="n"/>
+      <c r="H137" s="11" t="inlineStr">
+        <is>
+          <t>İnsan Vücudu ve Beyin</t>
+        </is>
+      </c>
+      <c r="I137" s="11" t="inlineStr">
+        <is>
+          <t>Mayo Clinic, Cleveland Clinic &amp; UCLA Health — Eyelid Myokymia</t>
+        </is>
+      </c>
+      <c r="J137" s="11" t="n"/>
+      <c r="K137" s="11" t="n"/>
+      <c r="L137" s="11" t="n"/>
+      <c r="M137" s="11" t="n"/>
+    </row>
+    <row r="138">
+      <c r="A138" s="10" t="inlineStr">
+        <is>
+          <t>BEKLEMEDE</t>
+        </is>
+      </c>
+      <c r="B138" s="10" t="inlineStr">
+        <is>
+          <t>video_134.mp4</t>
+        </is>
+      </c>
+      <c r="C138" s="11" t="inlineStr">
+        <is>
+          <t>Bir Esnedin, Etraf da Esnedi! Esnemenin Bulaşma Sırrı 😮🧠 #bilgidozu #shorts</t>
+        </is>
+      </c>
+      <c r="D138" s="11" t="inlineStr">
+        <is>
+          <t>Esneme neden bu kadar kolay bulaşıyor — ve neden bazı insanlara hiç bulaşmıyor? Cevap, yakınlık sırasına gizlenmiş.
+📍 BÖLÜMLER
+00:00 Neden herkesten aynı oranda bulaşmaz?
+00:10 Normal esneme ile bulaşıcı esneme farkı
+00:21 Pisa araştırması: akraba &gt; arkadaş &gt; yabancı
+00:35 Şempanzelerde de aynı desen
+00:40 Çocuklarda 4 yaş sonrası belirginleşme
+00:46 Sıradaki bölüm: güneşte hapşırma (ACHOO)
+📊 Kaynaklar:
+• Norscia &amp; Palagi (2011) PLoS ONE: https://journals.plos.org/plosone/article?id=10.1371/journal.pone.0028472
+• Campbell &amp; de Waal (2011) PLoS ONE: https://journals.plos.org/plosone/article?id=10.1371/journal.pone.0018283
+• Yavru şempanzelerde yaşla artan bulaşma (2013): https://journals.plos.org/plosone/article?id=10.1371/journal.pone.0076266
+🖼️ Görseller temsili (AI bilimsel canlandırma).
+Bir doz bilgi, her gün: 💊 ABONE OL!
+#bilgidozu #shorts #esneme #empati #beyin</t>
+        </is>
+      </c>
+      <c r="E138" s="11" t="inlineStr">
+        <is>
+          <t>#bilgidozu #shorts #esneme #empati #beyin</t>
+        </is>
+      </c>
+      <c r="F138" s="11" t="inlineStr">
+        <is>
+          <t>bilgidozu, shorts, bulaşıcı esneme, esneme neden bulaşır, empati, şempanze, sosyal davranış, beyin, psikoloji, bilgi dozu</t>
+        </is>
+      </c>
+      <c r="G138" s="11" t="inlineStr">
+        <is>
+          <t>Sana en çok kim esneme bulaştırır? Akraba 1, arkadaş 2, yabancı 3 yazsın! 👇</t>
+        </is>
+      </c>
+      <c r="H138" s="11" t="inlineStr">
+        <is>
+          <t>İnsan Vücudu ve Beyin</t>
+        </is>
+      </c>
+      <c r="I138" s="11" t="inlineStr">
+        <is>
+          <t>Norscia &amp; Palagi (2011) PLoS ONE &amp; Campbell &amp; de Waal (2011)</t>
+        </is>
+      </c>
+      <c r="J138" s="11" t="n"/>
+      <c r="K138" s="11" t="n"/>
+      <c r="L138" s="11" t="n"/>
+      <c r="M138" s="11" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add approved video_135 and video_136 to live queue manifest and sync metadata
</commit_message>
<xml_diff>
--- a/bilgidozu_yukleme_tablosu.xlsx
+++ b/bilgidozu_yukleme_tablosu.xlsx
@@ -524,7 +524,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M138"/>
+  <dimension ref="A1:M140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -8391,6 +8391,137 @@
       <c r="L138" s="11" t="n"/>
       <c r="M138" s="11" t="n"/>
     </row>
+    <row r="139">
+      <c r="A139" s="10" t="inlineStr">
+        <is>
+          <t>BEKLEMEDE</t>
+        </is>
+      </c>
+      <c r="B139" s="10" t="inlineStr">
+        <is>
+          <t>video_135.mp4</t>
+        </is>
+      </c>
+      <c r="C139" s="11" t="inlineStr">
+        <is>
+          <t>Güneşe Dönünce Hapşırıyor musun? Bu Bir Refleks: ACHOO! ☀️🤧 #bilgidozu #shorts</t>
+        </is>
+      </c>
+      <c r="D139" s="11" t="inlineStr">
+        <is>
+          <t>Güneşli havada hapşırıyorsan bu bir alerji değil: fotik hapşırma refleksi, yani ACHOO. Toplumun yaklaşık %18–%35'inde var.
+📍 BÖLÜMLER
+00:00 Fotik hapşırma refleksi (ACHOO) nedir?
+00:06 Otozomal baskın kalıtsallık: ebeveynden biri yeter
+00:12 Toplumda %18–%35 görülme sıklığı
+00:24 Mekanizma: görme ve trigeminal sinir komşuluğu
+00:36 Çoklu kromozom genetik işaretleri
+00:42 Sıradaki bölüm: dondurma sızısı (brain freeze)
+📊 Kaynaklar:
+• Nature Scientific Reports (2019 GWAS): https://www.nature.com/articles/s41598-019-41551-0
+• Cleveland Clinic Journal of Medicine: https://www.ccjm.org/content/ccjom/54/5/431.full.pdf
+• Derleme: https://en.wikipedia.org/wiki/Photic_sneeze_reflex
+🖼️ Görseller temsili (AI bilimsel canlandırma).
+Bir doz bilgi, her gün: 💊 ABONE OL!
+#bilgidozu #shorts #ACHOO #hapşırma #genetik</t>
+        </is>
+      </c>
+      <c r="E139" s="11" t="inlineStr">
+        <is>
+          <t>#bilgidozu #shorts #ACHOO #hapşırma #genetik</t>
+        </is>
+      </c>
+      <c r="F139" s="11" t="inlineStr">
+        <is>
+          <t>bilgidozu, shorts, ACHOO, fotik hapşırma, güneş hapşırması, hapşırma refleksi, genetik, otozomal dominant, insan vücudu, bilgi dozu</t>
+        </is>
+      </c>
+      <c r="G139" s="11" t="inlineStr">
+        <is>
+          <t>Güneşte hapşırıyorsan 1 yaz, hiç tepki vermeyen 2 yazsın! 👇</t>
+        </is>
+      </c>
+      <c r="H139" s="11" t="inlineStr">
+        <is>
+          <t>İnsan Vücudu ve Beyin</t>
+        </is>
+      </c>
+      <c r="I139" s="11" t="inlineStr">
+        <is>
+          <t>Nature Scientific Reports (2019) &amp; Cleveland Clinic JM</t>
+        </is>
+      </c>
+      <c r="J139" s="11" t="n"/>
+      <c r="K139" s="11" t="n"/>
+      <c r="L139" s="11" t="n"/>
+      <c r="M139" s="11" t="n"/>
+    </row>
+    <row r="140">
+      <c r="A140" s="10" t="inlineStr">
+        <is>
+          <t>BEKLEMEDE</t>
+        </is>
+      </c>
+      <c r="B140" s="10" t="inlineStr">
+        <is>
+          <t>video_136.mp4</t>
+        </is>
+      </c>
+      <c r="C140" s="11" t="inlineStr">
+        <is>
+          <t>Dondurma Damağına Değer Ama Neden Alnın Sızlar? 🧊🧠 #bilgidozu #shorts</t>
+        </is>
+      </c>
+      <c r="D140" s="11" t="inlineStr">
+        <is>
+          <t>Soğuk bir dondurma ya da buzlu su üst damağına değdiği halde sızı neden bir anda alnının ortasına vurur? Cevap beynin acil ısınma savunmasında gizli.
+📍 BÖLÜMLER
+00:00 Ağızdaki soğuk neden alında sızlar?
+00:13 Harvard beyin ultrasonu araştırması
+00:18 Ön beyin atardamarının ani genişlemesi
+00:29 Trigeminal sinir ve alına yansıyan ağrı
+00:39 Damarın daralması ve dil-damak çözümü
+00:47 Sıradaki bölüm: müzik ürpertisi (frisson)
+📊 Kaynaklar:
+• Serrador ve ark. (2012) Harvard Medical School / The FASEB Journal, 26(1): 685.4
+• ScienceDaily (American Physiological Society): https://www.sciencedaily.com/releases/2012/04/120422231742.htm
+• Cleveland Clinic — Brain Freeze: https://health.clevelandclinic.org/what-causes-brain-freeze
+🩺 Uyarı: Genel bilgi amaçlıdır, tıbbi tavsiye değildir.
+🖼️ Görseller temsili (AI bilimsel canlandırma).
+Bir doz bilgi, her gün: 💊 ABONE OL!
+#bilgidozu #shorts #beyin #dondurma #insanvücudu</t>
+        </is>
+      </c>
+      <c r="E140" s="11" t="inlineStr">
+        <is>
+          <t>#bilgidozu #shorts #beyin #dondurma #insanvücudu</t>
+        </is>
+      </c>
+      <c r="F140" s="11" t="inlineStr">
+        <is>
+          <t>bilgidozu, shorts, dondurma baş ağrısı, brain freeze, ön beyin atardamarı, trigeminal sinir, yansıyan ağrı, beyin, insan vücudu, bilgi dozu</t>
+        </is>
+      </c>
+      <c r="G140" s="11" t="inlineStr">
+        <is>
+          <t>Dondurma ya da buzlu suda alnı sızlayanlar 1, hiç yaşamayanlar 2 yazsın! 👇</t>
+        </is>
+      </c>
+      <c r="H140" s="11" t="inlineStr">
+        <is>
+          <t>İnsan Vücudu ve Beyin</t>
+        </is>
+      </c>
+      <c r="I140" s="11" t="inlineStr">
+        <is>
+          <t>Harvard Medical School — Jorge Serrador et al. (2012) FASEB Journal</t>
+        </is>
+      </c>
+      <c r="J140" s="11" t="n"/>
+      <c r="K140" s="11" t="n"/>
+      <c r="L140" s="11" t="n"/>
+      <c r="M140" s="11" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
EMIR 025: floor 131->47 (CEO: video_47+ kullanimilir) + eski stok 47-111 (64 satir) ASKIDA->BEKLEMEDE
</commit_message>
<xml_diff>
--- a/bilgidozu_yukleme_tablosu.xlsx
+++ b/bilgidozu_yukleme_tablosu.xlsx
@@ -3422,7 +3422,7 @@
     <row r="49" ht="42" customHeight="1">
       <c r="A49" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B49" s="7" t="inlineStr">
@@ -3474,7 +3474,7 @@
     <row r="50" ht="42" customHeight="1">
       <c r="A50" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B50" s="7" t="inlineStr">
@@ -3526,7 +3526,7 @@
     <row r="51" ht="42" customHeight="1">
       <c r="A51" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B51" s="7" t="inlineStr">
@@ -3578,7 +3578,7 @@
     <row r="52" ht="42" customHeight="1">
       <c r="A52" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B52" s="7" t="inlineStr">
@@ -3633,7 +3633,7 @@
     <row r="53" ht="42" customHeight="1">
       <c r="A53" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B53" s="7" t="inlineStr">
@@ -3688,7 +3688,7 @@
     <row r="54" ht="42" customHeight="1">
       <c r="A54" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B54" s="7" t="inlineStr">
@@ -3743,7 +3743,7 @@
     <row r="55" ht="42" customHeight="1">
       <c r="A55" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B55" s="7" t="inlineStr">
@@ -3798,7 +3798,7 @@
     <row r="56" ht="42" customHeight="1">
       <c r="A56" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B56" s="7" t="inlineStr">
@@ -3853,7 +3853,7 @@
     <row r="57" ht="42" customHeight="1">
       <c r="A57" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B57" s="7" t="inlineStr">
@@ -3908,7 +3908,7 @@
     <row r="58" ht="42" customHeight="1">
       <c r="A58" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B58" s="7" t="inlineStr">
@@ -3963,7 +3963,7 @@
     <row r="59" ht="42" customHeight="1">
       <c r="A59" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B59" s="7" t="inlineStr">
@@ -4018,7 +4018,7 @@
     <row r="60" ht="42" customHeight="1">
       <c r="A60" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B60" s="7" t="inlineStr">
@@ -4073,7 +4073,7 @@
     <row r="61" ht="42" customHeight="1">
       <c r="A61" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B61" s="7" t="inlineStr">
@@ -4128,7 +4128,7 @@
     <row r="62" ht="42" customHeight="1">
       <c r="A62" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B62" s="7" t="inlineStr">
@@ -4183,7 +4183,7 @@
     <row r="63" ht="42" customHeight="1">
       <c r="A63" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B63" s="7" t="inlineStr">
@@ -4922,7 +4922,7 @@
     <row r="76" ht="42" customHeight="1">
       <c r="A76" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B76" s="7" t="inlineStr">
@@ -4974,7 +4974,7 @@
     <row r="77" ht="42" customHeight="1">
       <c r="A77" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B77" s="7" t="inlineStr">
@@ -5026,7 +5026,7 @@
     <row r="78" ht="42" customHeight="1">
       <c r="A78" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B78" s="7" t="inlineStr">
@@ -5078,7 +5078,7 @@
     <row r="79" ht="42" customHeight="1">
       <c r="A79" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B79" s="7" t="inlineStr">
@@ -5130,7 +5130,7 @@
     <row r="80" ht="42" customHeight="1">
       <c r="A80" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B80" s="7" t="inlineStr">
@@ -5186,7 +5186,7 @@
     <row r="81" ht="42" customHeight="1">
       <c r="A81" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B81" s="7" t="inlineStr">
@@ -5238,7 +5238,7 @@
     <row r="82" ht="42" customHeight="1">
       <c r="A82" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B82" s="7" t="inlineStr">
@@ -5290,7 +5290,7 @@
     <row r="83" ht="42" customHeight="1">
       <c r="A83" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B83" s="7" t="inlineStr">
@@ -5342,7 +5342,7 @@
     <row r="84" ht="42" customHeight="1">
       <c r="A84" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B84" s="7" t="inlineStr">
@@ -5394,7 +5394,7 @@
     <row r="85" ht="42" customHeight="1">
       <c r="A85" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B85" s="7" t="inlineStr">
@@ -5446,7 +5446,7 @@
     <row r="86" ht="42" customHeight="1">
       <c r="A86" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B86" s="7" t="inlineStr">
@@ -5501,7 +5501,7 @@
     <row r="87" ht="42" customHeight="1">
       <c r="A87" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B87" s="7" t="inlineStr">
@@ -5556,7 +5556,7 @@
     <row r="88" ht="42" customHeight="1">
       <c r="A88" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B88" s="7" t="inlineStr">
@@ -5611,7 +5611,7 @@
     <row r="89" ht="42" customHeight="1">
       <c r="A89" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B89" s="7" t="inlineStr">
@@ -5666,7 +5666,7 @@
     <row r="90" ht="42" customHeight="1">
       <c r="A90" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B90" s="7" t="inlineStr">
@@ -5721,7 +5721,7 @@
     <row r="91" ht="42" customHeight="1">
       <c r="A91" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B91" s="7" t="inlineStr">
@@ -5776,7 +5776,7 @@
     <row r="92" ht="42" customHeight="1">
       <c r="A92" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B92" s="7" t="inlineStr">
@@ -5831,7 +5831,7 @@
     <row r="93" ht="42" customHeight="1">
       <c r="A93" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B93" s="7" t="inlineStr">
@@ -5886,7 +5886,7 @@
     <row r="94" ht="42" customHeight="1">
       <c r="A94" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B94" s="7" t="inlineStr">
@@ -5941,7 +5941,7 @@
     <row r="95" ht="42" customHeight="1">
       <c r="A95" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B95" s="7" t="inlineStr">
@@ -5996,7 +5996,7 @@
     <row r="96" ht="42" customHeight="1">
       <c r="A96" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B96" s="7" t="inlineStr">
@@ -6051,7 +6051,7 @@
     <row r="97" ht="42" customHeight="1">
       <c r="A97" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B97" s="7" t="inlineStr">
@@ -6106,7 +6106,7 @@
     <row r="98" ht="42" customHeight="1">
       <c r="A98" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B98" s="7" t="inlineStr">
@@ -6161,7 +6161,7 @@
     <row r="99" ht="42" customHeight="1">
       <c r="A99" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B99" s="7" t="inlineStr">
@@ -6216,7 +6216,7 @@
     <row r="100" ht="42" customHeight="1">
       <c r="A100" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B100" s="7" t="inlineStr">
@@ -6271,7 +6271,7 @@
     <row r="101" ht="42" customHeight="1">
       <c r="A101" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B101" s="7" t="inlineStr">
@@ -6326,7 +6326,7 @@
     <row r="102" ht="42" customHeight="1">
       <c r="A102" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B102" s="7" t="inlineStr">
@@ -6381,7 +6381,7 @@
     <row r="103" ht="42" customHeight="1">
       <c r="A103" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B103" s="7" t="inlineStr">
@@ -6436,7 +6436,7 @@
     <row r="104" ht="42" customHeight="1">
       <c r="A104" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B104" s="7" t="inlineStr">
@@ -6491,7 +6491,7 @@
     <row r="105" ht="42" customHeight="1">
       <c r="A105" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B105" s="7" t="inlineStr">
@@ -6546,7 +6546,7 @@
     <row r="106" ht="42" customHeight="1">
       <c r="A106" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B106" s="7" t="inlineStr">
@@ -6601,7 +6601,7 @@
     <row r="107" ht="42" customHeight="1">
       <c r="A107" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B107" s="7" t="inlineStr">
@@ -6656,7 +6656,7 @@
     <row r="108" ht="42" customHeight="1">
       <c r="A108" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B108" s="7" t="inlineStr">
@@ -6711,7 +6711,7 @@
     <row r="109" ht="42" customHeight="1">
       <c r="A109" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B109" s="7" t="inlineStr">
@@ -6766,7 +6766,7 @@
     <row r="110" ht="42" customHeight="1">
       <c r="A110" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B110" s="7" t="inlineStr">
@@ -6821,7 +6821,7 @@
     <row r="111" ht="42" customHeight="1">
       <c r="A111" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B111" s="7" t="inlineStr">
@@ -6876,7 +6876,7 @@
     <row r="112" ht="42" customHeight="1">
       <c r="A112" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B112" s="7" t="inlineStr">
@@ -6931,7 +6931,7 @@
     <row r="113" ht="42" customHeight="1">
       <c r="A113" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B113" s="7" t="inlineStr">
@@ -6986,7 +6986,7 @@
     <row r="114" ht="42" customHeight="1">
       <c r="A114" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B114" s="7" t="inlineStr">
@@ -7041,7 +7041,7 @@
     <row r="115" ht="42" customHeight="1">
       <c r="A115" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B115" s="7" t="inlineStr">
@@ -7096,7 +7096,7 @@
     <row r="116" ht="42" customHeight="1">
       <c r="A116" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B116" s="7" t="inlineStr">
@@ -7151,7 +7151,7 @@
     <row r="117" ht="42" customHeight="1">
       <c r="A117" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B117" s="7" t="inlineStr">
@@ -7206,7 +7206,7 @@
     <row r="118" ht="42" customHeight="1">
       <c r="A118" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B118" s="7" t="inlineStr">
@@ -7261,7 +7261,7 @@
     <row r="119" ht="42" customHeight="1">
       <c r="A119" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B119" s="7" t="inlineStr">
@@ -7316,7 +7316,7 @@
     <row r="120" ht="42" customHeight="1">
       <c r="A120" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B120" s="7" t="inlineStr">
@@ -7371,7 +7371,7 @@
     <row r="121" ht="42" customHeight="1">
       <c r="A121" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B121" s="7" t="inlineStr">
@@ -7426,7 +7426,7 @@
     <row r="122" ht="42" customHeight="1">
       <c r="A122" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B122" s="7" t="inlineStr">
@@ -7481,7 +7481,7 @@
     <row r="123" ht="42" customHeight="1">
       <c r="A123" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B123" s="7" t="inlineStr">
@@ -7536,7 +7536,7 @@
     <row r="124" ht="42" customHeight="1">
       <c r="A124" s="7" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B124" s="7" t="inlineStr">

</xml_diff>

<commit_message>
EMIR 025b: havuzdaki 66 baslikta cift emoji -> tek (konu emojisi kalir, marka/ikinci emoji silindi)
</commit_message>
<xml_diff>
--- a/bilgidozu_yukleme_tablosu.xlsx
+++ b/bilgidozu_yukleme_tablosu.xlsx
@@ -3484,7 +3484,7 @@
       </c>
       <c r="C50" s="8" t="inlineStr">
         <is>
-          <t>Vücudunda Kanla Değil, Doğrudan Havadan Nefes Alan Tek Doku! 👁️🌬️ #bilgidozu #shorts</t>
+          <t>Vücudunda Kanla Değil, Doğrudan Havadan Nefes Alan Tek Doku! 👁️ #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D50" s="8" t="inlineStr">
@@ -3536,7 +3536,7 @@
       </c>
       <c r="C51" s="8" t="inlineStr">
         <is>
-          <t>Bacak Kasların Yorulurken Kalbin Neden Hayat Boyu Hiç Yorulmaz? ❤️⚡ #bilgidozu #shorts</t>
+          <t>Bacak Kasların Yorulurken Kalbin Neden Hayat Boyu Hiç Yorulmaz? ❤️ #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D51" s="8" t="inlineStr">
@@ -3588,7 +3588,7 @@
       </c>
       <c r="C52" s="8" t="inlineStr">
         <is>
-          <t>Suda Kalan Parmaklarımız Su Çektiği İçin Buruşmuyor! İşte Gerçek Sebebi! 🖐️💧 #bilgidozu #shorts</t>
+          <t>Suda Kalan Parmaklarımız Su Çektiği İçin Buruşmuyor! İşte Gerçek Sebebi! 🖐️ #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D52" s="8" t="inlineStr">
@@ -3698,7 +3698,7 @@
       </c>
       <c r="C54" s="8" t="inlineStr">
         <is>
-          <t>Ses Kaydındaki Sesin Sana Neden Bambaşka Geliyor? 🎙️🧠 #bilgidozu #shorts</t>
+          <t>Ses Kaydındaki Sesin Sana Neden Bambaşka Geliyor? 🎙️ #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D54" s="8" t="inlineStr">
@@ -3753,7 +3753,7 @@
       </c>
       <c r="C55" s="8" t="inlineStr">
         <is>
-          <t>Gözlerin Açıkken Hapşırmak Neden İmkansız? Beynin O Salisede Ne Yapar? 🤧👁️ #bilgidozu #shorts</t>
+          <t>Gözlerin Açıkken Hapşırmak Neden İmkansız? Beynin O Salisede Ne Yapar? 🤧 #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D55" s="8" t="inlineStr">
@@ -3808,7 +3808,7 @@
       </c>
       <c r="C56" s="8" t="inlineStr">
         <is>
-          <t>Kendi Sesini Kayıtta Dinleyince Neden Tuhaf Gelir? 🎙️🧠 #bilgidozu #shorts</t>
+          <t>Kendi Sesini Kayıtta Dinleyince Neden Tuhaf Gelir? 🎙️ #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D56" s="8" t="inlineStr">
@@ -3863,7 +3863,7 @@
       </c>
       <c r="C57" s="8" t="inlineStr">
         <is>
-          <t>Yüksek Bir Yerden Bakınca Beyin Neden 'Atla' Diye Fısıldar? 🧗‍♂️🧠 #bilgidozu #shorts</t>
+          <t>Yüksek Bir Yerden Bakınca Beyin Neden 'Atla' Diye Fısıldar? 🧗 #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D57" s="8" t="inlineStr">
@@ -3918,7 +3918,7 @@
       </c>
       <c r="C58" s="8" t="inlineStr">
         <is>
-          <t>Acı Biber Aslında Ağzını Yakmaz — Beynini Nasıl Kandırır? 🌶️🔥 #bilgidozu #shorts</t>
+          <t>Acı Biber Aslında Ağzını Yakmaz — Beynini Nasıl Kandırır? 🌶️ #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D58" s="8" t="inlineStr">
@@ -4193,7 +4193,7 @@
       </c>
       <c r="C63" s="8" t="inlineStr">
         <is>
-          <t>Sevdiğin Birine Bakınca Göz Bebeğin Neden Otomatik Büyür? 👀❤️ #bilgidozu #shorts</t>
+          <t>Sevdiğin Birine Bakınca Göz Bebeğin Neden Otomatik Büyür? 👀 #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D63" s="8" t="inlineStr">
@@ -5036,7 +5036,7 @@
       </c>
       <c r="C78" s="8" t="inlineStr">
         <is>
-          <t>Uzay Boşluk Olmasaydı Güneş'in Devasa Uğultusunu Dünya'dan Duyardık! ☀️🔊 #bilgidozu #shorts</t>
+          <t>Uzay Boşluk Olmasaydı Güneş'in Devasa Uğultusunu Dünya'dan Duyardık! ☀️ #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D78" s="8" t="inlineStr">
@@ -5088,7 +5088,7 @@
       </c>
       <c r="C79" s="8" t="inlineStr">
         <is>
-          <t>Tutankhamun'un Mezarındaki Hançer Uzaydan Gelen Göktaşından Yapılmış! 🗡️☄️ #bilgidozu #shorts</t>
+          <t>Tutankhamun'un Mezarındaki Hançer Uzaydan Gelen Göktaşından Yapılmış! 🗡️ #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D79" s="8" t="inlineStr">
@@ -5196,7 +5196,7 @@
       </c>
       <c r="C81" s="8" t="inlineStr">
         <is>
-          <t>Uçak Pencerelerinin Altındaki O Minik Delik Neden Var? ✈️🪟 #bilgidozu #shorts</t>
+          <t>Uçak Pencerelerinin Altındaki O Minik Delik Neden Var? ✈️ #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D81" s="8" t="inlineStr">
@@ -5511,7 +5511,7 @@
       </c>
       <c r="C87" s="8" t="inlineStr">
         <is>
-          <t>Harç ve Çimento Olmadan Depremde Yıkılmayan 500 Yıllık İnka Duvarları! 🏛️🪨 #bilgidozu #shorts</t>
+          <t>Harç ve Çimento Olmadan Depremde Yıkılmayan 500 Yıllık İnka Duvarları! 🏛️ #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D87" s="8" t="inlineStr">
@@ -5621,7 +5621,7 @@
       </c>
       <c r="C89" s="8" t="inlineStr">
         <is>
-          <t>Tükenmez Kalem Kapağındaki O Küçük Delik Neden Hayat Kurtarır? 🖊️⚡ #bilgidozu #shorts</t>
+          <t>Tükenmez Kalem Kapağındaki O Küçük Delik Neden Hayat Kurtarır? 🖊️ #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D89" s="8" t="inlineStr">
@@ -5731,7 +5731,7 @@
       </c>
       <c r="C91" s="8" t="inlineStr">
         <is>
-          <t>2000 Yıllık Deniz Batığından Çıkan Dünyanın İlk Mekanik Bilgisayarı! ⚙️🏛️ #bilgidozu #shorts</t>
+          <t>2000 Yıllık Deniz Batığından Çıkan Dünyanın İlk Mekanik Bilgisayarı! ⚙️ #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D91" s="8" t="inlineStr">
@@ -5786,7 +5786,7 @@
       </c>
       <c r="C92" s="8" t="inlineStr">
         <is>
-          <t>70 Derece Çölde Yuvasını Adımlarını Sayarak Bulan Gümüş Karınca! 🐜☀️ #bilgidozu #shorts</t>
+          <t>70 Derece Çölde Yuvasını Adımlarını Sayarak Bulan Gümüş Karınca! 🐜 #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D92" s="8" t="inlineStr">
@@ -5896,7 +5896,7 @@
       </c>
       <c r="C94" s="8" t="inlineStr">
         <is>
-          <t>Satürn'ün Kuzey Kutbundaki Dev Altıgen Fırtınanın Sırrı! 🪐🌪️ #bilgidozu #shorts</t>
+          <t>Satürn'ün Kuzey Kutbundaki Dev Altıgen Fırtınanın Sırrı! 🪐 #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D94" s="8" t="inlineStr">
@@ -5951,7 +5951,7 @@
       </c>
       <c r="C95" s="8" t="inlineStr">
         <is>
-          <t>Efsanevi Şam Çeliği Kılıçların İçinden Karbon Nanotüp Çıktı! ⚔️🔬 #bilgidozu #shorts</t>
+          <t>Efsanevi Şam Çeliği Kılıçların İçinden Karbon Nanotüp Çıktı! ⚔️ #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D95" s="8" t="inlineStr">
@@ -6116,7 +6116,7 @@
       </c>
       <c r="C98" s="8" t="inlineStr">
         <is>
-          <t>Uzayda Ses Yayılsaydı Güneş Dünya'dan 100 Desibel Tren Gibi Gürlerdi! ☀️🔊 #bilgidozu #shorts</t>
+          <t>Uzayda Ses Yayılsaydı Güneş Dünya'dan 100 Desibel Tren Gibi Gürlerdi! ☀️ #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D98" s="8" t="inlineStr">
@@ -6171,7 +6171,7 @@
       </c>
       <c r="C99" s="8" t="inlineStr">
         <is>
-          <t>Paskalya Adası'ndaki 80 Tonluk Dev Taş Heykeller Nasıl Yürütüldü? 🗿🏛️ #bilgidozu #shorts</t>
+          <t>Paskalya Adası'ndaki 80 Tonluk Dev Taş Heykeller Nasıl Yürütüldü? 🗿 #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D99" s="8" t="inlineStr">
@@ -6281,7 +6281,7 @@
       </c>
       <c r="C101" s="8" t="inlineStr">
         <is>
-          <t>Yürüyen Merdiven Kenarındaki Fırçalar Ayakkabı Silmek İçin Değil! 👟⚠️ #bilgidozu #shorts</t>
+          <t>Yürüyen Merdiven Kenarındaki Fırçalar Ayakkabı Silmek İçin Değil! 👟 #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D101" s="8" t="inlineStr">
@@ -6501,7 +6501,7 @@
       </c>
       <c r="C105" s="8" t="inlineStr">
         <is>
-          <t>Yıldırım Yukarıdan Düşmez: Parlama Yerden Gökyüzüne Çıkar! ⚡🌩️ #bilgidozu #shorts</t>
+          <t>Yıldırım Yukarıdan Düşmez: Parlama Yerden Gökyüzüne Çıkar! ⚡ #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D105" s="8" t="inlineStr">
@@ -6776,7 +6776,7 @@
       </c>
       <c r="C110" s="8" t="inlineStr">
         <is>
-          <t>Güneş Bir Saniyeliğine Sönseydi Ne Olurdu? ☀️🌑 #bilgidozu #shorts</t>
+          <t>Güneş Bir Saniyeliğine Sönseydi Ne Olurdu? ☀️ #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D110" s="8" t="inlineStr">
@@ -6886,7 +6886,7 @@
       </c>
       <c r="C112" s="8" t="inlineStr">
         <is>
-          <t>Uzayda Ağlarsan Gözyaşların Neden Yanağından Akmaz? 🧑‍🚀💧 #bilgidozu #shorts</t>
+          <t>Uzayda Ağlarsan Gözyaşların Neden Yanağından Akmaz? 🧑 #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D112" s="8" t="inlineStr">
@@ -7051,7 +7051,7 @@
       </c>
       <c r="C115" s="8" t="inlineStr">
         <is>
-          <t>Dünya'nın En Issız Noktası Point Nemo: En Yakın İnsanlar Uzayda! 🌊🛰️ #bilgidozu #shorts</t>
+          <t>Dünya'nın En Issız Noktası Point Nemo: En Yakın İnsanlar Uzayda! 🌊 #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D115" s="8" t="inlineStr">
@@ -7161,7 +7161,7 @@
       </c>
       <c r="C117" s="8" t="inlineStr">
         <is>
-          <t>5,5 Milyon Yıldır Güneş Görmeyen Mühürlü Mağara: Movile! 🕳️🕷️ #bilgidozu #shorts</t>
+          <t>5,5 Milyon Yıldır Güneş Görmeyen Mühürlü Mağara: Movile! 🕳️ #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D117" s="8" t="inlineStr">
@@ -7271,7 +7271,7 @@
       </c>
       <c r="C119" s="8" t="inlineStr">
         <is>
-          <t>Yerin 2.224 Metre Altında Ne Var? Dünya'nın En Derin Mağarası! 🧗‍♂️🌑 #bilgidozu #shorts</t>
+          <t>Yerin 2.224 Metre Altında Ne Var? Dünya'nın En Derin Mağarası! 🧗 #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D119" s="8" t="inlineStr">
@@ -7326,7 +7326,7 @@
       </c>
       <c r="C120" s="8" t="inlineStr">
         <is>
-          <t>2.100 Yıllık Batıktan Çıkan İlk Analog Bilgisayar: Antikythera! ⚙️🏛️ #bilgidozu #shorts</t>
+          <t>2.100 Yıllık Batıktan Çıkan İlk Analog Bilgisayar: Antikythera! ⚙️ #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D120" s="8" t="inlineStr">
@@ -7381,7 +7381,7 @@
       </c>
       <c r="C121" s="8" t="inlineStr">
         <is>
-          <t>Derinkuyu Yeraltı Şehri: 20 Bin Kişi Yerin Altında Nasıl Nefes Aldı? 🏺🕯️ #bilgidozu #shorts</t>
+          <t>Derinkuyu Yeraltı Şehri: 20 Bin Kişi Yerin Altında Nasıl Nefes Aldı? 🏺 #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D121" s="8" t="inlineStr">
@@ -7546,7 +7546,7 @@
       </c>
       <c r="C124" s="8" t="inlineStr">
         <is>
-          <t>Babil'in Asma Bahçeleri Gerçekte Babil'de Değil Miydi? 🌿🏛️ #bilgidozu #shorts</t>
+          <t>Babil'in Asma Bahçeleri Gerçekte Babil'de Değil Miydi? 🌿 #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D124" s="8" t="inlineStr">
@@ -7886,7 +7886,7 @@
       </c>
       <c r="C129" s="11" t="inlineStr">
         <is>
-          <t>Güneşe Dönünce Hapşırıyor musun? Bu Bir Refleks: ACHOO! ☀️🤧 #bilgidozu #shorts</t>
+          <t>Güneşe Dönünce Hapşırıyor musun? Bu Bir Refleks: ACHOO! ☀️ #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D129" s="11" t="inlineStr">

</xml_diff>

<commit_message>
EMIR 025c: havuz 34 baslikta cift emoji -> tek (len bug fix sonrasi kalanlar)
</commit_message>
<xml_diff>
--- a/bilgidozu_yukleme_tablosu.xlsx
+++ b/bilgidozu_yukleme_tablosu.xlsx
@@ -3432,7 +3432,7 @@
       </c>
       <c r="C49" s="8" t="inlineStr">
         <is>
-          <t>Mide Asidi Bu Kadar Güçlüyken Miden Kendi Kendini Neden Sindirmez? 🧬🔥 #bilgidozu #shorts</t>
+          <t>Mide Asidi Bu Kadar Güçlüyken Miden Kendi Kendini Neden Sindirmez? 🧬 #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D49" s="8" t="inlineStr">
@@ -3643,7 +3643,7 @@
       </c>
       <c r="C53" s="8" t="inlineStr">
         <is>
-          <t>İnsan Vücudu Karanlıkta Gerçekten Işık Saçıyor Ama Gözümüz Göremiyor! ✨🧠 #bilgidozu #shorts</t>
+          <t>İnsan Vücudu Karanlıkta Gerçekten Işık Saçıyor Ama Gözümüz Göremiyor! ✨ #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D53" s="8" t="inlineStr">
@@ -3973,7 +3973,7 @@
       </c>
       <c r="C59" s="8" t="inlineStr">
         <is>
-          <t>Soğukta Dişlerin Neden İrade Dışı Takırdar? 🥶🦷 #bilgidozu #shorts</t>
+          <t>Soğukta Dişlerin Neden İrade Dışı Takırdar? 🥶 #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D59" s="8" t="inlineStr">
@@ -4028,7 +4028,7 @@
       </c>
       <c r="C60" s="8" t="inlineStr">
         <is>
-          <t>Utandığında Neden Sadece Yüzün ve Kulakların Kızarır? 😳🧠 #bilgidozu #shorts</t>
+          <t>Utandığında Neden Sadece Yüzün ve Kulakların Kızarır? 😳 #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D60" s="8" t="inlineStr">
@@ -4083,7 +4083,7 @@
       </c>
       <c r="C61" s="8" t="inlineStr">
         <is>
-          <t>Vücudundaki Hücrelerin Yarısından Fazlası Aslında Bakteri! 🦠🧬 #bilgidozu #shorts</t>
+          <t>Vücudundaki Hücrelerin Yarısından Fazlası Aslında Bakteri! 🦠 #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D61" s="8" t="inlineStr">
@@ -4932,7 +4932,7 @@
       </c>
       <c r="C76" s="8" t="inlineStr">
         <is>
-          <t>Bu Hayvanın Parmak İzi İnsanla O Kadar Aynı ki Mikroskopta Bile Karışıyor! 🐨🔍 #bilgidozu #shorts</t>
+          <t>Bu Hayvanın Parmak İzi İnsanla O Kadar Aynı ki Mikroskopta Bile Karışıyor! 🐨 #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D76" s="8" t="inlineStr">
@@ -4984,7 +4984,7 @@
       </c>
       <c r="C77" s="8" t="inlineStr">
         <is>
-          <t>Mikrodalga Fırın Yemeği İçeriden Dışarıya Doğru Pişirmez! İşte Gerçek! ⚡🔬 #bilgidozu #shorts</t>
+          <t>Mikrodalga Fırın Yemeği İçeriden Dışarıya Doğru Pişirmez! İşte Gerçek! ⚡ #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D77" s="8" t="inlineStr">
@@ -5140,7 +5140,7 @@
       </c>
       <c r="C80" s="8" t="inlineStr">
         <is>
-          <t>Koltuk Altındaki Gizli Cebinde Kendi Çekiç Taşını Taşıyan Hayvan! 🦦🪨 #bilgidozu #shorts</t>
+          <t>Koltuk Altındaki Gizli Cebinde Kendi Çekiç Taşını Taşıyan Hayvan! 🦦 #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D80" s="8" t="inlineStr">
@@ -5248,7 +5248,7 @@
       </c>
       <c r="C82" s="8" t="inlineStr">
         <is>
-          <t>Bir Kibrit Kutusu Kadar Parçası 3 Milyar Ton Çeken Yıldız! 🪐⚡ #bilgidozu #shorts</t>
+          <t>Bir Kibrit Kutusu Kadar Parçası 3 Milyar Ton Çeken Yıldız! 🪐 #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D82" s="8" t="inlineStr">
@@ -5300,7 +5300,7 @@
       </c>
       <c r="C83" s="8" t="inlineStr">
         <is>
-          <t>Vezüv Patlamasında Beyni Gerçek Siyah Cama Dönüşen Romalı! 🌋🖤 #bilgidozu #shorts</t>
+          <t>Vezüv Patlamasında Beyni Gerçek Siyah Cama Dönüşen Romalı! 🌋 #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D83" s="8" t="inlineStr">
@@ -5352,7 +5352,7 @@
       </c>
       <c r="C84" s="8" t="inlineStr">
         <is>
-          <t>Bu Hayvan Su Altında Nefesini Yunuslardan 4 Kat Uzun Tutuyor! 🦥🌊 #bilgidozu #shorts</t>
+          <t>Bu Hayvan Su Altında Nefesini Yunuslardan 4 Kat Uzun Tutuyor! 🦥 #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D84" s="8" t="inlineStr">
@@ -5404,7 +5404,7 @@
       </c>
       <c r="C85" s="8" t="inlineStr">
         <is>
-          <t>Araba Ön Camlarındaki Siyah Noktalar Neden Var? Süs Değilmiş! 🚗⚫ #bilgidozu #shorts</t>
+          <t>Araba Ön Camlarındaki Siyah Noktalar Neden Var? Süs Değilmiş! 🚗 #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D85" s="8" t="inlineStr">
@@ -5456,7 +5456,7 @@
       </c>
       <c r="C86" s="8" t="inlineStr">
         <is>
-          <t>Tepesinden Atlayınca Dibe Düşmenin 12 Dakika Sürdüğü 20 Km'lik Uçurum! 🪐🧗 #bilgidozu #shorts</t>
+          <t>Tepesinden Atlayınca Dibe Düşmenin 12 Dakika Sürdüğü 20 Km'lik Uçurum! 🪐 #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D86" s="8" t="inlineStr">
@@ -5566,7 +5566,7 @@
       </c>
       <c r="C88" s="8" t="inlineStr">
         <is>
-          <t>Baykuşlar Karanlıkta Uçarken Nasıl Sıfır Ses Çıkarır? Hayalet Kanat Sırrı! 🦉🌙 #bilgidozu #shorts</t>
+          <t>Baykuşlar Karanlıkta Uçarken Nasıl Sıfır Ses Çıkarır? Hayalet Kanat Sırrı! 🦉 #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D88" s="8" t="inlineStr">
@@ -5676,7 +5676,7 @@
       </c>
       <c r="C90" s="8" t="inlineStr">
         <is>
-          <t>Su Değil Sert Kaya Zemini Her Gün 100 Metre Yükselip Alçalan Uydu! 🪐🌋 #bilgidozu #shorts</t>
+          <t>Su Değil Sert Kaya Zemini Her Gün 100 Metre Yükselip Alçalan Uydu! 🪐 #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D90" s="8" t="inlineStr">
@@ -5841,7 +5841,7 @@
       </c>
       <c r="C93" s="8" t="inlineStr">
         <is>
-          <t>Benzin Pompası Depo Dolunca Çipsiz ve Sensörsüz Nasıl Kendi Durur? ⛽⚡ #bilgidozu #shorts</t>
+          <t>Benzin Pompası Depo Dolunca Çipsiz ve Sensörsüz Nasıl Kendi Durur? ⛽ #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D93" s="8" t="inlineStr">
@@ -6006,7 +6006,7 @@
       </c>
       <c r="C96" s="8" t="inlineStr">
         <is>
-          <t>Işığın Kırılmasını Hesaplayıp Böceği Suyla Vuran Keskin Nişancı Balık! 🐟🎯 #bilgidozu #shorts</t>
+          <t>Işığın Kırılmasını Hesaplayıp Böceği Suyla Vuran Keskin Nişancı Balık! 🐟 #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D96" s="8" t="inlineStr">
@@ -6061,7 +6061,7 @@
       </c>
       <c r="C97" s="8" t="inlineStr">
         <is>
-          <t>Mikrodalga Fırın Camındaki Delikli Siyah Tel Neden Var? ⚡🪟 #bilgidozu #shorts</t>
+          <t>Mikrodalga Fırın Camındaki Delikli Siyah Tel Neden Var? ⚡ #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D97" s="8" t="inlineStr">
@@ -6226,7 +6226,7 @@
       </c>
       <c r="C100" s="8" t="inlineStr">
         <is>
-          <t>Elektrikli Yılan Balığı 860 Volt Elektrik Üretirken Kendini Neden Çarpmaz? ⚡🐍 #bilgidozu #shorts</t>
+          <t>Elektrikli Yılan Balığı 860 Volt Elektrik Üretirken Kendini Neden Çarpmaz? ⚡ #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D100" s="8" t="inlineStr">
@@ -6336,7 +6336,7 @@
       </c>
       <c r="C102" s="8" t="inlineStr">
         <is>
-          <t>Neptün ve Uranüs'te Gökyüzünden Gerçek Elmas Yağıyor! 💎🪐 #bilgidozu #shorts</t>
+          <t>Neptün ve Uranüs'te Gökyüzünden Gerçek Elmas Yağıyor! 💎 #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D102" s="8" t="inlineStr">
@@ -6391,7 +6391,7 @@
       </c>
       <c r="C103" s="8" t="inlineStr">
         <is>
-          <t>Uzay Boşluğunda Bile Hayatta Kalan Canlı: Su Ayısı Tardigrad! 🐻🌌 #bilgidozu #shorts</t>
+          <t>Uzay Boşluğunda Bile Hayatta Kalan Canlı: Su Ayısı Tardigrad! 🐻 #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D103" s="8" t="inlineStr">
@@ -6446,7 +6446,7 @@
       </c>
       <c r="C104" s="8" t="inlineStr">
         <is>
-          <t>Tek Bir Ağaçtan Oluşan 47 Bin Gövdeli Dev Orman: Pando! 🌲🌍 #bilgidozu #shorts</t>
+          <t>Tek Bir Ağaçtan Oluşan 47 Bin Gövdeli Dev Orman: Pando! 🌲 #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D104" s="8" t="inlineStr">
@@ -6556,7 +6556,7 @@
       </c>
       <c r="C106" s="8" t="inlineStr">
         <is>
-          <t>Cam Zamanla Akan Bir Sıvı Değil: En Büyük Bilim Efsanesi! 🪟🔬 #bilgidozu #shorts</t>
+          <t>Cam Zamanla Akan Bir Sıvı Değil: En Büyük Bilim Efsanesi! 🪟 #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D106" s="8" t="inlineStr">
@@ -6611,7 +6611,7 @@
       </c>
       <c r="C107" s="8" t="inlineStr">
         <is>
-          <t>Ay Her Yıl Dünya'dan 3,8 Santimetre Uzaklaşıyor! 🌕🚀 #bilgidozu #shorts</t>
+          <t>Ay Her Yıl Dünya'dan 3,8 Santimetre Uzaklaşıyor! 🌕 #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D107" s="8" t="inlineStr">
@@ -6666,7 +6666,7 @@
       </c>
       <c r="C108" s="8" t="inlineStr">
         <is>
-          <t>Yetişkin Kediler Birbirine Değil Sadece İnsanlara Miyavlar! 🐱🔊 #bilgidozu #shorts</t>
+          <t>Yetişkin Kediler Birbirine Değil Sadece İnsanlara Miyavlar! 🐱 #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D108" s="8" t="inlineStr">
@@ -6721,7 +6721,7 @@
       </c>
       <c r="C109" s="8" t="inlineStr">
         <is>
-          <t>Dünya Uzayda Saniyede 30 Kilometre Hızla Uçuyor! 🌍⚡ #bilgidozu #shorts</t>
+          <t>Dünya Uzayda Saniyede 30 Kilometre Hızla Uçuyor! 🌍 #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D109" s="8" t="inlineStr">
@@ -6831,7 +6831,7 @@
       </c>
       <c r="C111" s="8" t="inlineStr">
         <is>
-          <t>Ay Dünya'ya Yaklaşsaydı Okyanuslara Ne Olurdu? 🌕🌊 #bilgidozu #shorts</t>
+          <t>Ay Dünya'ya Yaklaşsaydı Okyanuslara Ne Olurdu? 🌕 #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D111" s="8" t="inlineStr">
@@ -6941,7 +6941,7 @@
       </c>
       <c r="C113" s="8" t="inlineStr">
         <is>
-          <t>Dünya'ya 50 Işık Yılı Mesafede Süpernova Patlasa Ne Olur? 💥🌟 #bilgidozu #shorts</t>
+          <t>Dünya'ya 50 Işık Yılı Mesafede Süpernova Patlasa Ne Olur? 💥 #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D113" s="8" t="inlineStr">
@@ -6996,7 +6996,7 @@
       </c>
       <c r="C114" s="8" t="inlineStr">
         <is>
-          <t>Bir Çay Kaşığı Nötron Yıldızı Dünya'ya Düşse Ne Olur? 🥄🌌 #bilgidozu #shorts</t>
+          <t>Bir Çay Kaşığı Nötron Yıldızı Dünya'ya Düşse Ne Olur? 🥄 #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D114" s="8" t="inlineStr">
@@ -7106,7 +7106,7 @@
       </c>
       <c r="C116" s="8" t="inlineStr">
         <is>
-          <t>Antarktika'daki Buzuldan Neden Kan Kırmızısı Şelale Akıyor? 🧊🩸 #bilgidozu #shorts</t>
+          <t>Antarktika'daki Buzuldan Neden Kan Kırmızısı Şelale Akıyor? 🧊 #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D116" s="8" t="inlineStr">
@@ -7216,7 +7216,7 @@
       </c>
       <c r="C118" s="8" t="inlineStr">
         <is>
-          <t>Dallol Volkanı: Dünya Üzerindeki En Asidik ve Renkli Cehennem! 🌋🧪 #bilgidozu #shorts</t>
+          <t>Dallol Volkanı: Dünya Üzerindeki En Asidik ve Renkli Cehennem! 🌋 #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D118" s="8" t="inlineStr">
@@ -7436,7 +7436,7 @@
       </c>
       <c r="C122" s="8" t="inlineStr">
         <is>
-          <t>Voynich El Yazması: 600 Yıldır Kimsenin Okuyamadığı Şifreli Kitap! 📜🔍 #bilgidozu #shorts</t>
+          <t>Voynich El Yazması: 600 Yıldır Kimsenin Okuyamadığı Şifreli Kitap! 📜 #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D122" s="8" t="inlineStr">
@@ -7491,7 +7491,7 @@
       </c>
       <c r="C123" s="8" t="inlineStr">
         <is>
-          <t>Puma Punku H-Blokları: Jilet Bile Girmeyen Antik Taşların Sırrı! 🪨📐 #bilgidozu #shorts</t>
+          <t>Puma Punku H-Blokları: Jilet Bile Girmeyen Antik Taşların Sırrı! 🪨 #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D123" s="8" t="inlineStr">
@@ -7951,7 +7951,7 @@
       </c>
       <c r="C130" s="11" t="inlineStr">
         <is>
-          <t>Dondurma Damağına Değer Ama Neden Alnın Sızlar? 🧊🧠 #bilgidozu #shorts</t>
+          <t>Dondurma Damağına Değer Ama Neden Alnın Sızlar? 🧊 #bilgidozu #shorts</t>
         </is>
       </c>
       <c r="D130" s="11" t="inlineStr">

</xml_diff>

<commit_message>
EMİR: havuz 51+ — 47/49/50 arşive (ESKİ_STOK_ASKIDA); MIN_SHORTS_NUMBER 47→51
</commit_message>
<xml_diff>
--- a/bilgidozu_yukleme_tablosu.xlsx
+++ b/bilgidozu_yukleme_tablosu.xlsx
@@ -3422,7 +3422,7 @@
     <row r="49" ht="42" customHeight="1">
       <c r="A49" s="7" t="inlineStr">
         <is>
-          <t>BEKLEMEDE</t>
+          <t>ESKİ_STOK_ASKIDA</t>
         </is>
       </c>
       <c r="B49" s="7" t="inlineStr">
@@ -4922,7 +4922,7 @@
     <row r="76" ht="42" customHeight="1">
       <c r="A76" s="7" t="inlineStr">
         <is>
-          <t>BEKLEMEDE</t>
+          <t>ESKİ_STOK_ASKIDA</t>
         </is>
       </c>
       <c r="B76" s="7" t="inlineStr">
@@ -4974,7 +4974,7 @@
     <row r="77" ht="42" customHeight="1">
       <c r="A77" s="7" t="inlineStr">
         <is>
-          <t>BEKLEMEDE</t>
+          <t>ESKİ_STOK_ASKIDA</t>
         </is>
       </c>
       <c r="B77" s="7" t="inlineStr">

</xml_diff>

<commit_message>
docs: HANDOVER (yeni agent icin islemsiz brifing) + 4 kanaldan silinmis video SİLİNDİ isaretlendi (17/18/20/21)
</commit_message>
<xml_diff>
--- a/bilgidozu_yukleme_tablosu.xlsx
+++ b/bilgidozu_yukleme_tablosu.xlsx
@@ -1840,7 +1840,7 @@
     <row r="21" ht="42" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>YÜKLENDİ</t>
+          <t>SİLİNDİ</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -1899,7 +1899,7 @@
     <row r="22" ht="42" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>YÜKLENDİ</t>
+          <t>SİLİNDİ</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -2013,7 +2013,7 @@
     <row r="24" ht="42" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>YÜKLENDİ</t>
+          <t>SİLİNDİ</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -2076,7 +2076,7 @@
     <row r="25" ht="42" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>YÜKLENDİ</t>
+          <t>SİLİNDİ</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore: goruntülenme raporu (yt-dlp, 0 kota)
</commit_message>
<xml_diff>
--- a/bilgidozu_yukleme_tablosu.xlsx
+++ b/bilgidozu_yukleme_tablosu.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DRIVE" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ISCILER" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UYARILAR" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="DRIVE" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="ISCILER" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="UYARILAR" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -666,7 +666,7 @@
         </is>
       </c>
       <c r="L2" s="3" t="n">
-        <v>1233</v>
+        <v>1200</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>0</v>
@@ -730,7 +730,7 @@
         </is>
       </c>
       <c r="L3" s="3" t="n">
-        <v>1140</v>
+        <v>1100</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>1</v>
@@ -794,7 +794,7 @@
         </is>
       </c>
       <c r="L4" s="3" t="n">
-        <v>1006</v>
+        <v>1000</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>2</v>
@@ -858,7 +858,7 @@
         </is>
       </c>
       <c r="L5" s="3" t="n">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>1</v>
@@ -922,7 +922,7 @@
         </is>
       </c>
       <c r="L6" s="3" t="n">
-        <v>519</v>
+        <v>525</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>3</v>
@@ -986,7 +986,7 @@
         </is>
       </c>
       <c r="L7" s="3" t="n">
-        <v>964</v>
+        <v>972</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>1</v>
@@ -1050,7 +1050,7 @@
         </is>
       </c>
       <c r="L8" s="3" t="n">
-        <v>947</v>
+        <v>949</v>
       </c>
       <c r="M8" s="3" t="n">
         <v>1</v>
@@ -1114,7 +1114,7 @@
         </is>
       </c>
       <c r="L9" s="3" t="n">
-        <v>1086</v>
+        <v>1100</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>1</v>
@@ -1178,7 +1178,7 @@
         </is>
       </c>
       <c r="L10" s="3" t="n">
-        <v>1023</v>
+        <v>1000</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>1</v>
@@ -1242,7 +1242,7 @@
         </is>
       </c>
       <c r="L11" s="3" t="n">
-        <v>509</v>
+        <v>520</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>1</v>
@@ -1306,7 +1306,7 @@
         </is>
       </c>
       <c r="L12" s="3" t="n">
-        <v>975</v>
+        <v>986</v>
       </c>
       <c r="M12" s="3" t="n">
         <v>1</v>
@@ -1370,7 +1370,7 @@
         </is>
       </c>
       <c r="L13" s="3" t="n">
-        <v>1288</v>
+        <v>1300</v>
       </c>
       <c r="M13" s="3" t="n">
         <v>1</v>
@@ -1434,7 +1434,7 @@
         </is>
       </c>
       <c r="L14" s="3" t="n">
-        <v>1014</v>
+        <v>1000</v>
       </c>
       <c r="M14" s="3" t="n">
         <v>1</v>
@@ -1498,7 +1498,7 @@
         </is>
       </c>
       <c r="L15" s="3" t="n">
-        <v>1111</v>
+        <v>1100</v>
       </c>
       <c r="M15" s="3" t="n">
         <v>1</v>
@@ -1562,7 +1562,7 @@
         </is>
       </c>
       <c r="L16" s="3" t="n">
-        <v>1007</v>
+        <v>1000</v>
       </c>
       <c r="M16" s="3" t="n">
         <v>1</v>
@@ -1632,7 +1632,7 @@
         </is>
       </c>
       <c r="L17" s="3" t="n">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="M17" s="3" t="n">
         <v>1</v>
@@ -1702,7 +1702,7 @@
         </is>
       </c>
       <c r="L18" s="3" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="M18" s="3" t="n">
         <v>0</v>
@@ -1771,7 +1771,9 @@
           <t>2026-10-25 18:20</t>
         </is>
       </c>
-      <c r="L19" s="3" t="n"/>
+      <c r="L19" s="3" t="n">
+        <v>70</v>
+      </c>
       <c r="M19" s="3" t="n"/>
     </row>
     <row r="20" ht="42" customHeight="1">
@@ -1831,7 +1833,7 @@
         </is>
       </c>
       <c r="L20" s="3" t="n">
-        <v>962</v>
+        <v>1000</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>3</v>
@@ -2809,7 +2811,7 @@
         </is>
       </c>
       <c r="L38" s="3" t="n">
-        <v>208</v>
+        <v>454</v>
       </c>
       <c r="M38" s="3" t="n">
         <v>1</v>
@@ -2873,7 +2875,7 @@
         </is>
       </c>
       <c r="L39" s="3" t="n">
-        <v>338</v>
+        <v>962</v>
       </c>
       <c r="M39" s="3" t="n">
         <v>1</v>
@@ -2936,7 +2938,9 @@
           <t>2026-10-23 18:24</t>
         </is>
       </c>
-      <c r="L40" s="3" t="n"/>
+      <c r="L40" s="3" t="n">
+        <v>80</v>
+      </c>
       <c r="M40" s="3" t="n"/>
     </row>
     <row r="41" ht="42" customHeight="1">
@@ -2996,7 +3000,9 @@
           <t>2026-10-24 11:24</t>
         </is>
       </c>
-      <c r="L41" s="3" t="n"/>
+      <c r="L41" s="3" t="n">
+        <v>111</v>
+      </c>
       <c r="M41" s="3" t="n"/>
     </row>
     <row r="42" ht="42" customHeight="1">
@@ -3056,7 +3062,9 @@
           <t>2026-10-24 15:22</t>
         </is>
       </c>
-      <c r="L42" s="3" t="n"/>
+      <c r="L42" s="3" t="n">
+        <v>187</v>
+      </c>
       <c r="M42" s="3" t="n"/>
     </row>
     <row r="43" ht="42" customHeight="1">
@@ -3116,7 +3124,9 @@
           <t>2026-10-24 18:18</t>
         </is>
       </c>
-      <c r="L43" s="3" t="n"/>
+      <c r="L43" s="3" t="n">
+        <v>104</v>
+      </c>
       <c r="M43" s="3" t="n"/>
     </row>
     <row r="44" ht="42" customHeight="1">
@@ -3176,7 +3186,9 @@
           <t>2026-10-24 20:18</t>
         </is>
       </c>
-      <c r="L44" s="3" t="n"/>
+      <c r="L44" s="3" t="n">
+        <v>313</v>
+      </c>
       <c r="M44" s="3" t="n"/>
     </row>
     <row r="45" ht="42" customHeight="1">
@@ -3236,7 +3248,9 @@
           <t>2026-10-24 20:23</t>
         </is>
       </c>
-      <c r="L45" s="3" t="n"/>
+      <c r="L45" s="3" t="n">
+        <v>146</v>
+      </c>
       <c r="M45" s="3" t="n"/>
     </row>
     <row r="46" ht="42" customHeight="1">
@@ -3296,7 +3310,9 @@
           <t>2026-10-25 11:24</t>
         </is>
       </c>
-      <c r="L46" s="3" t="n"/>
+      <c r="L46" s="3" t="n">
+        <v>147</v>
+      </c>
       <c r="M46" s="3" t="n"/>
     </row>
     <row r="47" ht="42" customHeight="1">
@@ -3356,7 +3372,9 @@
           <t>2026-10-25 15:22</t>
         </is>
       </c>
-      <c r="L47" s="3" t="n"/>
+      <c r="L47" s="3" t="n">
+        <v>103</v>
+      </c>
       <c r="M47" s="3" t="n"/>
     </row>
     <row r="48" ht="42" customHeight="1">
@@ -3416,7 +3434,9 @@
           <t>2026-10-25 15:29</t>
         </is>
       </c>
-      <c r="L48" s="3" t="n"/>
+      <c r="L48" s="3" t="n">
+        <v>42</v>
+      </c>
       <c r="M48" s="3" t="n"/>
     </row>
     <row r="49" ht="42" customHeight="1">
@@ -4656,7 +4676,9 @@
           <t>2026-10-26 11:39</t>
         </is>
       </c>
-      <c r="L70" s="3" t="n"/>
+      <c r="L70" s="3" t="n">
+        <v>649</v>
+      </c>
       <c r="M70" s="3" t="n"/>
     </row>
     <row r="71" ht="42" customHeight="1">
@@ -7648,7 +7670,9 @@
           <t>2026-10-26 19:36</t>
         </is>
       </c>
-      <c r="L125" s="3" t="n"/>
+      <c r="L125" s="3" t="n">
+        <v>731</v>
+      </c>
       <c r="M125" s="3" t="n"/>
     </row>
     <row r="126" ht="42" customHeight="1">
@@ -7723,7 +7747,9 @@
           <t>2026-10-27 10:48</t>
         </is>
       </c>
-      <c r="L126" s="3" t="n"/>
+      <c r="L126" s="3" t="n">
+        <v>649</v>
+      </c>
       <c r="M126" s="3" t="n"/>
     </row>
     <row r="127" ht="42" customHeight="1">
@@ -7797,7 +7823,9 @@
           <t>2026-10-27 19:34</t>
         </is>
       </c>
-      <c r="L127" s="3" t="n"/>
+      <c r="L127" s="3" t="n">
+        <v>204</v>
+      </c>
       <c r="M127" s="3" t="n"/>
     </row>
     <row r="128" ht="42" customHeight="1">
@@ -7870,7 +7898,9 @@
           <t>2026-10-27 23:09</t>
         </is>
       </c>
-      <c r="L128" s="3" t="n"/>
+      <c r="L128" s="3" t="n">
+        <v>52</v>
+      </c>
       <c r="M128" s="3" t="n"/>
     </row>
     <row r="129" ht="42" customHeight="1">

</xml_diff>

<commit_message>
feat(stok): Cloud'un ilk videosu havuza girdi (suda parmak buruşması) + video_62 ikiz oldugu icin askiya alindi
</commit_message>
<xml_diff>
--- a/bilgidozu_yukleme_tablosu.xlsx
+++ b/bilgidozu_yukleme_tablosu.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="DRIVE" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="ISCILER" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="UYARILAR" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DRIVE" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ISCILER" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UYARILAR" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -524,7 +524,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M130"/>
+  <dimension ref="A1:M131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3598,7 +3598,7 @@
     <row r="52" ht="42" customHeight="1">
       <c r="A52" s="7" t="inlineStr">
         <is>
-          <t>BEKLEMEDE</t>
+          <t>ESKİ_STOK_ASKIDA</t>
         </is>
       </c>
       <c r="B52" s="7" t="inlineStr">
@@ -8034,7 +8034,54 @@
       <c r="L130" s="11" t="n"/>
       <c r="M130" s="11" t="n"/>
     </row>
-    <row r="131" ht="42" customHeight="1"/>
+    <row r="131" ht="42" customHeight="1">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>BEKLEMEDE</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>bilgi_dozu_suda_parmaklar_neden_burusur_shorts.mp4</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Suda Kalınca Parmak Uçların Neden Buruşur? Sebebi Su Değil! 🖐️ #bilgidozu #shorts</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Duşta, denizde ya da havuzda biraz fazla kaldığında parmak uçların neden buruşur? Çoğumuz derinin suyu sünger gibi emip şiştiğini sanırız; ancak gerçek bambaşka! Suya girdiğinde ter kanallarından sızan su ciltteki tuz dengesini düşürür ve otonom sinir sistemin kılcal damarları büzerek deriyi içeri doğru çeker. Üstelik oluşan bu "yağmur lastiği" kanalları ıslak nesneleri %12 daha hızlı kavramamızı sağlar ve her seferinde tıpkı parmak izi gibi aynı desende oluşur!
+Daha fazla bilgi dozu için takip etmeyi unutma!</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>#bilgidozu #shorts #insanvücudu #nörobilim #bilim</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>bilgidozu, shorts, buruşuk parmak, parmak uçları, biyoloji, insan vücudu, yağmur lastiği refleksi</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>Bunun su emilimi değil de beynin "yağmur lastiği" refleksi olduğunu daha önce duymuş muydun? 🖐️ Bilenler "1", ilk kez öğrenip şaşıranlar "2" yazsın! 👇</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>Biyoloji ve Vücut</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>Laytin &amp; German (2025) Binghamton University — J. Mech. Behavior of Biomedical Materials + Kareklas, Nettle &amp; Smulders (2013) Newcastle University — Biology Letters</t>
+        </is>
+      </c>
+    </row>
     <row r="132" ht="42" customHeight="1"/>
     <row r="133" ht="42" customHeight="1"/>
     <row r="134" ht="42" customHeight="1"/>

</xml_diff>

<commit_message>
feat(stok): 12 bedeni-serisi videosu stoğa alındı (video_139-147 + uzun_video_14-16 BEKLEMEDE) — Cloud batch'i stok kararıyla havuza
</commit_message>
<xml_diff>
--- a/bilgidozu_yukleme_tablosu.xlsx
+++ b/bilgidozu_yukleme_tablosu.xlsx
@@ -524,7 +524,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M131"/>
+  <dimension ref="A1:M143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -8082,9 +8082,748 @@
         </is>
       </c>
     </row>
-    <row r="132" ht="42" customHeight="1"/>
-    <row r="133" ht="42" customHeight="1"/>
-    <row r="134" ht="42" customHeight="1"/>
+    <row r="132" ht="42" customHeight="1">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>BEKLEMEDE</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>video_139.mp4</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Dirseğini Çarpınca Neden Elektrik Çarpmış Gibi Olur? ⚡ #bilgidozu #shorts</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>Dirseğini masanın köşesine çarptığında yüzük ve serçe parmağına kadar yayılan o elektrik şoku kemikten değil, zırhsız kalan ulnar sinirden kaynaklanır.
+📍 BÖLÜMLER
+00:00 Dirsek çarpınca yayılan elektrik hissi
+00:12 Kemik değil: büyük ulnar sinir hattı
+00:19 Kübital tünelde incecik deri altı geçiş
+00:28 Kemik ile sert yüzey arasında sıkışma
+00:36 Yüzük ve serçe parmakta karıncalanma
+00:43 Sıradaki bölüm: parmak çıtlatma sesi
+📊 Kaynaklar:
+• Johns Hopkins Medicine — Cubital Tunnel Syndrome &amp; Ulnar Nerve: https://www.hopkinsmedicine.org/health/conditions-and-diseases/cubital-tunnel-syndrome
+• Cleveland Clinic — Ulnar Nerve Entrapment: https://my.clevelandclinic.org/health/diseases/22272-ulnar-nerve-entrapment
+🩺 Uyarı: Genel bilimsel bilgi amaçlıdır, tıbbi tanı veya tavsiye değildir.
+🖼️ Görseller temsilîdir (bilimsel görselleştirme).
+Bir doz bilgi, her gün: 💊 ABONE OL!
+#bilgidozu #shorts #insanvücudu #ulnarsinir #bilim</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>#bilgidozu #shorts #insanvücudu #ulnarsinir #bilim</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>bilgidozu, shorts, dirsek çarpınca elektrik çarpması, ulnar sinir, kübital tünel, komik kemik, parmak uyuşması, sinir sistemi, insan vücudu, bilgi dozu</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>Dirseğini çarpıp bu elektrik şokunu yaşayanlar 1, hiç yaşamayanlar 2 yazsın! 👇</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>Biyoloji ve Vücut</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>Johns Hopkins Medicine &amp; Cleveland Clinic — Cubital Tunnel / Ulnar Nerve</t>
+        </is>
+      </c>
+    </row>
+    <row r="133" ht="42" customHeight="1">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>BEKLEMEDE</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>video_140.mp4</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Parmak Çıtlatınca Çıkan Ses Kemik Sesi Değilmiş! 🦴 #bilgidozu #shorts</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>Parmak çıtlattığında duyduğun o keskin ses kemiklerin sürtünmesi ya da baloncuk patlaması değil; eklem sıvısında milisaniyeler içinde oluşan vakum boşluğudur.
+📍 BÖLÜMLER
+00:00 Parmak çıtlatma sesi nereden gelir?
+00:11 Sinovyal sıvı ve vakum olayı
+00:21 Gerçek zamanlı MRI deneyi (Kawchuk 2015)
+00:30 Tribonükleasyon: 310 milisaniyede boşluk oluşumu
+00:39 Dr. Donald Unger'in 50 yıllık kireçlenme deneyi
+00:46 Sıradaki bölüm: ayak uyuşması ve karıncalanma
+📊 Kaynaklar:
+• Kawchuk GN et al. (2015) Real-Time MRI of Joint Cavitation, PLOS ONE: https://doi.org/10.1371/journal.pone.0119470
+• Unger DL (1998) Does Knuckle Cracking Lead to Arthritis of the Fingers?, Arthritis &amp; Rheumatism, 41(5): 949–950
+🩺 Uyarı: Genel bilimsel bilgi amaçlıdır, tıbbi tanı veya tavsiye değildir.
+🖼️ Görseller temsilîdir (bilimsel görselleştirme).
+Bir doz bilgi, her gün: 💊 ABONE OL!
+#bilgidozu #shorts #parmakçıtlatma #eklem #bilim</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>#bilgidozu #shorts #parmakçıtlatma #eklem #bilim</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>bilgidozu, shorts, parmak çıtlatmak, parmak çıtlatma sesi, kireçlenme yapar mı, sinovyal sıvı, tribonükleasyon, donald unger, insan vücudu, bilgi dozu</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>Gün içinde parmaklarını çıtlatanlar 1, o sese hiç dayanamayanlar 2 yazsın! 👇</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>Biyoloji ve Vücut</t>
+        </is>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>Kawchuk et al. (2015) PLOS ONE Real-Time MRI &amp; Unger (1998) Arthritis &amp; Rheumatism</t>
+        </is>
+      </c>
+    </row>
+    <row r="134" ht="42" customHeight="1">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>BEKLEMEDE</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>video_141.mp4</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Uyuşan Ayağın Açılırken Neden Binlerce İğne Batar? 🦶 #bilgidozu #shorts</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>Uzun süre bacak bacak üstüne attığında ayağının uyuşup kalkarken binlerce iğne batması kanın durmasından çok, çevresel sinir hatlarının yeniden uyanma fırtınasıdır.
+📍 BÖLÜMLER
+00:00 Ayak uyuşması ve iğnelenme neden olur?
+00:10 Damar mı yoksa çevresel sinir kabloları mı?
+00:18 Sinir lifleri ve kılcal damar basısı
+00:27 Geçici parestezi: uyanan sinirlerin sinyal fırtınası
+00:34 Beynin parazit sinyalleri karıncalanma okuması
+00:43 Sıradaki bölüm: tüylerin diken diken olması
+📊 Kaynaklar:
+• Cleveland Clinic — Paresthesia (Pins and Needles): https://my.clevelandclinic.org/health/symptoms/24932-paresthesia
+• NINDS / NIH — Peripheral Neuropathy &amp; Nerve Compression Overview
+🩺 Uyarı: Genel bilimsel bilgi amaçlıdır, tıbbi tanı veya tavsiye değildir.
+🖼️ Görseller temsilîdir (bilimsel görselleştirme).
+Bir doz bilgi, her gün: 💊 ABONE OL!
+#bilgidozu #shorts #ayakuyuşması #parestezi #sinirsistemi</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>#bilgidozu #shorts #ayakuyuşması #parestezi #sinirsistemi</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>bilgidozu, shorts, ayak uyuşması, bacak uyuşması, karıncalanma neden olur, parestezi, sinir sıkışması, iğne batması hissi, insan vücudu, bilgi dozu</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>Ayağı uyuşunca sekerek yürüyenler 1, kıpırdamadan geçmesini bekleyenler 2 yazsın! 👇</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>Beyin ve Psikoloji</t>
+        </is>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>Cleveland Clinic &amp; NINDS/NIH — Paresthesia &amp; Peripheral Nerve Compression</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>BEKLEMEDE</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>uzun_video_14.mp4</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Dirsek Elektriği, Parmak Çıtlatma ve Ayak Uyuşmasının Gerçek Bilimi 🧠 #bilgidozu</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>Vücudunda her gün yaşadığın ama gerçek mekanizmasını çoğu kişinin yanlış bildiği 3 büyüleyici sinir ve eklem olayını tek belgeselde inceliyoruz: dirsekteki kübital tünel elektrik şoku, parmak çıtlatmanın gerçek zamanlı MRI sırrı ve uyuşan bacakta kopan parestezi fırtınası.
+📍 BÖLÜMLER
+00:00 Giriş ve dirsekteki elektrik şoku
+00:28 Ulnar sinir ve kübital tünel zırhsızlığı
+00:52 Parmak çıtlatma sesi kemikten mi gelir?
+01:20 Tribonükleasyon vakumu ve 50 yıllık deney
+01:46 Ayak uyuşması: damar mı sinir mi?
+02:11 Sinir lifleri ve mikro damar basısı
+02:27 Geçici parestezi: karıncalanma fırtınası
+02:36 Özet: tek bir sinir ağı
+📊 Kaynaklar:
+• Johns Hopkins Medicine — Cubital Tunnel Syndrome: https://www.hopkinsmedicine.org/health/conditions-and-diseases/cubital-tunnel-syndrome
+• Kawchuk GN et al. (2015) PLOS ONE — Joint Cavitation MRI: https://doi.org/10.1371/journal.pone.0119470
+• Unger DL (1998) Arthritis &amp; Rheumatism 41(5): 949–950
+• Cleveland Clinic — Paresthesia: https://my.clevelandclinic.org/health/symptoms/24932-paresthesia
+🩺 Uyarı: Genel bilimsel bilgi amaçlıdır, tıbbi tanı veya tavsiye değildir.
+🖼️ Görseller temsilîdir (bilimsel görselleştirme).
+Bir doz bilgi, her gün: 💊 ABONE OL!
+#bilgidozu #insanvücudu #sinirsistemi #bilim #belgesel</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>#bilgidozu #insanvücudu #sinirsistemi #bilim #belgesel</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>bilgidozu, insan vücudu sırları, dirsek elektrik çarpması, ulnar sinir, parmak çıtlatma sesi, ayak uyuşması neden olur, parestezi, sinir sistemi belgeseli, bilim, bilgi dozu</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>Bu 3 sinir ve eklem olayından en sık hangisini yaşıyorsun? ⚡ 1-Dirsek şoku 2-Parmak çıtlatma 3-Ayak uyuşması — Numaranı yorumlara bırak! 👇</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>Uzun — Biyoloji ve Vücut</t>
+        </is>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>Johns Hopkins Medicine, Kawchuk et al. (2015) PLOS ONE &amp; Cleveland Clinic</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>BEKLEMEDE</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>video_142.mp4</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Üşüyünce ve Müzik Dinleyince Tüyler Neden Diken Diken Olur? 🧠 #bilgidozu #shorts</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>Üşüdüğünde ya da duygulandığında tüylerinin diken diken olması sadece atalarımızdan kalan bir yalıtım refleksi değil; Harvard araştırmacıları bu sinirlerin kıl kökü kök hücrelerini de uyardığını keşfetti!
+📍 BÖLÜMLER
+00:00 Üşüyünce ve ürperince kabaran deri
+00:11 Arrector pili: kıl köklerindeki mikroskobik kaslar
+00:19 Sempatik sinir sistemi ve kasılma emri
+00:28 Harvard 2020 keşfi: kök hücrelerle ikili hat
+00:36 Uzun süreli soğukta yeni tüy üretimi emri
+00:45 Sıradaki bölüm: hıçkırık refleksinin sırrı
+📊 Kaynaklar:
+• Shwartz Y, Gonzalez-Celeiro M, Chen CL, Hsu YC et al. (2020) Cell Types Promoting Goosebumps Form a Niche to Regulate Hair Follicle Stem Cells, Cell, 182(3): 578–593: https://doi.org/10.1016/j.cell.2020.06.031
+• Harvard Stem Cell Institute News: https://hscrb.harvard.edu/news/the-real-reason-behind-goosebumps/
+🩺 Uyarı: Genel bilimsel bilgi amaçlıdır, tıbbi tanı veya tavsiye değildir.
+🖼️ Görseller temsilîdir (bilimsel görselleştirme).
+Bir doz bilgi, her gün: 💊 ABONE OL!
+#bilgidozu #shorts #ürperti #kökhücre #harvard</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>#bilgidozu #shorts #ürperti #kökhücre #harvard</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>bilgidozu, shorts, tüyler neden diken diken olur, ürperti bilimi, arrector pili, harvard araştırması, kıl kökü kök hücre, sempatik sinir sistemi, insan vücudu, bilgi dozu</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>Tüyleri müzik dinlerken bile diken diken olanlar 1, sadece soğukta yaşayanlar 2 yazsın! 👇</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>Biyoloji ve Vücut</t>
+        </is>
+      </c>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>Harvard University — Shwartz, Hsu et al. (2020) Cell 182(3): 578–593</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>BEKLEMEDE</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>video_143.mp4</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Hıçkırık Mideden Gelmiyor: 35 Milisaniyelik Antik Refleks! 🫁 #bilgidozu #shorts</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>Hiç beklemediğin anda başlayan hıçkırık diyafram kasının ani spazmı ve sadece 35 milisaniye sonra ses tellerinin kilitlenmesidir; kökeni ise yüz milyonlarca yıllık amfibi solunum mirasına uzanır.
+📍 BÖLÜMLER
+00:00 Aniden başlayan hıçkırık krizi
+00:11 Frenik ve vagus siniri — diyafram spazmı
+00:20 35 milisaniye sonra kapanan ses telleri (glottis)
+00:30 Amfibi solungaç-akciğer evrimsel mirası
+00:39 Bebeklerde beslenme sırasında hava tahliyesi
+00:48 Sıradaki bölüm: soğan doğrarken göz yanması
+📊 Kaynaklar:
+• Straus C et al. (2003) A phylogenetic hypothesis for the origin of hiccough, BioEssays, 25(2): 182–188: https://doi.org/10.1002/bies.10257
+• Cleveland Clinic — Hiccups Causes &amp; Reflex Arc: https://my.clevelandclinic.org/health/diseases/17672-hiccups
+🩺 Uyarı: Genel bilimsel bilgi amaçlıdır, tıbbi tanı veya tavsiye değildir.
+🖼️ Görseller temsilîdir (bilimsel görselleştirme).
+Bir doz bilgi, her gün: 💊 ABONE OL!
+#bilgidozu #shorts #hıçkırık #diyafram #evrim</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>#bilgidozu #shorts #hıçkırık #diyafram #evrim</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>bilgidozu, shorts, hıçkırık neden tutar, hıçkırık nasıl geçer, diyafram spazmı, vagus siniri, glottis, evrimsel miras, insan vücudu, bilgi dozu</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>Hıçkırığı nefes tutarak geçirenler 1, soğuk su içenler 2 yazsın! 👇</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>Biyoloji ve Vücut</t>
+        </is>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>Straus et al. (2003) BioEssays &amp; Cleveland Clinic — Hiccup Reflex Arc</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>BEKLEMEDE</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>video_144.mp4</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Soğan Doğrarken Gözlerin Kokusundan Değil Kimyasal Gazdan Yanıyor! 🧅 #bilgidozu #shorts</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>Soğan doğrarken gözlerinin yanıp yaşarması kokusundan değil; bıçak darbesiyle birleşen enzimlerin havaya saldığı uçucu kükürt gazının göz neminde mikroskobik sülfürik aside dönüşmesindendir.
+📍 BÖLÜMLER
+00:00 Soğan doğrarken başlayan kimyasal savunma
+00:11 Hücrelerde ayrı kilitli tutulan kükürt ve enzimler
+00:19 Gözyaşı faktörü sentaz enzimi (Nature 2002)
+00:28 Göz neminde mikroskobik sülfürik asit oluşumu
+00:36 Kornea sinirleri ve acil gözyaşı yıkama emri
+00:44 Sıradaki bölüm: göz ovunca görülen renkli ışıklar
+📊 Kaynaklar:
+• Imai S et al. (2002) An onion enzyme that makes the eyes water, Nature, 419: 685: https://doi.org/10.1038/419685a
+• Library of Congress — Why does chopping an onion make you cry?: https://www.loc.gov/everyday-mysteries/food-and-nutrition/item/why-does-chopping-an-onion-make-you-cry/
+🩺 Uyarı: Genel bilimsel bilgi amaçlıdır, tıbbi tanı veya tavsiye değildir.
+🖼️ Görseller temsilîdir (bilimsel görselleştirme).
+Bir doz bilgi, her gün: 💊 ABONE OL!
+#bilgidozu #shorts #soğan #kimya #insanvücudu</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>#bilgidozu #shorts #soğan #kimya #insanvücudu</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>bilgidozu, shorts, soğan neden göz yaşartır, soğan doğrarken göz yanması, gözyaşı faktörü sentaz, sülfürik asit, kornea refleksi, günlük bilim, bilgi dozu</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>Soğan doğrarken hemen ağlayanlar 1, hiç etkilenmeyenler 2 yazsın! 👇</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>Fizik ve Kimya</t>
+        </is>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>Imai et al. (2002) Nature 419:685 &amp; Library of Congress</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>BEKLEMEDE</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>uzun_video_15.mp4</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Diken Diken Tüyler, Hıçkırık ve Soğan Gazının Gizli Mekanizması 🔬 #bilgidozu</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>Vücudunun senden izin almadan saniyeler içinde devreye soktuğu 3 otomatik savunma ve alarm mekanizmasını inceliyoruz: tüyleri diken diken eden kasların kök hücre bağlantısı, 35 milisaniyelik antik hıçkırık refleksi ve soğanın kimyasal gazına karşı korneanın acil yıkama kalkanı.
+📍 BÖLÜMLER
+00:00 Giriş: bedenin 3 otomatik savunma alarmı
+00:28 Arrector pili kasları ve Harvard kök hücre keşfi
+00:54 Hıçkırık refleksi ve diyafram spazmı
+01:21 35 milisaniye kilitlenme ve amfibi mirası
+01:49 Mutfaktaki kimyasal savunma: soğan hücreleri
+02:15 Gözyaşı faktörü sentaz ve uçucu gaz
+02:33 Kornea sinirleri ve gözyaşı kalkanı
+02:41 Özet: üç otomatik koruma sistemi
+📊 Kaynaklar:
+• Shwartz Y et al. (2020) Cell 182(3): 578–593 (Harvard Univ.): https://doi.org/10.1016/j.cell.2020.06.031
+• Straus C et al. (2003) BioEssays 25(2): 182–188 &amp; Cleveland Clinic
+• Imai S et al. (2002) Nature 419: 685 &amp; Library of Congress
+🩺 Uyarı: Genel bilimsel bilgi amaçlıdır, tıbbi tanı veya tavsiye değildir.
+🖼️ Görseller temsilîdir (bilimsel görselleştirme).
+Bir doz bilgi, her gün: 💊 ABONE OL!
+#bilgidozu #insanvücudu #refleks #bilim #belgesel</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>#bilgidozu #insanvücudu #refleks #bilim #belgesel</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>bilgidozu, vücudun savunma mekanizmaları, tüylerin diken diken olması, hıçkırık neden olur, soğan neden göz yakar, harvard kök hücre, biyoloji belgeseli, bilgi dozu</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>Vücudun bu 3 otomatik kalkanından hangisi seni daha çok şaşırttı? 🛡️ 1-Ürperti ve kök hücre 2-Hıçkırık mirası 3-Soğan kimyası — Numaranı yaz! 👇</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>Uzun — Biyoloji ve Vücut</t>
+        </is>
+      </c>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>Harvard Cell (2020), Straus BioEssays (2003) &amp; Imai Nature (2002)</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>BEKLEMEDE</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>video_145.mp4</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Gözünü Ovunca Karanlıkta Çıkan Renkli Işıklar Hayal Değil! 👁️ #bilgidozu #shorts</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>Gözlerini kapatıp hafifçe ovuşturduğunda karanlıkta beliren renkli yıldızlar ve halkalar hayal ürünü değil; göze tek foton girmeden retina hücrelerinin basınçla ateşlediği gerçek 'fosfen' sinyalleridir!
+📍 BÖLÜMLER
+00:00 Karanlıkta beliren renkli yıldızlar ve halkalar
+00:10 Fosfen: ışıksız görme deneyimi nedir?
+00:18 Retina hücrelerinin fiziksel basınca duyarlılığı
+00:27 Mekanik baskıyla ateşlenen elektrik sinyali
+00:36 Görsel korteksin sinyali ışık gibi çizmesi
+00:45 Sıradaki bölüm: uçakta kulak tıkanması
+📊 Kaynaklar:
+• Cleveland Clinic — Phosphenes (Seeing Stars): https://my.clevelandclinic.org/health/symptoms/24888-phosphenes
+• StatPearls / NCBI — Physiology, Phototransduction &amp; Retinal Ganglion Signaling
+🩺 Uyarı: Genel bilimsel bilgi amaçlıdır, tıbbi tanı veya tavsiye değildir.
+🖼️ Görseller temsilîdir (bilimsel görselleştirme).
+Bir doz bilgi, her gün: 💊 ABONE OL!
+#bilgidozu #shorts #fosfen #gözsağlığı #beyin</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>#bilgidozu #shorts #fosfen #gözsağlığı #beyin</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>bilgidozu, shorts, göz ovunca görülen ışıklar, fosfen nedir, karanlıkta renkli halkalar, retina, görsel korteks, nörobilim, insan vücudu, bilgi dozu</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>Gözünü kapatınca o renkli halkaları görenler 1, adını ilk kez duyanlar 2 yazsın! 👇</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>Beyin ve Psikoloji</t>
+        </is>
+      </c>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>Cleveland Clinic — Mechanical Phosphenes &amp; Retinal Ganglion Physiology</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>BEKLEMEDE</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>video_146.mp4</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Uçakta Tıkanan Kulağın Yutkununca Neden Çıt Sesiyle Açılır? ✈️ #bilgidozu #shorts</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>Uçak yükselirken ya da dağ yolunda çıkarken kulaklarının boğuklaşıp yutkunduğun an 'çıt' sesiyle açılması, orta kulaktaki kapalı basınç odasını dengeleyen gizli Östaki borusunun marifetidir.
+📍 BÖLÜMLER
+00:00 Yükseldikçe tıkanan kulak ve çıt sesi
+00:10 Kulak zarının arkasındaki yalıtılmış orta kulak
+00:18 İrtifa arttıkça zarı dışa iten basınç farkı
+00:27 Gerilen zarda su altı gibi boğuklaşan sesler
+00:34 Yutkunma ile açılan Östaki borusu ve denge
+00:44 Sıradaki bölüm: karın guruldamasının sırrı
+📊 Kaynaklar:
+• Cleveland Clinic — Ear Barotrauma &amp; Retracted Eardrum: https://my.clevelandclinic.org/health/diseases/25019-retracted-eardrum
+• Mayo Clinic — Airplane Ear (Ear Barotrauma) &amp; Eustachian Tube Function
+🩺 Uyarı: Genel bilimsel bilgi amaçlıdır, tıbbi tanı veya tavsiye değildir.
+🖼️ Görseller temsilîdir (bilimsel görselleştirme).
+Bir doz bilgi, her gün: 💊 ABONE OL!
+#bilgidozu #shorts #kulaktıkanması #uçak #bilim</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>#bilgidozu #shorts #kulaktıkanması #uçak #bilim</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>bilgidozu, shorts, uçakta kulak tıkanması, yüksekte kulak neden tıkanır, östaki borusu, orta kulak basıncı, kulak çıtlaması, insan vücudu, bilgi dozu</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>Yolculukta kulağı hemen tıkananlar 1, sakız veya esnemeyle anında açanlar 2 yazsın! 👇</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>Biyoloji ve Vücut</t>
+        </is>
+      </c>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>Cleveland Clinic &amp; Mayo Clinic — Ear Barotrauma &amp; Eustachian Tube</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>BEKLEMEDE</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>video_147.mp4</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Karın Guruldaması Açlık Değil: 90 Dakikalık Otomatik Temizlik! 🔬 #bilgidozu #shorts</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>Sessiz bir ortamda karnından yükselen gurultu (borborygmi) sadece açlık alarmı değil; sindirim sisteminin her 90 dakikada bir başlattığı 'Göç Eden Motor Kompleks' adlı otomatik iç temizlik dalgasıdır!
+📍 BÖLÜMLER
+00:00 Sessiz odada yankılanan karın gurultusu
+00:11 Borborygmi: mide ve ince bağırsak kanalları
+00:18 Her 90 dakikada başlayan Göç Eden Motor Kompleks
+00:27 Boş kanallarda akustik yankı ve iç süpürme
+00:36 Açlık alarmı değil, dip köşe bağırsak temizliği
+00:43 Yeni seri köprüsü: sabah ağız kokusunun sırrı
+📊 Kaynaklar:
+• Deloose E, Janssen P, Depoortere I, Tack J (2012) The migrating motor complex: control mechanisms and its role in health and disease, Nat. Rev. Gastroenterol. Hepatol., 9(5): 271–285: https://pubmed.ncbi.nlm.nih.gov/22450306/
+• Cleveland Clinic — Stomach Growling (Borborygmi)
+🩺 Uyarı: Genel bilimsel bilgi amaçlıdır, tıbbi tanı veya tavsiye değildir.
+🖼️ Görseller temsilîdir (bilimsel görselleştirme).
+Bir doz bilgi, her gün: 💊 ABONE OL!
+#bilgidozu #shorts #karıngurultusu #sindirim #bilim</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>#bilgidozu #shorts #karıngurultusu #sindirim #bilim</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>bilgidozu, shorts, karın neden guruldar, mide guruldaması, borborygmi, göç eden motor kompleks, bağırsak temizliği, sindirim sistemi, insan vücudu, bilgi dozu</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>En sessiz ortamda karnı guruldayanlar 1, su içip bastırmaya çalışanlar 2 yazsın! 👇</t>
+        </is>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>Biyoloji ve Vücut</t>
+        </is>
+      </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>Deloose et al. (2012) Nature Reviews Gastroenterology &amp; Hepatology (PMID: 22450306)</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>BEKLEMEDE</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>uzun_video_16.mp4</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Karanlıkta Renkli Işıklar, Kulak Tıkanması ve Karın Gurultusunun Sırrı ⚡ #bilgidozu</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>Gözünün, kulağının ve sindirim sisteminin her gün gönderdiği 3 gizemli iç sinyali tek belgeselde çözüyoruz: karanlıkta göz ovunca çakan mekanik fosfen ışıkları, yüksek irtifada kilitlenen orta kulak basıncı ve her 90 dakikada bağırsakları süpüren Göç Eden Motor Kompleks.
+📍 BÖLÜMLER
+00:00 Giriş: duyuların ve iç organların gizli sinyalleri
+00:28 Mekanik fosfen: ışıksız retina ve görsel korteks
+00:56 Uçakta ve dağ yolunda kulak tıkanması
+01:22 Orta kulak basıncı ve Östaki borusu kilidi
+01:47 Karın gurultusu (borborygmi) nereden gelir?
+02:14 Göç Eden Motor Kompleks: 90 dakikalık dalga
+02:32 Boş kanallarda akustik yankı ve iç temizlik
+02:39 Özet ve yeni seri duyurusu
+📊 Kaynaklar:
+• Cleveland Clinic — Phosphenes: https://my.clevelandclinic.org/health/symptoms/24888-phosphenes
+• Cleveland Clinic — Ear Barotrauma &amp; Eustachian Tube: https://my.clevelandclinic.org/health/diseases/25019-retracted-eardrum
+• Deloose E et al. (2012) Nat. Rev. Gastroenterol. Hepatol. 9(5): 271–285: https://pubmed.ncbi.nlm.nih.gov/22450306/
+🩺 Uyarı: Genel bilimsel bilgi amaçlıdır, tıbbi tanı veya tavsiye değildir.
+🖼️ Görseller temsilîdir (bilimsel görselleştirme).
+Bir doz bilgi, her gün: 💊 ABONE OL!
+#bilgidozu #insanvücudu #beyin #bilim #belgesel</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>#bilgidozu #insanvücudu #beyin #bilim #belgesel</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>bilgidozu, duyuların gizli sinyalleri, fosfen nedir, uçakta kulak tıkanması, östaki borusu, karın guruldaması neden olur, borborygmi, insan vücudu belgeseli, bilgi dozu</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>Vücudun bu 3 gizli sinyalinden hangisini daha sık yaşıyorsun? 👁️ 1-Karanlıkta ışık halkaları 2-Kulak tıkanması 3-Karın gurultusu — Numaranı bırak! 👇</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>Uzun — Beyin ve Psikoloji</t>
+        </is>
+      </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>Cleveland Clinic (Phosphenes &amp; Barotrauma) &amp; Deloose et al. (2012) Nat. Rev.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix(stok): 12 stok videosu yayın kuyruğundan çekildi — ESKİ_STOK_ASKIDA (kullanici: stok=yedek, siraya koyulmadi)
</commit_message>
<xml_diff>
--- a/bilgidozu_yukleme_tablosu.xlsx
+++ b/bilgidozu_yukleme_tablosu.xlsx
@@ -8085,7 +8085,7 @@
     <row r="132" ht="42" customHeight="1">
       <c r="A132" t="inlineStr">
         <is>
-          <t>BEKLEMEDE</t>
+          <t>ESKİ_STOK_ASKIDA</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -8146,7 +8146,7 @@
     <row r="133" ht="42" customHeight="1">
       <c r="A133" t="inlineStr">
         <is>
-          <t>BEKLEMEDE</t>
+          <t>ESKİ_STOK_ASKIDA</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -8207,7 +8207,7 @@
     <row r="134" ht="42" customHeight="1">
       <c r="A134" t="inlineStr">
         <is>
-          <t>BEKLEMEDE</t>
+          <t>ESKİ_STOK_ASKIDA</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -8268,7 +8268,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>BEKLEMEDE</t>
+          <t>ESKİ_STOK_ASKIDA</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -8333,7 +8333,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>BEKLEMEDE</t>
+          <t>ESKİ_STOK_ASKIDA</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -8394,7 +8394,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>BEKLEMEDE</t>
+          <t>ESKİ_STOK_ASKIDA</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -8455,7 +8455,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>BEKLEMEDE</t>
+          <t>ESKİ_STOK_ASKIDA</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -8516,7 +8516,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>BEKLEMEDE</t>
+          <t>ESKİ_STOK_ASKIDA</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -8580,7 +8580,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>BEKLEMEDE</t>
+          <t>ESKİ_STOK_ASKIDA</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -8641,7 +8641,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>BEKLEMEDE</t>
+          <t>ESKİ_STOK_ASKIDA</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -8702,7 +8702,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>BEKLEMEDE</t>
+          <t>ESKİ_STOK_ASKIDA</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -8763,7 +8763,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>BEKLEMEDE</t>
+          <t>ESKİ_STOK_ASKIDA</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">

</xml_diff>

<commit_message>
feat(stok): 9 short (139-147) kuyruğa alındı — 3 uzun (14-16) askıda kalıyor (kullanici karari)
</commit_message>
<xml_diff>
--- a/bilgidozu_yukleme_tablosu.xlsx
+++ b/bilgidozu_yukleme_tablosu.xlsx
@@ -8085,7 +8085,7 @@
     <row r="132" ht="42" customHeight="1">
       <c r="A132" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -8146,7 +8146,7 @@
     <row r="133" ht="42" customHeight="1">
       <c r="A133" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -8207,7 +8207,7 @@
     <row r="134" ht="42" customHeight="1">
       <c r="A134" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -8333,7 +8333,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -8394,7 +8394,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -8455,7 +8455,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -8580,7 +8580,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -8641,7 +8641,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -8702,7 +8702,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">

</xml_diff>

<commit_message>
feat(seri-zinciri): 'İlgili Video' (relatedVideos) otomatik bağlantı — uzun yayınlanınca 3 short'a, short yayınlanınca uzununa bağlar; tabloya 'İlgili Video' sütunu + stok 14-16 eşlemesi
</commit_message>
<xml_diff>
--- a/bilgidozu_yukleme_tablosu.xlsx
+++ b/bilgidozu_yukleme_tablosu.xlsx
@@ -524,7 +524,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M143"/>
+  <dimension ref="A1:N143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -605,6 +605,11 @@
       <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Yorum Sayısı</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>İlgili Video</t>
         </is>
       </c>
     </row>
@@ -8329,6 +8334,11 @@
           <t>Johns Hopkins Medicine, Kawchuk et al. (2015) PLOS ONE &amp; Cleveland Clinic</t>
         </is>
       </c>
+      <c r="N135" t="inlineStr">
+        <is>
+          <t>video_139.mp4, video_140.mp4, video_141.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -8576,6 +8586,11 @@
           <t>Harvard Cell (2020), Straus BioEssays (2003) &amp; Imai Nature (2002)</t>
         </is>
       </c>
+      <c r="N139" t="inlineStr">
+        <is>
+          <t>video_142.mp4, video_143.mp4, video_144.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -8823,6 +8838,11 @@
           <t>Cleveland Clinic (Phosphenes &amp; Barotrauma) &amp; Deloose et al. (2012) Nat. Rev.</t>
         </is>
       </c>
+      <c r="N143" t="inlineStr">
+        <is>
+          <t>video_145.mp4, video_146.mp4, video_147.mp4</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(stok): REİS emri — 3 stok uzun (14-16) kuyruğa; MIN_LONG_NUMBER 101->14 (14-16 + yeni seri 17+ yayina, eski 1..13 kilitli kalir)
</commit_message>
<xml_diff>
--- a/bilgidozu_yukleme_tablosu.xlsx
+++ b/bilgidozu_yukleme_tablosu.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="DRIVE" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="ISCILER" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="UYARILAR" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DRIVE" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ISCILER" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UYARILAR" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -8273,7 +8273,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -8526,7 +8526,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -8778,7 +8778,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>ESKİ_STOK_ASKIDA</t>
+          <t>BEKLEMEDE</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">

</xml_diff>

<commit_message>
feat(kopru): video_157 (29 Ekim Cumhuriyet ozel) kuyruga + FORCE: 19:30 TR slotuna sabitlendi
</commit_message>
<xml_diff>
--- a/bilgidozu_yukleme_tablosu.xlsx
+++ b/bilgidozu_yukleme_tablosu.xlsx
@@ -524,7 +524,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N143"/>
+  <dimension ref="A1:N144"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -8844,6 +8844,66 @@
         </is>
       </c>
     </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>BEKLEMEDE</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>video_157.mp4</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Üçgen ve Açı Kelimelerini Atatürk'ün Bizzat Türettiğini Biliyor muydun? 🇹🇷 #bilgidozu #shorts</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>Bugün okulda tek nefeste söylediğin üçgen, kare, açı ve artı kelimelerini kimin oturup türettiğini hiç düşündün mü? Bin dokuz yüz otuz altı kışında Atatürk masa başına geçti ve adını bile koymadığı kırk dört sayfalık Geometri kitabını yazdı.
+📍 BÖLÜMLER
+00:00 Üçgen, kare ve açi adini — Ki̇m türetti̇ bi̇li̇yor musun?
+00:08 Cumhuri̇yet'ten önce üçgen: — Ezberi̇ zor ağir teri̇mler!
+00:17 1936 kişi i̇si̇msi̇z eser: — 44 sayfalik geometri̇ ki̇tabi!
+00:26 Arti, eksi̇, çap, uzay: — Bi̇li̇m di̇li̇ tertemi̇z oldu!
+00:37 29 eki̇m'i̇n gerçek ruhu: — Akil ve bi̇li̇m devri̇mi̇!
+00:46 103. yilimiz kutlu olsun! — Yoruma yaz &amp; taki̇p et!
+📊 Kaynaklar:
+• Kaynak: Türk Dil Kurumu &amp; Kültür Bakanlığı Geometri Kılavuzu (1937)
+• https://tdk.gov.tr/
+🖼️ Görseller temsili (AI bilimsel canlandırma).
+Cumhuriyetimizin 103. yılı kutlu olsun! Daha fazla bilgi dozu için takip etmeyi unutma! 🔔
+#bilgidozu #shorts #29ekim #cumhuriyetbayramı #bilim #tarih</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>#bilgidozu #shorts #29ekim #cumhuriyetbayramı #bilim #tarih</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>bilgidozu, shorts, 29 ekim, cumhuriyet bayramı, atatürk geometri kitabı, üçgen kelimesini kim buldu, bilim tarihi, türkçe matematik terimleri, bilgi dozu</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>Üçgen, açı, uzay, köşegen, artı, eksi... Senin en sevdiğin Türkçe bilim kelimesi hangisi? 29 Ekim Cumhuriyet Bayramımız kutlu olsun! 👇</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>29 Ekim Özel — Bilim Tarihi</t>
+        </is>
+      </c>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>Türk Dil Kurumu (TDK) &amp; Kültür Bakanlığı Geometri Kılavuzu (1937)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix(kayit): video_157 YUKLENDI — botun kayit push'u dusmustu (dispatch run failure), elle tamamlandi
</commit_message>
<xml_diff>
--- a/bilgidozu_yukleme_tablosu.xlsx
+++ b/bilgidozu_yukleme_tablosu.xlsx
@@ -8847,7 +8847,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>BEKLEMEDE</t>
+          <t>YÜKLENDİ</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -8901,6 +8901,16 @@
       <c r="I144" t="inlineStr">
         <is>
           <t>Türk Dil Kurumu (TDK) &amp; Kültür Bakanlığı Geometri Kılavuzu (1937)</t>
+        </is>
+      </c>
+      <c r="J144" t="inlineStr">
+        <is>
+          <t>https://youtu.be/t2lphcITKXs</t>
+        </is>
+      </c>
+      <c r="K144" t="inlineStr">
+        <is>
+          <t>2026-10-29 19:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(qc) CLOUD bildirimi MADDE 1-5 (REIS emri, 30.10):
1) Onarim mekanizmasi: repair_video.json + workflow adimi (--repair) ->
   QhqHWaVWLJY canli aciklama (YouTube uyumlu bolumler) + Cloud kapaği
   (17RrU2QB2hl4ujhtRFg6nSrqqJwrjU2qF) giydirilecek
2) Kapaklar: KAPAKLAR'da 17-22 Cloud'un 1920x1080 yuksek-CTR versiyonlariyla
   degistirildi (eski '3 BOLUM • TEK VİDEO' şablonlari trash)
3) İlgili Video 1'e 1: u17→148, u18→151, u19→155, u20→158, u21→161, u22→164
4) Tablo AÇIKLAMA'ları Cloud baslik.xlsx v7'den senkron (>=15 sn bolumler,
   🔗 iç notlar ve i̇ kaymalari temiz); bota sanitizer eklendi (🔗 satirlari
   asla yayina gitmez, <10 sn aralık uyarir)
5) CUMA IKIZ KURALI: bugün uzun yayınlanırsa 19:30 = o uzunun 1'e 1 twin
   short'u; BUGÜN 19:30 = video_148.mp4 (force + kural çift güvence)
</commit_message>
<xml_diff>
--- a/bilgidozu_yukleme_tablosu.xlsx
+++ b/bilgidozu_yukleme_tablosu.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="DRIVE" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="ISCILER" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="UYARILAR" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DRIVE" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ISCILER" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UYARILAR" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -124,7 +124,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -159,6 +159,8 @@
     <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -524,7 +526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N144"/>
+  <dimension ref="A1:N168"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1247,7 +1249,7 @@
         </is>
       </c>
       <c r="L11" s="3" t="n">
-        <v>522</v>
+        <v>520</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>1</v>
@@ -1777,7 +1779,7 @@
         </is>
       </c>
       <c r="L19" s="3" t="n">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="M19" s="3" t="n"/>
     </row>
@@ -1847,7 +1849,7 @@
     <row r="21" ht="42" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>SİLİNDİ</t>
+          <t>YÜKLENDİ</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -1906,7 +1908,7 @@
     <row r="22" ht="42" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>SİLİNDİ</t>
+          <t>YÜKLENDİ</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -2020,7 +2022,7 @@
     <row r="24" ht="42" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>SİLİNDİ</t>
+          <t>YÜKLENDİ</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -2083,7 +2085,7 @@
     <row r="25" ht="42" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>SİLİNDİ</t>
+          <t>YÜKLENDİ</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -2816,7 +2818,7 @@
         </is>
       </c>
       <c r="L38" s="3" t="n">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="M38" s="3" t="n">
         <v>1</v>
@@ -3130,7 +3132,7 @@
         </is>
       </c>
       <c r="L43" s="3" t="n">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="M43" s="3" t="n"/>
     </row>
@@ -3254,7 +3256,7 @@
         </is>
       </c>
       <c r="L45" s="3" t="n">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="M45" s="3" t="n"/>
     </row>
@@ -3821,22 +3823,22 @@
       <c r="M55" s="8" t="n"/>
     </row>
     <row r="56" ht="42" customHeight="1">
-      <c r="A56" s="7" t="inlineStr">
-        <is>
-          <t>BEKLEMEDE</t>
-        </is>
-      </c>
-      <c r="B56" s="7" t="inlineStr">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>YÜKLENDİ</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
         <is>
           <t>video_96.mp4</t>
         </is>
       </c>
-      <c r="C56" s="8" t="inlineStr">
+      <c r="C56" s="3" t="inlineStr">
         <is>
           <t>Kendi Sesini Kayıtta Dinleyince Neden Tuhaf Gelir? 🎙️ #bilgidozu #shorts</t>
         </is>
       </c>
-      <c r="D56" s="8" t="inlineStr">
+      <c r="D56" s="3" t="inlineStr">
         <is>
           <t>Bir ses kaydında kendi sesini duyduğun an “Bu gerçekten benim sesim mi?” diye yüzünü buruşturduğun oldu mu? Merak etme, yalnız değilsin. Sen konuşurken sesini iki farklı yoldan aynı anda duyarsın. Hem havadan kulağına gelen dalgalarla, hem de ses tellerinin kafatası kemiklerini titreştirerek iç kulağına gönderdiği kemik iletimiyle. Kafatası kemiklerin bas frekansları güçlendirdiği için kendi sesini hep daha tok ve derin algılarsın. Ama kayıtta, kemik iletimi devreden çıkar ve başkalarının duyduğu o gerçek sesine yüzleşirsin. Peki sen kayıtlarda kendi sesini dinlemeye alışabildin mi, yoksa duyunca hemen kapatıyor musun? Yorumlarda buluşalım.
 💬 Peki sen kendi sesini kayıtlarda dinlemeye alışabildin mi, yoksa duyunca hâlâ hemen kapatıyor musun? Yorumlarda buluşalım! 👇
@@ -3845,35 +3847,43 @@
 #bilgidozu #shorts #nörobilim #insanbedeni #psikoloji #bilim</t>
         </is>
       </c>
-      <c r="E56" s="8" t="inlineStr">
+      <c r="E56" s="3" t="inlineStr">
         <is>
           <t>#bilgidozu #shorts #nörobilim #insanbedeni #psikoloji #bilim</t>
         </is>
       </c>
-      <c r="F56" s="8" t="inlineStr">
+      <c r="F56" s="3" t="inlineStr">
         <is>
           <t>bilgidozu, shorts, nörobilim, insan bedeni, psikoloji, bilim</t>
         </is>
       </c>
-      <c r="G56" s="8" t="inlineStr">
+      <c r="G56" s="3" t="inlineStr">
         <is>
           <t>Peki sen kendi sesini kayıtlarda dinlemeye alışabildin mi, yoksa duyunca hâlâ hemen kapatıyor musun? Yorumlarda buluşalım! 👇</t>
         </is>
       </c>
-      <c r="H56" s="8" t="inlineStr">
+      <c r="H56" s="3" t="inlineStr">
         <is>
           <t>Nörobilim ve İnsan Bedeni</t>
         </is>
       </c>
-      <c r="I56" s="8" t="inlineStr">
+      <c r="I56" s="3" t="inlineStr">
         <is>
           <t>Journal of Voice / Wikipedia — Bone Conduction (Kafatası Kemik İletimi): https://en.wikipedia.org/wiki/Bone_conduction</t>
         </is>
       </c>
-      <c r="J56" s="8" t="n"/>
-      <c r="K56" s="8" t="n"/>
-      <c r="L56" s="8" t="n"/>
-      <c r="M56" s="8" t="n"/>
+      <c r="J56" s="3" t="inlineStr">
+        <is>
+          <t>https://youtu.be/aat1STZfbps</t>
+        </is>
+      </c>
+      <c r="K56" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-29 21:11</t>
+        </is>
+      </c>
+      <c r="L56" s="3" t="n"/>
+      <c r="M56" s="3" t="n"/>
     </row>
     <row r="57" ht="42" customHeight="1">
       <c r="A57" s="7" t="inlineStr">
@@ -4041,22 +4051,22 @@
       <c r="M59" s="8" t="n"/>
     </row>
     <row r="60" ht="42" customHeight="1">
-      <c r="A60" s="7" t="inlineStr">
-        <is>
-          <t>BEKLEMEDE</t>
-        </is>
-      </c>
-      <c r="B60" s="7" t="inlineStr">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>YÜKLENDİ</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
         <is>
           <t>video_100.mp4</t>
         </is>
       </c>
-      <c r="C60" s="8" t="inlineStr">
+      <c r="C60" s="3" t="inlineStr">
         <is>
           <t>Utandığında Neden Sadece Yüzün ve Kulakların Kızarır? 😳 #bilgidozu #shorts</t>
         </is>
       </c>
-      <c r="D60" s="8" t="inlineStr">
+      <c r="D60" s="3" t="inlineStr">
         <is>
           <t>Herkesin içinde bir anda utandığında neden kolların değil de sadece yanakların ve kulakların alev alev kızarır? Üstelik sakın kızarma dedikçe daha da kıpkırmızı olursun. Charles Darwin'in tüm duyguların en insaniye olanı dediği bu tepki vücudunun gizli dürüstlük mekanizmasıdır. Utandığın saniye beynin ani bir adrenalin salgılar ve sadece yüzündeki özel kılcal damarlar genişleyerek cildinin altına sıcak kan hücum eder. Evrimsel olarak bu tek kelime etmeden çevrendekilere hata yaptım ve farkındayım demenin sessiz yoludur. Peki sen utandığında sakin kalabilenlerden misin, yoksa saniyesinde kızaranlardan mı? Yorumlarda buluşalım.
 💬 Peki sen utandığında rengini belli etmeden sakin kalabilenlerden misin, yoksa saniyesinde pancar gibi kızaranlardan mı? Yorumlarda buluşalım! 👇
@@ -4065,53 +4075,61 @@
 #bilgidozu #shorts #nörobilim #insanbedeni #psikoloji #bilim</t>
         </is>
       </c>
-      <c r="E60" s="8" t="inlineStr">
+      <c r="E60" s="3" t="inlineStr">
         <is>
           <t>#bilgidozu #shorts #nörobilim #insanbedeni #psikoloji #bilim</t>
         </is>
       </c>
-      <c r="F60" s="8" t="inlineStr">
+      <c r="F60" s="3" t="inlineStr">
         <is>
           <t>bilgidozu, shorts, nörobilim, insan bedeni, psikoloji, bilim</t>
         </is>
       </c>
-      <c r="G60" s="8" t="inlineStr">
+      <c r="G60" s="3" t="inlineStr">
         <is>
           <t>Peki sen utandığında rengini belli etmeden sakin kalabilenlerden misin, yoksa saniyesinde pancar gibi kızaranlardan mı? Yorumlarda buluşalım! 👇</t>
         </is>
       </c>
-      <c r="H60" s="8" t="inlineStr">
+      <c r="H60" s="3" t="inlineStr">
         <is>
           <t>Nörobilim ve İnsan Bedeni</t>
         </is>
       </c>
-      <c r="I60" s="8" t="inlineStr">
+      <c r="I60" s="3" t="inlineStr">
         <is>
           <t>Charles Darwin / Wikipedia — Blushing Physiology (Yüz Kızarması Mekanizması): https://en.wikipedia.org/wiki/Blushing</t>
         </is>
       </c>
-      <c r="J60" s="8" t="n"/>
-      <c r="K60" s="8" t="n"/>
-      <c r="L60" s="8" t="n"/>
-      <c r="M60" s="8" t="n"/>
+      <c r="J60" s="3" t="inlineStr">
+        <is>
+          <t>https://youtu.be/j8J7rqtyyFg</t>
+        </is>
+      </c>
+      <c r="K60" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-28 19:37</t>
+        </is>
+      </c>
+      <c r="L60" s="3" t="n"/>
+      <c r="M60" s="3" t="n"/>
     </row>
     <row r="61" ht="42" customHeight="1">
-      <c r="A61" s="7" t="inlineStr">
-        <is>
-          <t>BEKLEMEDE</t>
-        </is>
-      </c>
-      <c r="B61" s="7" t="inlineStr">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>YÜKLENDİ</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
         <is>
           <t>video_86.mp4</t>
         </is>
       </c>
-      <c r="C61" s="8" t="inlineStr">
+      <c r="C61" s="3" t="inlineStr">
         <is>
           <t>Vücudundaki Hücrelerin Yarısından Fazlası Aslında Bakteri! 🦠 #bilgidozu #shorts</t>
         </is>
       </c>
-      <c r="D61" s="8" t="inlineStr">
+      <c r="D61" s="3" t="inlineStr">
         <is>
           <t>İnsan bedeninde yaklaşık 30 trilyon insan hücresine karşılık 38 trilyondan fazla dost bakteri hücresi yaşar.
 Peki vücudunuzda kendi hücrelerinizden daha fazla bakteri yaşaması size nasıl hissettiriyor? Yorumlara yazın! 👇
@@ -4120,35 +4138,43 @@
 #bilgidozu #shorts #insanvücudu #bilim #biyoloji</t>
         </is>
       </c>
-      <c r="E61" s="8" t="inlineStr">
+      <c r="E61" s="3" t="inlineStr">
         <is>
           <t>#bilgidozu #shorts #insanvücudu #bilim #biyoloji</t>
         </is>
       </c>
-      <c r="F61" s="8" t="inlineStr">
+      <c r="F61" s="3" t="inlineStr">
         <is>
           <t>bilgi dozu, insan vücudu, bakteri, biyoloji, bilim, shorts</t>
         </is>
       </c>
-      <c r="G61" s="8" t="inlineStr">
+      <c r="G61" s="3" t="inlineStr">
         <is>
           <t>Peki vücudunuzda kendi hücrelerinizden daha fazla bakteri yaşaması size nasıl hissettiriyor? Yorumlara yazın! 👇</t>
         </is>
       </c>
-      <c r="H61" s="8" t="inlineStr">
+      <c r="H61" s="3" t="inlineStr">
         <is>
           <t>İnsan Vücudu ve Psikoloji</t>
         </is>
       </c>
-      <c r="I61" s="8" t="inlineStr">
+      <c r="I61" s="3" t="inlineStr">
         <is>
           <t>PLOS Biology (Sender et al., 2016) — Revised Estimates for Human &amp; Bacteria Cells: https://journals.plos.org/plosbiology/article?id=10.1371/journal.pbio.1002533</t>
         </is>
       </c>
-      <c r="J61" s="8" t="n"/>
-      <c r="K61" s="8" t="n"/>
-      <c r="L61" s="8" t="n"/>
-      <c r="M61" s="8" t="n"/>
+      <c r="J61" s="3" t="inlineStr">
+        <is>
+          <t>https://youtu.be/Bn5vzNjsnWo</t>
+        </is>
+      </c>
+      <c r="K61" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-28 21:10</t>
+        </is>
+      </c>
+      <c r="L61" s="3" t="n"/>
+      <c r="M61" s="3" t="n"/>
     </row>
     <row r="62" ht="42" customHeight="1">
       <c r="A62" s="7" t="inlineStr">
@@ -4206,22 +4232,22 @@
       <c r="M62" s="8" t="n"/>
     </row>
     <row r="63" ht="42" customHeight="1">
-      <c r="A63" s="7" t="inlineStr">
-        <is>
-          <t>BEKLEMEDE</t>
-        </is>
-      </c>
-      <c r="B63" s="7" t="inlineStr">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>YÜKLENDİ</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
         <is>
           <t>video_83.mp4</t>
         </is>
       </c>
-      <c r="C63" s="8" t="inlineStr">
+      <c r="C63" s="3" t="inlineStr">
         <is>
           <t>Sevdiğin Birine Bakınca Göz Bebeğin Neden Otomatik Büyür? 👀 #bilgidozu #shorts</t>
         </is>
       </c>
-      <c r="D63" s="8" t="inlineStr">
+      <c r="D63" s="3" t="inlineStr">
         <is>
           <t>Hoşlandığımız birine baktığımızda dopamin ve oksitosin etkisiyle sempatik sinir sistemi göz bebeklerimizi istemsizce büyütür.
 Siz konuşurken karşınızdakinin göz bebeklerine dikkat eder misiniz? Yorumlara yazın! 👇
@@ -4230,35 +4256,43 @@
 #bilgidozu #shorts #psikoloji #insanvücudu #bilim</t>
         </is>
       </c>
-      <c r="E63" s="8" t="inlineStr">
+      <c r="E63" s="3" t="inlineStr">
         <is>
           <t>#bilgidozu #shorts #psikoloji #insanvücudu #bilim</t>
         </is>
       </c>
-      <c r="F63" s="8" t="inlineStr">
+      <c r="F63" s="3" t="inlineStr">
         <is>
           <t>bilgi dozu, psikoloji, göz bebeği, insan vücudu, bilim, shorts</t>
         </is>
       </c>
-      <c r="G63" s="8" t="inlineStr">
+      <c r="G63" s="3" t="inlineStr">
         <is>
           <t>Siz konuşurken karşınızdakinin göz bebeklerine dikkat eder misiniz? Yorumlara yazın! 👇</t>
         </is>
       </c>
-      <c r="H63" s="8" t="inlineStr">
+      <c r="H63" s="3" t="inlineStr">
         <is>
           <t>İnsan Vücudu ve Psikoloji</t>
         </is>
       </c>
-      <c r="I63" s="8" t="inlineStr">
+      <c r="I63" s="3" t="inlineStr">
         <is>
           <t>Hess &amp; Polt (1960) / Wikipedia — Pupillometry Research: https://en.wikipedia.org/wiki/Pupillometry</t>
         </is>
       </c>
-      <c r="J63" s="8" t="n"/>
-      <c r="K63" s="8" t="n"/>
-      <c r="L63" s="8" t="n"/>
-      <c r="M63" s="8" t="n"/>
+      <c r="J63" s="3" t="inlineStr">
+        <is>
+          <t>https://youtu.be/0vGKrBpJh0Q</t>
+        </is>
+      </c>
+      <c r="K63" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-28 14:07</t>
+        </is>
+      </c>
+      <c r="L63" s="3" t="n"/>
+      <c r="M63" s="3" t="n"/>
     </row>
     <row r="64" ht="42" customHeight="1">
       <c r="A64" s="7" t="inlineStr">
@@ -4682,7 +4716,7 @@
         </is>
       </c>
       <c r="L70" s="3" t="n">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="M70" s="3" t="n"/>
     </row>
@@ -7451,22 +7485,22 @@
       <c r="M121" s="8" t="n"/>
     </row>
     <row r="122" ht="42" customHeight="1">
-      <c r="A122" s="7" t="inlineStr">
-        <is>
-          <t>BEKLEMEDE</t>
-        </is>
-      </c>
-      <c r="B122" s="7" t="inlineStr">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
+          <t>YÜKLENDİ</t>
+        </is>
+      </c>
+      <c r="B122" s="2" t="inlineStr">
         <is>
           <t>video_108.mp4</t>
         </is>
       </c>
-      <c r="C122" s="8" t="inlineStr">
+      <c r="C122" s="3" t="inlineStr">
         <is>
           <t>Voynich El Yazması: 600 Yıldır Kimsenin Okuyamadığı Şifreli Kitap! 📜 #bilgidozu #shorts</t>
         </is>
       </c>
-      <c r="D122" s="8" t="inlineStr">
+      <c r="D122" s="3" t="inlineStr">
         <is>
           <t>Dünyanın en iyi şifre çözücüleri, dilbilimcileri ve yapay zekâları bir araya geldi ama altı yüz yıllık bu kitabın tek bir cümlesini bile okuyamadı: Voynich El Yazması.
 💬 Peki sence bu kitap unutulmuş gizli bir bilimin şifreli kaydı mı, yoksa tarihin en zekice kurgulanmış bilmecesi mi? Yorumlarda buluşalım! 👇
@@ -7475,35 +7509,43 @@
 #bilgidozu #shorts #tarih #arkeoloji #bilim</t>
         </is>
       </c>
-      <c r="E122" s="8" t="inlineStr">
+      <c r="E122" s="3" t="inlineStr">
         <is>
           <t>#bilgidozu #shorts #tarih #arkeoloji #bilim #dozdışı</t>
         </is>
       </c>
-      <c r="F122" s="8" t="inlineStr">
+      <c r="F122" s="3" t="inlineStr">
         <is>
           <t>bilgi dozu, antik mühendislik, tarih, arkeoloji, gizemli yapılar, bilim, shorts, doz dışı</t>
         </is>
       </c>
-      <c r="G122" s="8" t="inlineStr">
+      <c r="G122" s="3" t="inlineStr">
         <is>
           <t>Peki sence bu kitap unutulmuş gizli bir bilimin şifreli kaydı mı, yoksa tarihin en zekice kurgulanmış bilmecesi mi? Yorumlarda buluşalım! 👇</t>
         </is>
       </c>
-      <c r="H122" s="8" t="inlineStr">
+      <c r="H122" s="3" t="inlineStr">
         <is>
           <t>Tarih ve Antik Mühendislik</t>
         </is>
       </c>
-      <c r="I122" s="8" t="inlineStr">
+      <c r="I122" s="3" t="inlineStr">
         <is>
           <t>Yale Beinecke Library / Wikipedia — Voynich Manuscript (Voynich El Yazması): https://en.wikipedia.org/wiki/Voynich_manuscript</t>
         </is>
       </c>
-      <c r="J122" s="8" t="n"/>
-      <c r="K122" s="8" t="n"/>
-      <c r="L122" s="8" t="n"/>
-      <c r="M122" s="8" t="n"/>
+      <c r="J122" s="3" t="inlineStr">
+        <is>
+          <t>https://youtu.be/7DG1etjQlR4</t>
+        </is>
+      </c>
+      <c r="K122" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-28 10:58</t>
+        </is>
+      </c>
+      <c r="L122" s="3" t="n"/>
+      <c r="M122" s="3" t="n"/>
     </row>
     <row r="123" ht="42" customHeight="1">
       <c r="A123" s="7" t="inlineStr">
@@ -7753,7 +7795,7 @@
         </is>
       </c>
       <c r="L126" s="3" t="n">
-        <v>705</v>
+        <v>700</v>
       </c>
       <c r="M126" s="3" t="n"/>
     </row>
@@ -7829,7 +7871,7 @@
         </is>
       </c>
       <c r="L127" s="3" t="n">
-        <v>238</v>
+        <v>225</v>
       </c>
       <c r="M127" s="3" t="n"/>
     </row>
@@ -7904,27 +7946,27 @@
         </is>
       </c>
       <c r="L128" s="3" t="n">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="M128" s="3" t="n"/>
     </row>
     <row r="129" ht="42" customHeight="1">
-      <c r="A129" s="10" t="inlineStr">
-        <is>
-          <t>BEKLEMEDE</t>
-        </is>
-      </c>
-      <c r="B129" s="10" t="inlineStr">
+      <c r="A129" s="2" t="inlineStr">
+        <is>
+          <t>YÜKLENDİ</t>
+        </is>
+      </c>
+      <c r="B129" s="2" t="inlineStr">
         <is>
           <t>video_135.mp4</t>
         </is>
       </c>
-      <c r="C129" s="11" t="inlineStr">
+      <c r="C129" s="3" t="inlineStr">
         <is>
           <t>Güneşe Dönünce Hapşırıyor musun? Bu Bir Refleks: ACHOO! ☀️ #bilgidozu #shorts</t>
         </is>
       </c>
-      <c r="D129" s="11" t="inlineStr">
+      <c r="D129" s="3" t="inlineStr">
         <is>
           <t>Güneşli havada hapşırıyorsan bu bir alerji değil: fotik hapşırma refleksi, yani ACHOO. Toplumun yaklaşık %18–%35'inde var.
 📍 BÖLÜMLER
@@ -7943,35 +7985,43 @@
 #bilgidozu #shorts #ACHOO #hapşırma #genetik</t>
         </is>
       </c>
-      <c r="E129" s="11" t="inlineStr">
+      <c r="E129" s="3" t="inlineStr">
         <is>
           <t>#bilgidozu #shorts #ACHOO #hapşırma #genetik</t>
         </is>
       </c>
-      <c r="F129" s="11" t="inlineStr">
+      <c r="F129" s="3" t="inlineStr">
         <is>
           <t>bilgidozu, shorts, ACHOO, fotik hapşırma, güneş hapşırması, hapşırma refleksi, genetik, otozomal dominant, insan vücudu, bilgi dozu</t>
         </is>
       </c>
-      <c r="G129" s="11" t="inlineStr">
+      <c r="G129" s="3" t="inlineStr">
         <is>
           <t>Güneşte hapşırıyorsan 1 yaz, hiç tepki vermeyen 2 yazsın! 👇</t>
         </is>
       </c>
-      <c r="H129" s="11" t="inlineStr">
+      <c r="H129" s="3" t="inlineStr">
         <is>
           <t>İnsan Vücudu ve Beyin</t>
         </is>
       </c>
-      <c r="I129" s="11" t="inlineStr">
+      <c r="I129" s="3" t="inlineStr">
         <is>
           <t>Nature Scientific Reports (2019) &amp; Cleveland Clinic JM</t>
         </is>
       </c>
-      <c r="J129" s="11" t="n"/>
-      <c r="K129" s="11" t="n"/>
-      <c r="L129" s="11" t="n"/>
-      <c r="M129" s="11" t="n"/>
+      <c r="J129" s="3" t="inlineStr">
+        <is>
+          <t>https://youtu.be/LGXmOwTtGOw</t>
+        </is>
+      </c>
+      <c r="K129" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-28 01:00</t>
+        </is>
+      </c>
+      <c r="L129" s="3" t="n"/>
+      <c r="M129" s="3" t="n"/>
     </row>
     <row r="130" ht="42" customHeight="1">
       <c r="A130" s="10" t="inlineStr">
@@ -8845,31 +8895,28 @@
       </c>
     </row>
     <row r="144">
-      <c r="A144" t="inlineStr">
+      <c r="A144" s="12" t="inlineStr">
         <is>
           <t>YÜKLENDİ</t>
         </is>
       </c>
-      <c r="B144" t="inlineStr">
+      <c r="B144" s="12" t="inlineStr">
         <is>
           <t>video_157.mp4</t>
         </is>
       </c>
-      <c r="C144" t="inlineStr">
+      <c r="C144" s="13" t="inlineStr">
         <is>
           <t>Üçgen ve Açı Kelimelerini Atatürk'ün Bizzat Türettiğini Biliyor muydun? 🇹🇷 #bilgidozu #shorts</t>
         </is>
       </c>
-      <c r="D144" t="inlineStr">
+      <c r="D144" s="13" t="inlineStr">
         <is>
           <t>Bugün okulda tek nefeste söylediğin üçgen, kare, açı ve artı kelimelerini kimin oturup türettiğini hiç düşündün mü? Bin dokuz yüz otuz altı kışında Atatürk masa başına geçti ve adını bile koymadığı kırk dört sayfalık Geometri kitabını yazdı.
 📍 BÖLÜMLER
-00:00 Üçgen, kare ve açi adini — Ki̇m türetti̇ bi̇li̇yor musun?
-00:08 Cumhuri̇yet'ten önce üçgen: — Ezberi̇ zor ağir teri̇mler!
-00:17 1936 kişi i̇si̇msi̇z eser: — 44 sayfalik geometri̇ ki̇tabi!
-00:26 Arti, eksi̇, çap, uzay: — Bi̇li̇m di̇li̇ tertemi̇z oldu!
-00:37 29 eki̇m'i̇n gerçek ruhu: — Akil ve bi̇li̇m devri̇mi̇!
-00:46 103. yilimiz kutlu olsun! — Yoruma yaz &amp; taki̇p et!
+00:00 Üçgen, kare ve açi adini — Kim türetti biliyor musun?
+00:17 1936 kişi isimsiz eser: — 44 sayfalik geometri kitabi!
+00:37 29 ekim'in gerçek ruhu: — Akil ve bilim devrimi!
 📊 Kaynaklar:
 • Kaynak: Türk Dil Kurumu &amp; Kültür Bakanlığı Geometri Kılavuzu (1937)
 • https://tdk.gov.tr/
@@ -8878,43 +8925,1458 @@
 #bilgidozu #shorts #29ekim #cumhuriyetbayramı #bilim #tarih</t>
         </is>
       </c>
-      <c r="E144" t="inlineStr">
+      <c r="E144" s="13" t="inlineStr">
         <is>
           <t>#bilgidozu #shorts #29ekim #cumhuriyetbayramı #bilim #tarih</t>
         </is>
       </c>
-      <c r="F144" t="inlineStr">
+      <c r="F144" s="13" t="inlineStr">
         <is>
           <t>bilgidozu, shorts, 29 ekim, cumhuriyet bayramı, atatürk geometri kitabı, üçgen kelimesini kim buldu, bilim tarihi, türkçe matematik terimleri, bilgi dozu</t>
         </is>
       </c>
-      <c r="G144" t="inlineStr">
+      <c r="G144" s="13" t="inlineStr">
         <is>
           <t>Üçgen, açı, uzay, köşegen, artı, eksi... Senin en sevdiğin Türkçe bilim kelimesi hangisi? 29 Ekim Cumhuriyet Bayramımız kutlu olsun! 👇</t>
         </is>
       </c>
-      <c r="H144" t="inlineStr">
+      <c r="H144" s="13" t="inlineStr">
         <is>
           <t>29 Ekim Özel — Bilim Tarihi</t>
         </is>
       </c>
-      <c r="I144" t="inlineStr">
+      <c r="I144" s="13" t="inlineStr">
         <is>
           <t>Türk Dil Kurumu (TDK) &amp; Kültür Bakanlığı Geometri Kılavuzu (1937)</t>
         </is>
       </c>
-      <c r="J144" t="inlineStr">
+      <c r="J144" s="13" t="inlineStr">
         <is>
           <t>https://youtu.be/t2lphcITKXs</t>
         </is>
       </c>
-      <c r="K144" t="inlineStr">
+      <c r="K144" s="13" t="inlineStr">
         <is>
           <t>2026-10-29 19:30</t>
         </is>
       </c>
-      <c r="L144" t="n">
-        <v>36</v>
+      <c r="L144" s="13" t="n"/>
+      <c r="M144" s="13" t="n"/>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>BEKLEMEDE</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>video_148.mp4</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Karanlık Odaya Girince Gözün Gece Görüşünü 20 Dakikada Nasıl Açar? 👁️ #bilgidozu #shorts</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>Aydınlıktan karanlık bir odaya girdiğinde ilk saniye hiçbir şey göremezken dakikalar içinde gece görüşün nasıl açılır? Göz arkasında gündüz çalışan koni hücreleri karanlıkta susar; nöbeti yüz yirmi milyon çubuk hücresi devralır.
+📍 BÖLÜMLER
+00:00 Işık kapanınca gözün — Neden önce kör olur?
+00:18 Gizli kimyasal yakıt: — Rodopsin pigmenti!
+00:36 Tek telefon ışığı — Sayacı sıfırlar!
+📊 Kaynaklar:
+• American Academy of Ophthalmology &amp; Harvard Ophthalmology
+• https://www.aao.org/eye-health/anatomy/photoreceptors
+🖼️ Görseller temsilîdir (AI bilimsel canlandırma).
+Daha fazla bilgi dozu için takip etmeyi unutma! 🔔
+#bilgidozu #shorts #göz #insanvücudu #bilim</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>#bilgidozu #shorts #göz #insanvücudu #bilim</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>bilgidozu, shorts, karanlıkta göz nasıl alışır, gece görüşü, rodopsin, göz anatomisi, insan vücudu, bilim, bilgi dozu</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>Bu gece ışığı kapattığında ilk saniye ile üçüncü dakika arasındaki farkı test et, gördüğün değişimi yoruma bırak! 👇</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>İnsan Vücudu ve Beyin</t>
+        </is>
+      </c>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>American Academy of Ophthalmology &amp; Harvard Ophthalmology</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>BEKLEMEDE</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>video_149.mp4</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Nane Şekeri Ağzını Gerçekte Soğutmaz: Beynini Nasıl Kandırır? 🌿 #bilgidozu #shorts</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>Keskin bir nane şekeri attığında ağzının içi buz kesmiş gibi ferahlar; peki nane sıcaklığı gerçekten düşürür mü? Ağzına hassas termometre koysan sıcaklık hiç düşmez; çünkü ortada kusursuz bir kimyasal illüzyon vardır.
+📍 BÖLÜMLER
+00:00 Nane ağzını gerçekten — Soğutuyor mu?
+00:18 Nobel ödüllü keşif: — Sahte soğuk anahtarı!
+00:36 Üstüne su içince — Neden iki kat çarpar?
+📊 Kaynaklar:
+• Nobel Prize in Physiology or Medicine (David Julius, 2021)
+• https://www.nobelprize.org/prizes/medicine/2021/press-release/
+🖼️ Görseller temsilîdir (AI bilimsel canlandırma).
+Daha fazla bilgi dozu için takip etmeyi unutma! 🔔
+#bilgidozu #shorts #bilim #beyin #insanvücudu</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>#bilgidozu #shorts #bilim #beyin #insanvücudu</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>bilgidozu, shorts, nane neden serinletir, mentol soğuk hissi, trpm8 reseptörü, nobel tıp, beyin hilesi, bilgi dozu</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>Naneli sakız üstüne su içip yüzünü buruşturan o arkadaşına bunu gönder, sebebini öğrensin! 👇</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>İnsan Vücudu ve Beyin</t>
+        </is>
+      </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>Nobel Prize in Physiology or Medicine (David Julius, 2021)</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>BEKLEMEDE</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>video_150.mp4</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Sabah Uyandığında Boyun Geceye Göre Neden 2 Santim Daha Uzun Çıkar? 📏 #bilgidozu #shorts</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>Sabah yataktan kalktığın an boyunu ölçsen, geceye göre iki santimetre daha uzun çıktığını biliyor muydun? Sırrı omurga kemiklerinin arasına dizilmiş yirmi üç adet jelatinimsi yastıkçıkta, yani esnek omurga disklerinde gizlidir.
+📍 BÖLÜMLER
+00:00 Sabah uyanınca boyun — Gerçekten uzuyor mu?
+00:17 Gün boyu yerçekimi — Sünger gibi sıkar!
+00:35 Uzaydaki astronotlar — 5 santim bile uzar!
+📊 Kaynaklar:
+• Cleveland Clinic &amp; NASA Spine Decompression Research
+• https://my.clevelandclinic.org/health/body/22460-intervertebral-disc
+🖼️ Görseller temsilîdir (AI bilimsel canlandırma).
+Daha fazla bilgi dozu için takip etmeyi unutma! 🔔
+#bilgidozu #shorts #insanvücudu #omurga #bilim</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>#bilgidozu #shorts #insanvücudu #omurga #bilim</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>bilgidozu, shorts, sabah boy neden uzun çıkar, omurga diskleri, uzayda astronot boyu, insan vücudu, anatomi, bilgi dozu</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>Sabah uyanır uyanmaz ve gece yatmadan duvara işaret koyup ölçmeyi dene, farkı yoruma yaz! 👇</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>İnsan Vücudu ve Beyin</t>
+        </is>
+      </c>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>Cleveland Clinic &amp; NASA Spine Decompression Research</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>BEKLEMEDE</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>uzun_video_17.mp4</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Karanlıkta Gözümüz Gece Görüşünü Nasıl Açar? Korsan Bandı ve Rodopsin Sırrı 👁️ #bilgidozu</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>Aydınlıktan karanlık bir odaya girdiğinde ilk saniye hiçbir şey göremezken dakikalar içinde gece görüşün nasıl açılır? Peki eski denizcilerin ve korsanların taktığı meşhur göz bandının bu yirmi dakikalık kimyayla doğrudan bağlantılı olduğunu biliyor muydun? Güneşli güverteden karanlık gemi altına inen bir denizci yirmi dakika kör kalmayı göze alamazdı. Bir gözünü bantla sürekli karanlıkta hazır tutuyor, alt kata indiği saniye bandı diğer göze kaydırıp anında net görüyordu.
+📍 BÖLÜMLER
+00:00 Işık kapanınca gözün — Neden önce kör olur?
+00:16 Gizli kimyasal yakıt: — Rodopsin pigmenti!
+00:32 Tek telefon ışığı — Sayacı sıfırlar!
+01:06 Denizaltılarda neden — Kırmızı ışık yanar?
+01:27 Soluk yıldızı görmek için — Tam üstüne bakma!
+01:47 Yıldız taktiğini dene! — Yoruma yaz &amp; takip et!
+📊 Kaynaklar:
+• American Academy of Ophthalmology &amp; Naval Aerospace Medical Inst.
+• https://www.aao.org/eye-health/anatomy/photoreceptors
+🖼️ Görseller temsilîdir (AI bilimsel canlandırma).
+Daha fazla bilgi dozu için takip etmeyi unutma! 🔔
+#bilgidozu #göz #beyin #insanvücudu #bilim</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>#bilgidozu #göz #beyin #insanvücudu #bilim</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>bilgidozu, karanlıkta gece görüşü, göz karanlığa nasıl alışır, rodopsin nedir, korsanlar neden göz bandı takar, kırmızı ışık gece görüşü, bilgi dozu</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>Korsanların göz bandı taktiğini daha önce duymuş muydun, yoksa yaralı olduklarını mı sanıyordun? Yoruma yaz! 👇</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>İnsan Vücudu ve Beyin</t>
+        </is>
+      </c>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>American Academy of Ophthalmology &amp; Naval Aerospace Medical Inst.</t>
+        </is>
+      </c>
+      <c r="N148" t="inlineStr">
+        <is>
+          <t>video_148.mp4</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>BEKLEMEDE</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>video_151.mp4</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Odaya Girince Buraya Neden Gelmiştim Diye Unutmanın Bilimsel Sırrı! 🚪 #bilgidozu #shorts</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>İçeriden bir şey almaya mutfağa gidip kapıdan adım attığın saniye ben buraya neden gelmiştim diye kalakalman neden olur? Merak etme, hafızan zayıflamıyor; Notre Dame Üniversitesi bilimcileri bu olaya kapı eşiği etkisi adını verdi.
+📍 BÖLÜMLER
+00:00 Mutfağa girince — Neden bir anda unutursun?
+00:17 Beyin anıları bölüm — Dosyalarına ayırır!
+00:35 Eski odaya dönünce — Neden hemen akla gelir?
+📊 Kaynaklar:
+• Univ. of Notre Dame (Radvansky et al., 2011) Q. J. Exp. Psychol.
+• https://news.nd.edu/news/walking-through-doorways-causes-forgetting-new-research-shows/
+🖼️ Görseller temsilîdir (AI bilimsel canlandırma).
+Daha fazla bilgi dozu için takip etmeyi unutma! 🔔
+#bilgidozu #shorts #beyin #hafıza #psikoloji #bilim</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>#bilgidozu #shorts #beyin #hafıza #psikoloji #bilim</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>bilgidozu, shorts, odaya girince unutmak, kapı eşiği etkisi, doorway effect, unutkanlık neden olur, beyin hafıza, bilgi dozu</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>Mutfağa gidip elinde bambaşka bir şeyle döndüğün en komik anını yoruma yaz! 👇</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>İnsan Vücudu ve Beyin</t>
+        </is>
+      </c>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>Univ. of Notre Dame (Radvansky et al., 2011) Q. J. Exp. Psychol.</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>BEKLEMEDE</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>video_152.mp4</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>İlk Yudum Su Daha Kana Karışmadan Susuzluğunu Nasıl Anında Keser? 💧 #bilgidozu #shorts</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>İçtiğin suyun mideden kana karışması on beş dakikayı bulur; peki nasıl daha ilk yudumda susuzluğun anında kesilir? Kanındaki su azalıp tuz yoğunluğu yükseldiğinde beynindeki özel osmoreseptör nöronları aralıksız susuzluk alarmı çalmaya başlar.
+📍 BÖLÜMLER
+00:00 Suyun kana karışması — 15 dakika sürer ama...
+00:18 15 dakika bekleseydi — Fazla su içerdin!
+00:36 Soğuk su alarmı — Daha hızlı susturur!
+📊 Kaynaklar:
+• UCSF (Zimmerman &amp; Knight, 2016) Nature
+• https://www.ucsf.edu/news/2016/08/403796/thirst-neurons-anticipate-future-hydration-needs
+🖼️ Görseller temsilîdir (AI bilimsel canlandırma).
+Daha fazla bilgi dozu için takip etmeyi unutma! 🔔
+#bilgidozu #shorts #su #beyin #insanvücudu #bilim</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>#bilgidozu #shorts #su #beyin #insanvücudu #bilim</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>bilgidozu, shorts, su içince susuzluk nasıl geçer, beyin susuzluk merkezi, osmoreseptör, insan vücudu, bilim, bilgi dozu</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>Çok susadığında soğuk suyun o ilk yudumdaki ani ferahlığını sen de yaşıyor musun? Yorumlarda buluşalım! 👇</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>İnsan Vücudu ve Beyin</t>
+        </is>
+      </c>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>UCSF (Zimmerman &amp; Knight, 2016) Nature</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>BEKLEMEDE</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>video_153.mp4</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Spordan Ertesi Gün Çıkan Kas Ağrısının Sebebi Laktik Asit Değilmiş! 💪 #bilgidozu #shorts</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>Uzun aradan sonra spor yaptığında ertesi sabah merdiven bile inememene yol açan o hamlama ağrısını hâlâ laktik asit mi sanıyorsun? Spor bilimi bu efsaneyi çürüttü; çünkü oluşan laktik asit, antrenmandan sonraki bir saat içinde tamamen temizlenir.
+📍 BÖLÜMLER
+00:00 Spordan ertesi gün — Kaslar neden sızlar?
+00:18 Gerçek sebep: — Mikroskobik lif çatlakları!
+00:36 Bir sonraki antrenmanda — Kas daha dayanıklı!
+📊 Kaynaklar:
+• American College of Sports Medicine &amp; Sports Medicine Journal
+• https://www.acsm.org/
+🖼️ Görseller temsilîdir (AI bilimsel canlandırma).
+Daha fazla bilgi dozu için takip etmeyi unutma! 🔔
+#bilgidozu #shorts #spor #kas #insanvücudu #bilim</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>#bilgidozu #shorts #spor #kas #insanvücudu #bilim</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>bilgidozu, shorts, kas ağrısı neden olur, hamlama sebebi, laktik asit efsanesi, doms nedir, spor bilimi, bilgi dozu</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>Uzun aradan sonra spora dönüp merdiven inemediğin o gün en çok hangi kasın ağrımıştı? Yoruma yaz! 👇</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>İnsan Vücudu ve Beyin</t>
+        </is>
+      </c>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>American College of Sports Medicine &amp; Sports Medicine Journal</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>BEKLEMEDE</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>uzun_video_18.mp4</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Odaya Girince Ne Alacağını Neden Unutursun? Kapı Eşiği Etkisi ve Beyin 🚪 #bilgidozu</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>İçeriden bir şey almaya mutfağa gidip kapıdan adım attığın saniye ben buraya neden gelmiştim diye kalakalman neden olur? Bilim insanları unutmanın yürüyerek geçen süreden mi yoksa kapıdan mı kaynaklandığını ölçmek için sanal gerçeklik testi kurdu. Aynı mesafeyi düz ve büyük bir salonda yürüyen gönüllüler nesneleri net hatırlarken, aynı mesafede tek bir kapıdan geçenlerin hata oranı iki katına çıktı. Yani hafızayı sıfırlayan şey adımların değil, mekân sınırını geçmekti.
+📍 BÖLÜMLER
+00:00 Mutfağa girince — Neden bir anda unutursun?
+00:16 Beyin anıları bölüm — Dosyalarına ayırır!
+00:32 Eski odaya dönünce — Neden hemen akla gelir?
+01:04 Telefonda sekme açmak: — Dijital kapı eşiği!
+01:20 Unutmamak için 3 saniyelik — Beyin kilitleme tekniği!
+01:40 Telefonda da yaşıyor musun? — Yoruma yaz &amp; takip et!
+📊 Kaynaklar:
+• Univ. of Notre Dame (Radvansky, 2011) &amp; Bond University (2021)
+• https://news.nd.edu/news/walking-through-doorways-causes-forgetting-new-research-shows/
+🖼️ Görseller temsilîdir (AI bilimsel canlandırma).
+Daha fazla bilgi dozu için takip etmeyi unutma! 🔔
+#bilgidozu #beyin #hafıza #psikoloji #bilim</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>#bilgidozu #beyin #hafıza #psikoloji #bilim</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>bilgidozu, kapı eşiği etkisi, odaya girince unutmak, doorway effect, çalışma belleği, dijital unutkanlık, beyin sırları, bilgi dozu</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>Telefon ekranında yeni sekme açınca ne arayacağını unuttuğun da oluyor mu? Yoruma yaz! 👇</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>İnsan Vücudu ve Beyin</t>
+        </is>
+      </c>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>Univ. of Notre Dame (Radvansky, 2011) &amp; Bond University (2021)</t>
+        </is>
+      </c>
+      <c r="N152" t="inlineStr">
+        <is>
+          <t>video_151.mp4</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>BEKLEMEDE</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>video_154.mp4</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Kesilen Elma Dakikalar İçinde Neden Kararır: Gizli Savunma Zırhı! 🍏 #bilgidozu #shorts</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>Bembeyaz kestiğin bir elma dilimi tabakta birkaç dakika beklediğinde neden bozulmuş gibi hızla kahverengiye döner? Gördüğün o renk değişimi çürüme değildir; aslında elmanın yaralanan dokusunu mikroplardan korumak için ördüğü kimyasal bir zırhtır.
+📍 BÖLÜMLER
+00:00 Kesilen elma neden — Dakikalarda kararır?
+00:17 Bıçak hücreyi kesince — Oksijenle birleşir!
+00:35 Bir damla limon — Enzimi nasıl durdurur?
+📊 Kaynaklar:
+• Journal of Agricultural and Food Chemistry &amp; Scientific American
+• https://www.scientificamerican.com/article/why-do-apple-slices-turn-brown-after-being-cut/
+🖼️ Görseller temsilîdir (AI bilimsel canlandırma).
+Daha fazla bilgi dozu için takip etmeyi unutma! 🔔
+#bilgidozu #shorts #kimya #bilim #ilginçbilgiler</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>#bilgidozu #shorts #kimya #bilim #ilginçbilgiler</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>bilgidozu, shorts, kesilen elma neden kararır, elmaya limon sıkmak, polifenol oksidaz, kimya, günlük bilim, bilgi dozu</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>Dilimlenmiş elmayı kararmasın diye limonla mı saklıyorsun, yoksa başka bir yöntemin mi var? Yoruma yaz! 👇</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>Doğa ve Kimya</t>
+        </is>
+      </c>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>Journal of Agricultural and Food Chemistry &amp; Scientific American</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>BEKLEMEDE</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>video_155.mp4</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Buzun Üzeri Neden Kaygandır: Eksi Derecede Bile Akan Gizli Katman! 🧊 #bilgidozu #shorts</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>Düz betonda rahatça yürürken katı buza bastığın saniye ayağının neden sabun gibi kaydığını düşündün mü? Yıllarca ayakkabı basıncının buzu erittiği anlatıldı; oysa insan ağırlığının oluşturduğu basınç buzu eritmeye asla yetmez.
+📍 BÖLÜMLER
+00:00 Taş ve cam kuruyken — Buz neden kaygandır?
+00:17 Amsterdam keşfi: — Gevşek yüzey atomları!
+00:36 -7 derece en kaygan an: — Aşırı soğukta azalır!
+📊 Kaynaklar:
+• Univ. of Amsterdam (Weber &amp; Bonn, 2018) J. Phys. Chem. Lett.
+• https://iop.uva.nl/content/news/2018/05/why-is-ice-slippery.html
+🖼️ Görseller temsilîdir (AI bilimsel canlandırma).
+Daha fazla bilgi dozu için takip etmeyi unutma! 🔔
+#bilgidozu #shorts #fizik #buz #bilim #ilginçbilgiler</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>#bilgidozu #shorts #fizik #buz #bilim #ilginçbilgiler</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>bilgidozu, shorts, buz neden kaygandır, buz üstünde neden kayılır, su molekülleri, fizik sırları, bilim, bilgi dozu</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>Kışın düz yolda yürürken bile kaymayı başaran o arkadaşına bunu gönder! 👇</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>Fizik ve Bilim</t>
+        </is>
+      </c>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>Univ. of Amsterdam (Weber &amp; Bonn, 2018) J. Phys. Chem. Lett.</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>BEKLEMEDE</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>video_156.mp4</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Havuç Gece Görüşünü Güçlendirir Efsanesi Nasıl Gizli Radar Oyunu Çıktı? 🥕 #bilgidozu #shorts</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>Çok havuç yersen karanlıkta kedi gibi görürsün sözünü hep duyarız; peki bu gerçek mi yoksa askeri bir sır mı? Havuçtaki A vitamini göz sağlığını korur; fakat eksiklik yoksa fazlası sağlıklı göze ekstra gece görüşü vermez.
+📍 BÖLÜMLER
+00:00 Bol havuç yemek gece — Görüşünü açar mı?
+00:18 1940 gece gökyüzünde — Gizli radar icadı!
+00:37 80 yıldır süren — En başarılı kampanya!
+📊 Kaynaklar:
+• Smithsonian Magazine &amp; Imperial War Museums Archives
+• https://www.smithsonianmag.com/arts-culture/a-wwii-propaganda-campaign-popularized-the-myth-that-carrots-help-you-see-in-the-dark-28812484/
+🖼️ Görseller temsilîdir (AI bilimsel canlandırma).
+Daha fazla bilgi dozu için takip etmeyi unutma! 🔔
+#bilgidozu #shorts #tarih #bilim #efsaneler #ilginçbilgiler</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>#bilgidozu #shorts #tarih #bilim #efsaneler #ilginçbilgiler</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>bilgidozu, shorts, havuç göze iyi gelir mi, havuç gece görüşü efsanesi, ikinci dünya savaşı radar sırrı, bilim tarihi, bilgi dozu</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>Çocukken doğru sanıp büyüyünce şaşırdığın başka hangi meşhur efsane var? Yoruma bırak! 👇</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>Bilim Tarihi ve Efsaneler</t>
+        </is>
+      </c>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>Smithsonian Magazine &amp; Imperial War Museums Archives</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>BEKLEMEDE</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>uzun_video_19.mp4</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Buz Neden Kaygandır? 150 Yıllık Fizik Tartışmasını Çözen Molekül Sırrı 🧊 #bilgidozu</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>Düz betonda rahatça yürürken katı buza bastığın saniye ayağının neden sabun gibi kaydığını düşündün mü? Buzun yüzeyindeki bu görünmez hareketli katmanı ilk hisseden bilim insanı bin sekiz yüz elli yılında ünlü fizikçi Michael Faraday olmuştu. İki buz küpünü birbirine hafifçe bastırdığında aralarındaki o ince hareketli katman artık dış yüzey olmaktan çıkıp anında donuyor ve iki küp tek parça halinde birbirine kaynıyordu.
+📍 BÖLÜMLER
+00:00 Taş ve cam kuruyken — Buz neden kaygandır?
+00:17 Amsterdam keşfi: — Gevşek yüzey atomları!
+00:36 -7 derece en kaygan an: — Aşırı soğukta azalır!
+01:09 Paten bıçağı buzda — Saniyede nasıl süzülür?
+01:27 Su doğadaki kuralları — Bozan tek sıvıdır!
+01:44 Suyun en ilginç özelliği ne? — Yoruma yaz &amp; takip et!
+📊 Kaynaklar:
+• Univ. of Amsterdam (Bonn, 2018) &amp; Physical Review X
+• https://iop.uva.nl/content/news/2018/05/why-is-ice-slippery.html
+🖼️ Görseller temsilîdir (AI bilimsel canlandırma).
+Daha fazla bilgi dozu için takip etmeyi unutma! 🔔
+#bilgidozu #fizik #buz #bilim #keşif</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>#bilgidozu #fizik #buz #bilim #keşif</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>bilgidozu, buz neden kaygandır, faraday buz deneyi, paten buzda nasıl kayar, suyun ilginç özellikleri, fizik bilimi, bilgi dozu</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>Suyun donunca genleşmesi mi yoksa buzun kayganlığı mı sence daha şaşırtıcı? Yoruma yaz! 👇</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>Fizik ve Bilim</t>
+        </is>
+      </c>
+      <c r="I156" t="inlineStr">
+        <is>
+          <t>Univ. of Amsterdam (Bonn, 2018) &amp; Physical Review X</t>
+        </is>
+      </c>
+      <c r="N156" t="inlineStr">
+        <is>
+          <t>video_155.mp4</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>BEKLEMEDE</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>video_158.mp4</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Ağlamamak İçin Kendini Tuttuğunda Boğazına Neden Yumru Oturur? 😢 #bilgidozu #shorts</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>Ağlamamak için kendini zor tuttuğun an boğazına koca bir yumru oturmuş gibi yutkunmakta neden zorlanırsın? Yoğun üzüntü başladığında beynin tıpkı tehlike anındaki gibi savaş ya da kaç sistemini devreye sokup daha çok oksijen ister.
+📍 BÖLÜMLER
+00:00 Gözyaşını tuttuğun an — Boğazın neden düğümlenir?
+00:16 Ses telleri arasındaki — Nefes kapısı açılır!
+00:35 Ortada hiçbir cisim yok: — Kas çatışması yumru gibi!
+📊 Kaynaklar:
+• Cleveland Clinic &amp; Journal of Voice (Autonomic Laryngeal Physiology)
+• https://my.clevelandclinic.org/health/symptoms/globus-sensation
+🖼️ Görseller temsilîdir (AI bilimsel canlandırma).
+Daha fazla bilgi dozu için takip etmeyi unutma! 🔔
+#bilgidozu #shorts #insanvücudu #beyin #psikoloji #bilim</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>#bilgidozu #shorts #insanvücudu #beyin #psikoloji #bilim</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>bilgidozu, shorts, boğaz düğümlenmesi neden olur, ağlarken boğazda yumru hissi, globus hissi, insan vücudu, beyin, bilim, bilgi dozu</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>Boğazının en son düğümlendiği o an bir film sahnesi miydi yoksa gerçek hayat mı? Yoruma bırak! 👇</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>İnsan Vücudu ve Beyin</t>
+        </is>
+      </c>
+      <c r="I157" t="inlineStr">
+        <is>
+          <t>Cleveland Clinic &amp; Journal of Voice (Autonomic Laryngeal Physiology)</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>BEKLEMEDE</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>video_159.mp4</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Aynı Kelimeyi 20 Kez Söyleyince Neden Anlamı Bir Anda Silinir? 🧠 #bilgidozu #shorts</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>Her gün kullandığın kapı kelimesini yirmi kez üst üste söylediğinde neden bir anda tuhaf bir sese dönüşür? Normalde bir kelimeyi duyduğun salisede beyin kabuğundaki nöron ağı o sesi hafızandaki anlamıyla birleştirir.
+📍 BÖLÜMLER
+00:00 Bildiğin kelime 20 saniyede — Neden yabancı dile döner?
+00:15 Peş peşe ateşlenen hücre — Enerji korumaya geçer!
+00:33 Kulak sesi duyar ama — Anlam köprüsü susar!
+📊 Kaynaklar:
+• McGill University (Jakobovits James, 1962) &amp; Psychological Science
+• https://www.apa.org/pubs/journals/xge
+🖼️ Görseller temsilîdir (AI bilimsel canlandırma).
+Daha fazla bilgi dozu için takip etmeyi unutma! 🔔
+#bilgidozu #shorts #beyin #psikoloji #nörobilim #bilim</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>#bilgidozu #shorts #beyin #psikoloji #nörobilim #bilim</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>bilgidozu, shorts, kelimeyi tekrarlayınca anlamsız gelmesi, anlamsal doygunluk, semantic satiation, beyin sırları, psikoloji, bilim, bilgi dozu</t>
+        </is>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>Şu an 'kaşık' ya da 'kapı' kelimesini 15 kez üst üste fısılda; kaçıncı tekrarda yabancılaştı? Yoruma yaz! 👇</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>Beyin ve Psikoloji</t>
+        </is>
+      </c>
+      <c r="I158" t="inlineStr">
+        <is>
+          <t>McGill University (Jakobovits James, 1962) &amp; Psychological Science</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>BEKLEMEDE</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>video_160.mp4</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Gece Yatakta Tek Ayağını Yorgandan Çıkarınca Neden Hemen Uykun Gelir? 🦶 #bilgidozu #shorts</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>Gece yatakta dönerken tek ayağını yorganın dışına çıkardığın an neden saniyeler içinde ferahlayıp uyursun? Beyninin uyku şalterini açması için iç vücut sıcaklığının bir derece düşmesi şarttır; kalın yorgan ise ısıyı hapseder.
+📍 BÖLÜMLER
+00:00 Tek ayağı yorgandan çıkarmak — Neden anında uyutur?
+00:17 Ayak tabanında gizli — Özel radyatör damarlar!
+00:35 Serinleyen kan beyne — Uyku sinyalini verir!
+📊 Kaynaklar:
+• National Sleep Foundation &amp; Northumbria Univ. Sleep Research
+• https://www.sleepfoundation.org/bedroom-environment/touch/what-temperature-should-your-bedroom-be
+🖼️ Görseller temsilîdir (AI bilimsel canlandırma).
+Daha fazla bilgi dozu için takip etmeyi unutma! 🔔
+#bilgidozu #shorts #uyku #insanvücudu #beyin #bilim</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>#bilgidozu #shorts #uyku #insanvücudu #beyin #bilim</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>bilgidozu, shorts, uyurken ayağı yorgandan çıkarmak, hızlı uyuma tekniği, vücut sıcaklığı uyku, insan vücudu, bilim, bilgi dozu</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>Sen de yaz kış demeden tek ayağını yorganın dışına çıkaranlardan mısın? Yoruma yaz! 👇</t>
+        </is>
+      </c>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>İnsan Vücudu ve Beyin</t>
+        </is>
+      </c>
+      <c r="I159" t="inlineStr">
+        <is>
+          <t>National Sleep Foundation &amp; Northumbria Univ. Sleep Research</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>BEKLEMEDE</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>uzun_video_20.mp4</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>Ağlarken Boğazımız Neden Düğümlenir? Beynin Gizli Glottis Savaşı ve Çözümü 😢 #bilgidozu</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>Ağlamamak için kendini zor tuttuğun an boğazına koca bir yumru oturmuş gibi yutkunmakta neden zorlanırsın? Peki ağlamak yerine kendini sıktığında bu düğüm neden iki kat büyür? Çünkü gözyaşını durdurmak için yüz, çene ve boyun çevresindeki yirmiden fazla yardımcı kası aynı anda kasarsın. Gırtlağı askıda tutan bu dış kaslar gerildikçe içerideki nefes kapısının hareket alanı iyice daralır ve basınç hissi zirveye çıkar.
+📍 BÖLÜMLER
+00:00 Gözyaşını tuttuğun an — Boğazın neden düğümlenir?
+00:16 Ses telleri arasındaki — Nefes kapısı açılır!
+00:34 Ortada hiçbir cisim yok: — Kas çatışması yumru gibi!
+01:05 Tek yudum ılık su — Sinir kilidini nasıl açar?
+01:27 Ağlamak zayıflık değil: — Kimyasal boşaltım sistemi!
+01:47 Seni en çok ne duygulandırır? — Yoruma yaz &amp; abone ol!
+📊 Kaynaklar:
+• Cleveland Clinic &amp; Journal of Voice (Autonomic Laryngeal Physiology)
+• https://my.clevelandclinic.org/health/symptoms/globus-sensation
+🖼️ Görseller temsilîdir (AI bilimsel canlandırma).
+Daha fazla bilgi dozu için takip etmeyi unutma! 🔔
+#bilgidozu #insanvücudu #beyin #psikoloji #bilim</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>#bilgidozu #insanvücudu #beyin #psikoloji #bilim</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>bilgidozu, boğaz düğümlenmesi neden olur, ağlarken boğazda yumru, globus pharyngeus, glottis nedir, vagus siniri, insan vücudu, bilgi dozu</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>Boğazın düğümlendiğinde bir yudum ılık su taktiğini biliyor muydun, yoksa yutkunmaya mı çalışıyordun? Yoruma yaz! 👇</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>İnsan Vücudu ve Beyin</t>
+        </is>
+      </c>
+      <c r="I160" t="inlineStr">
+        <is>
+          <t>Cleveland Clinic &amp; Journal of Voice (Autonomic Laryngeal Physiology)</t>
+        </is>
+      </c>
+      <c r="N160" t="inlineStr">
+        <is>
+          <t>video_158.mp4</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>BEKLEMEDE</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>video_161.mp4</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Saate İlk Baktığın Saniye Neden Donmuş Gibi Daha Uzun Sürer? ⏱️ #bilgidozu #shorts</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>Gözünü aniden duvar saatine çevirdiğin ilk an saniye ibresinin bozulmuş gibi daha uzun beklediğini fark ettin mi? Gözün saate hızla sıçrarken görüntü bulanıklaşmasın diye beynin yaklaşık elli milisaniye boyunca kaydı kapatır.
+📍 BÖLÜMLER
+00:00 Saate ilk baktığın an — Saniye neden donakalır?
+00:16 Karanlık boşluğu örtmek için — Geriye dönük montaj!
+00:35 Aynada kendi gözünün — Hareketini göremezsin!
+📊 Kaynaklar:
+• University College London (Yarrow et al., Nature 2001)
+• https://www.nature.com/articles/35104551
+🖼️ Görseller temsilîdir (AI bilimsel canlandırma).
+Daha fazla bilgi dozu için takip etmeyi unutma! 🔔
+#bilgidozu #shorts #beyin #zaman #psikoloji #bilim</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>#bilgidozu #shorts #beyin #zaman #psikoloji #bilim</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>bilgidozu, shorts, durmuş saat yanılsaması, kronostaz nedir, saate bakınca saniyenin durması, beyin zaman algısı, nörobilim, bilgi dozu</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>Bu videodan hemen sonra bir saate ya da telefon sayacına hızla gözünü çevirip ilk saniyeyi dene; fark ettin mi? 👇</t>
+        </is>
+      </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>Beyin ve Psikoloji</t>
+        </is>
+      </c>
+      <c r="I161" t="inlineStr">
+        <is>
+          <t>University College London (Yarrow et al., Nature 2001)</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>BEKLEMEDE</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>video_162.mp4</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>Çok Tuzlu Çekirdek Yediğinde Dudakların Neden Kuruyup Büzüşür? 🧂 #bilgidozu #shorts</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>Bir avuç tuzlu çekirdek yediğinde dudaklarının kuruyup beyazladığını ve büzüştüğünü hiç fark ettin mi? Ağız içini kaplayan yumuşak hücrelerin üzerine yoğun tuz yapıştığında fiziğin ozmoz yasası saniyede devreye girer.
+📍 BÖLÜMLER
+00:00 Tuzlu çekirdek yiyince — Dudaklar neden büzüşür?
+00:16 Hücre içindeki saf su — Dışarı doğru emilir!
+00:35 Bir bardak saf suyla — Denge geri kurulur!
+📊 Kaynaklar:
+• Nature Neuroscience (Oka et al., High-Salt Taste Receptors) &amp; NIH
+• https://www.nih.gov/news-events/nih-research-matters/how-tongue-detects-high-salt-levels
+🖼️ Görseller temsilîdir (AI bilimsel canlandırma).
+Daha fazla bilgi dozu için takip etmeyi unutma! 🔔
+#bilgidozu #shorts #biyoloji #insanvücudu #kimya #bilim</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>#bilgidozu #shorts #biyoloji #insanvücudu #kimya #bilim</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>bilgidozu, shorts, tuzlu çekirdek dudak büzüşmesi, tuz neden susatır, ozmoz nedir, insan vücudu, biyoloji, bilim, bilgi dozu</t>
+        </is>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>Çekirdek çitlemeye başlayınca dudakların beyazlayana kadar duramayan arkadaşını etiketle veya ona gönder! 👇</t>
+        </is>
+      </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>Biyoloji ve Vücut</t>
+        </is>
+      </c>
+      <c r="I162" t="inlineStr">
+        <is>
+          <t>Nature Neuroscience (Oka et al., High-Salt Taste Receptors) &amp; NIH</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>BEKLEMEDE</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>video_163.mp4</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Üzgün Olmasan Bile Her 5 Dakikada Bir Neden Fark Etmeden İç Çekersin? 🫁 #bilgidozu #shorts</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>Hiçbir derdin yokken otururken göğsünün neden her beş dakikada bir kendiliğinden derin iç çektiğini biliyor musun? Akciğerlerindeki beş yüz milyon minik hava keseciği normal sığ nefeslerde ıslak balon gibi yavaşça söner.
+📍 BÖLÜMLER
+00:00 Üzgün olmadığın halde — Neden derin iç çekersin?
+00:17 Beyin sapındaki saat: — Saatte 12 kez ateşlenir!
+00:36 Stresi 10 saniyede kesen — Çift nefes tekniği!
+📊 Kaynaklar:
+• Nature (Li, Feldman &amp; Krasnow, UCLA &amp; Stanford Medicine)
+• https://med.stanford.edu/news/all-news/2016/02/study-pinpoints-brain-circuitry-that-causes-sighing.html
+🖼️ Görseller temsilîdir (AI bilimsel canlandırma).
+Daha fazla bilgi dozu için takip etmeyi unutma! 🔔
+#bilgidozu #shorts #akciğer #nefes #insanvücudu #bilim</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>#bilgidozu #shorts #akciğer #nefes #insanvücudu #bilim</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>bilgidozu, shorts, neden iç çekeriz, fizyolojik iç çekiş, akciğer alveol, stanford nefes tekniği, insan vücudu, bilim, bilgi dozu</t>
+        </is>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>Şimdi burnundan üst üste iki kısa nefes çekip ağzından yavaşça ver; o anlık rahatlamayı hissettin mi? 👇</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>İnsan Vücudu ve Beyin</t>
+        </is>
+      </c>
+      <c r="I163" t="inlineStr">
+        <is>
+          <t>Nature (Li, Feldman &amp; Krasnow, UCLA &amp; Stanford Medicine)</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>BEKLEMEDE</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>uzun_video_21.mp4</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>Saate İlk Baktığında Saniye Neden Donar? Beynin Zamanı Geriye Saran Hilesi ⏱️ #bilgidozu</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>Gözünü aniden duvar saatine çevirdiğin ilk an saniye ibresinin bozulmuş gibi daha uzun beklediğini fark ettin mi? İnsan gözü çevreyi tararken saniyede üç kez hızlı sıçrama yapar; yani uyanık olduğun tek bir günde yaklaşık yüz elli bin kez görüntün kesilir. Toplamda günde kırk dakikadan fazla görsel karanlıkta kalırsın ama beynin kurgu masası gibi boşlukları geriye dönük doldurduğu için dünyayı kesintisiz bir film sanırsın.
+📍 BÖLÜMLER
+00:00 Saate ilk baktığın an — Saniye neden donakalır?
+00:15 Karanlık boşluğu örtmek için — Geriye dönük montaj!
+00:32 Aynada kendi gözünün — Hareketini göremezsin!
+01:02 Sadece gözde değil: — Ses ve dokunmada da olur!
+01:19 80 milisaniye geriden: — Geçmişi şimdi sanıyorsun!
+01:41 Ayna testini denedin mi? — Yoruma yaz &amp; abone ol!
+📊 Kaynaklar:
+• University College London (Yarrow et al., Nature 2001) &amp; Salk Institute
+• https://www.nature.com/articles/35104551
+🖼️ Görseller temsilîdir (AI bilimsel canlandırma).
+Daha fazla bilgi dozu için takip etmeyi unutma! 🔔
+#bilgidozu #beyin #zaman #nörobilim #bilim</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>#bilgidozu #beyin #zaman #nörobilim #bilim</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>bilgidozu, durmuş saat yanılsaması, kronostaz, beynin zaman algısı, aynada göz hareketini görememek, nörobilim, psikoloji, bilgi dozu</t>
+        </is>
+      </c>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>Aynada sağ gözünden sol gözüne bakarken hareketi yakalamayı denedin mi? Sonucu yoruma yaz! 👇</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>Beyin ve Psikoloji</t>
+        </is>
+      </c>
+      <c r="I164" t="inlineStr">
+        <is>
+          <t>University College London (Yarrow et al., Nature 2001) &amp; Salk Institute</t>
+        </is>
+      </c>
+      <c r="N164" t="inlineStr">
+        <is>
+          <t>video_161.mp4</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>BEKLEMEDE</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>video_164.mp4</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>Tıka Basa Doysan Bile Tatlıya Neden Her Zaman Yer Açılır? 🍰 #bilgidozu #shorts</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>Akşam yemeğinde tek lokma bile yiyemeyecek kadar doyduğun halde masaya tatlı geldiği an midende nasıl mucizevi yer açılır? Şaka sandığımız tatlı için ayrı mide sözü gerçek çıktı; Max Planck Enstitüsü bu gizli şalterin tam beyinde olduğunu kanıtladı.
+📍 BÖLÜMLER
+00:00 Tek lokma yiyemeyecekken — Tatlıya nasıl yer açılır?
+00:19 Tokluk nöronları yemekte — Artık doydun diyor!
+00:38 Atalarımızdan kalan — Hızlı enerji kodu!
+📊 Kaynaklar:
+• Max Planck Institute for Metabolism Research (Science, 2025)
+• https://www.mpg.de/24159607/0211-neur-dessert-stomach-emerges-in-the-brain-153735-x
+🖼️ Görseller temsilîdir (AI bilimsel canlandırma).
+Daha fazla bilgi dozu için takip etmeyi unutma! 🔔
+#bilgidozu #shorts #beyin #tatlı #insanvücudu #bilim</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>#bilgidozu #shorts #beyin #tatlı #insanvücudu #bilim</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>bilgidozu, shorts, tokken neden tatlı isteriz, tatlı midesi gerçek mi, yemekten sonra tatlı krizi, beyin ve iştah, bilim, bilgi dozu</t>
+        </is>
+      </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>Yemekten sonra ne kadar tok olursan ol asla hayır diyemediğin o tatlı hangisi? Yoruma yaz! 👇</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>İnsan Vücudu ve Beyin</t>
+        </is>
+      </c>
+      <c r="I165" t="inlineStr">
+        <is>
+          <t>Max Planck Institute for Metabolism Research (Science, 2025)</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>BEKLEMEDE</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>video_165.mp4</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>Kuru Kum Dağılırken Yüzde 1 Su Kumdan Kaleyi Nasıl Taş Gibi Tutar? 🏰 #bilgidozu #shorts</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>Sahilde kuru kum parmaklarının arasından su gibi akarken, biraz ıslattığında nasıl metrelerce yüksek kale gibi dimdik durur? Kuma az miktarda su eklediğinde su damlacıkları kum tanelerinin arasına yerleşip görünmez kapiler sıvı köprüleri kurar.
+📍 BÖLÜMLER
+00:00 Kuru kum akıp giderken — Islak kum nasıl taşlaşır?
+00:19 Yüzey gerilimi taneleri — Vantuz gibi çeker!
+00:38 Fazla su köprüyü yıkar: — Kale çamur olup çöker!
+📊 Kaynaklar:
+• Univ. of Amsterdam (Fall &amp; Bonn, Nature Scientific Reports)
+• https://www.nature.com/articles/srep00549
+🖼️ Görseller temsilîdir (AI bilimsel canlandırma).
+Daha fazla bilgi dozu için takip etmeyi unutma! 🔔
+#bilgidozu #shorts #fizik #doğa #keşif #bilim</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>#bilgidozu #shorts #fizik #doğa #keşif #bilim</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>bilgidozu, shorts, ıslak kum neden yapışır, kumdan kale fiziği, kapiler sıvı köprüsü, yüzey gerilimi, fizik bilimi, bilgi dozu</t>
+        </is>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>Sahilde kumdan kale yaparken senin de kulelerin fazla sudan çökmüş müydü? Yoruma yaz! 👇</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>Fizik ve Bilim</t>
+        </is>
+      </c>
+      <c r="I166" t="inlineStr">
+        <is>
+          <t>Univ. of Amsterdam (Fall &amp; Bonn, Nature Scientific Reports)</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>BEKLEMEDE</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>video_166.mp4</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>Okulda Öğretilen Dil Tat Haritası Nasıl 100 Yıllık Çeviri Hatası Çıktı? 👅 #bilgidozu #shorts</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>Okulda yıllarca ezberletilen dilin ucu tatlıyı, arkası acıyı alır haritasının koca bir hata olduğunu biliyor muydun? Bin dokuz yüz birde Alman bilimci David Hänig dilin her yerinin tat aldığını, sadece ufak farklar olduğunu yazdı.
+📍 BÖLÜMLER
+00:00 Okulda öğretilen dil haritası — Tamamen yanlış çıktı!
+00:17 1942 grafik çevirisinde — Efsane nasıl doğdu?
+00:36 Tek saniyelik kanıt: — Dilinin ucuna kahve değdir!
+📊 Kaynaklar:
+• Nature (Chandrashekar et al., 2006) &amp; Smithsonian Science
+• https://www.smithsonianmag.com/science-nature/neat-and-tidy-map-tastes-tongue-you-learned-school-all-wrong-180963407/
+🖼️ Görseller temsilîdir (AI bilimsel canlandırma).
+Daha fazla bilgi dozu için takip etmeyi unutma! 🔔
+#bilgidozu #shorts #efsaneler #insanvücudu #bilim #tarih</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>#bilgidozu #shorts #efsaneler #insanvücudu #bilim #tarih</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>bilgidozu, shorts, dil tat haritası yanlış mı, dilin ucu tatlı alır efsanesi, umami nedir, bilim efsaneleri, insan vücudu, bilgi dozu</t>
+        </is>
+      </c>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>Okulda sana da 'dilin ucu tatlı, yanları ekşi alır' şeması çizdirilmiş miydi? Yoruma yaz! 👇</t>
+        </is>
+      </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>Bilim Tarihi ve Efsaneler</t>
+        </is>
+      </c>
+      <c r="I167" t="inlineStr">
+        <is>
+          <t>Nature (Chandrashekar et al., 2006) &amp; Smithsonian Science</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>BEKLEMEDE</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>uzun_video_22.mp4</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>Tokken Neden Tatlı İsteriz? Beyindeki 'Tatlı Midesi' Şalterinin 2025 Bilimsel Kanıtı 🍰 #bilgidozu</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>Akşam yemeğinde tek lokma bile yiyemeyecek kadar doyduğun halde masaya tatlı geldiği an midende nasıl mucizevi yer açılır? Tatlı krizinin arkasındaki ikinci büyük güç Oxford Üniversitesi'nden Edmund Rolls'un tanımladığı duyusal özgül tokluktur. Beynin tek tip tuzlu yemekten sıkıldığında miden tam dolmasa bile o tada karşı fren yapar; fakat önüne bambaşka koku ve dokuda tatlı bir tabak geldiğinde iştah sayacı sıfırlanır.
+📍 BÖLÜMLER
+00:00 Tek lokma yiyemeyecekken — Tatlıya nasıl yer açılır?
+00:18 Tokluk nöronları yemekte — Artık doydun diyor!
+00:36 Atalarımızdan kalan — Hızlı enerji kodu!
+01:06 Daha ilk lokmadan önce — Görmek bile şalteri açar!
+01:28 Tatlı krizini kandıran — 15 dakika kuralı!
+01:51 15 dakika kuralını dene! — Yoruma yaz &amp; abone ol!
+📊 Kaynaklar:
+• Max Planck Institute (Minère et al., Science 2025) &amp; Oxford University
+• https://www.mpg.de/24159607/0211-neur-dessert-stomach-emerges-in-the-brain-153735-x
+🖼️ Görseller temsilîdir (AI bilimsel canlandırma).
+Daha fazla bilgi dozu için takip etmeyi unutma! 🔔
+#bilgidozu #beyin #beslenme #insanvücudu #bilim</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>#bilgidozu #beyin #beslenme #insanvücudu #bilim</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>bilgidozu, yemekten sonra tatlı isteği neden olur, tatlı midesi gerçek mi, max planck tatlı araştırması, duyusal özgül tokluk, beyin, bilgi dozu</t>
+        </is>
+      </c>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>Yemekten hemen sonra tatlı arayanlardan mısın yoksa çayla geçiştirebilenlerden mi? Yoruma yaz! 👇</t>
+        </is>
+      </c>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>İnsan Vücudu ve Beyin</t>
+        </is>
+      </c>
+      <c r="I168" t="inlineStr">
+        <is>
+          <t>Max Planck Institute (Minère et al., Science 2025) &amp; Oxford University</t>
+        </is>
+      </c>
+      <c r="N168" t="inlineStr">
+        <is>
+          <t>video_164.mp4</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>